<commit_message>
Perbarui struktur organisasi (2026-09-14T07:03:00.809Z)
</commit_message>
<xml_diff>
--- a/data/struktur-organisasi.xlsx
+++ b/data/struktur-organisasi.xlsx
@@ -78173,7 +78173,7 @@
     </row>
     <row r="2043">
       <c r="A2043" t="str">
-        <v>Kmu0warcw58qw</v>
+        <v>Kmu0wbkuka9up</v>
       </c>
       <c r="B2043" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78211,7 +78211,7 @@
     </row>
     <row r="2044">
       <c r="A2044" t="str">
-        <v>Kmu0warcwuc1z</v>
+        <v>Kmu0wbkulxw6k</v>
       </c>
       <c r="B2044" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78249,7 +78249,7 @@
     </row>
     <row r="2045">
       <c r="A2045" t="str">
-        <v>Kmu0warcw8v9p</v>
+        <v>Kmu0wbkulf29d</v>
       </c>
       <c r="B2045" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78325,7 +78325,7 @@
     </row>
     <row r="2047">
       <c r="A2047" t="str">
-        <v>Kmu0warcwq8eq</v>
+        <v>Kmu0wbkulazt2</v>
       </c>
       <c r="B2047" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78363,7 +78363,7 @@
     </row>
     <row r="2048">
       <c r="A2048" t="str">
-        <v>Kmu0warcwyb8l</v>
+        <v>Kmu0wbkulfx0l</v>
       </c>
       <c r="B2048" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78401,7 +78401,7 @@
     </row>
     <row r="2049">
       <c r="A2049" t="str">
-        <v>Kmu0warcwdbzz</v>
+        <v>Kmu0wbkulek5h</v>
       </c>
       <c r="B2049" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78477,7 +78477,7 @@
     </row>
     <row r="2051">
       <c r="A2051" t="str">
-        <v>Kmu0warcwke7e</v>
+        <v>Kmu0wbkulkgj8</v>
       </c>
       <c r="B2051" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78515,7 +78515,7 @@
     </row>
     <row r="2052">
       <c r="A2052" t="str">
-        <v>Kmu0warcwjfoc</v>
+        <v>Kmu0wbkulclyg</v>
       </c>
       <c r="B2052" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78553,7 +78553,7 @@
     </row>
     <row r="2053">
       <c r="A2053" t="str">
-        <v>Kmu0warcw9kqx</v>
+        <v>Kmu0wbkultmsq</v>
       </c>
       <c r="B2053" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78591,7 +78591,7 @@
     </row>
     <row r="2054">
       <c r="A2054" t="str">
-        <v>Kmu0warcwaxdo</v>
+        <v>Kmu0wbkulo9si</v>
       </c>
       <c r="B2054" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -78629,7 +78629,7 @@
     </row>
     <row r="2055">
       <c r="A2055" t="str">
-        <v>Kmu0warcwf92d</v>
+        <v>Kmu0wbkul1vjd</v>
       </c>
       <c r="B2055" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -78667,7 +78667,7 @@
     </row>
     <row r="2056">
       <c r="A2056" t="str">
-        <v>Kmu0warcw09qr</v>
+        <v>Kmu0wbkul52ok</v>
       </c>
       <c r="B2056" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -78705,7 +78705,7 @@
     </row>
     <row r="2057">
       <c r="A2057" t="str">
-        <v>Kmu0warcw2y4z</v>
+        <v>Kmu0wbkul5o65</v>
       </c>
       <c r="B2057" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -78743,7 +78743,7 @@
     </row>
     <row r="2058">
       <c r="A2058" t="str">
-        <v>Kmu0warcwjyhn</v>
+        <v>Kmu0wbkul506o</v>
       </c>
       <c r="B2058" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -78857,7 +78857,7 @@
     </row>
     <row r="2061">
       <c r="A2061" t="str">
-        <v>Kmu0warcww3tm</v>
+        <v>Kmu0wbkulporm</v>
       </c>
       <c r="B2061" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78895,7 +78895,7 @@
     </row>
     <row r="2062">
       <c r="A2062" t="str">
-        <v>Kmu0warcwgrsv</v>
+        <v>Kmu0wbkulbe2e</v>
       </c>
       <c r="B2062" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78933,7 +78933,7 @@
     </row>
     <row r="2063">
       <c r="A2063" t="str">
-        <v>Kmu0warcwes13</v>
+        <v>Kmu0wbkulkgng</v>
       </c>
       <c r="B2063" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79009,7 +79009,7 @@
     </row>
     <row r="2065">
       <c r="A2065" t="str">
-        <v>Kmu0warcwcfjj</v>
+        <v>Kmu0wbkulg7wh</v>
       </c>
       <c r="B2065" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79047,7 +79047,7 @@
     </row>
     <row r="2066">
       <c r="A2066" t="str">
-        <v>Kmu0warcwttzg</v>
+        <v>Kmu0wbkulw7zw</v>
       </c>
       <c r="B2066" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79085,7 +79085,7 @@
     </row>
     <row r="2067">
       <c r="A2067" t="str">
-        <v>Kmu0warcwmvog</v>
+        <v>Kmu0wbkulkzj7</v>
       </c>
       <c r="B2067" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79161,7 +79161,7 @@
     </row>
     <row r="2069">
       <c r="A2069" t="str">
-        <v>Kmu0warcwcokw</v>
+        <v>Kmu0wbkulthdv</v>
       </c>
       <c r="B2069" t="str">
         <v>Penata Layanan Operasional</v>
@@ -79199,7 +79199,7 @@
     </row>
     <row r="2070">
       <c r="A2070" t="str">
-        <v>Kmu0warcwb5j8</v>
+        <v>Kmu0wbkulcev5</v>
       </c>
       <c r="B2070" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79237,7 +79237,7 @@
     </row>
     <row r="2071">
       <c r="A2071" t="str">
-        <v>Kmu0warcwrwhj</v>
+        <v>Kmu0wbkuletk8</v>
       </c>
       <c r="B2071" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79313,7 +79313,7 @@
     </row>
     <row r="2073">
       <c r="A2073" t="str">
-        <v>Kmu0warcwvhus</v>
+        <v>Kmu0wbkulg1np</v>
       </c>
       <c r="B2073" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79351,7 +79351,7 @@
     </row>
     <row r="2074">
       <c r="A2074" t="str">
-        <v>Kmu0warcwhwii</v>
+        <v>Kmu0wbkul85r7</v>
       </c>
       <c r="B2074" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79389,7 +79389,7 @@
     </row>
     <row r="2075">
       <c r="A2075" t="str">
-        <v>Kmu0warcwghf5</v>
+        <v>Kmu0wbkul8pb6</v>
       </c>
       <c r="B2075" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79427,7 +79427,7 @@
     </row>
     <row r="2076">
       <c r="A2076" t="str">
-        <v>Kmu0warcw9s7k</v>
+        <v>Kmu0wbkulr1yq</v>
       </c>
       <c r="B2076" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -79465,7 +79465,7 @@
     </row>
     <row r="2077">
       <c r="A2077" t="str">
-        <v>Kmu0warcw5fgx</v>
+        <v>Kmu0wbkuld0ez</v>
       </c>
       <c r="B2077" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -79503,7 +79503,7 @@
     </row>
     <row r="2078">
       <c r="A2078" t="str">
-        <v>Kmu0warcwer8a</v>
+        <v>Kmu0wbkul9unk</v>
       </c>
       <c r="B2078" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -79541,7 +79541,7 @@
     </row>
     <row r="2079">
       <c r="A2079" t="str">
-        <v>Kmu0warcwhqnt</v>
+        <v>Kmu0wbkulxqee</v>
       </c>
       <c r="B2079" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -79579,7 +79579,7 @@
     </row>
     <row r="2080">
       <c r="A2080" t="str">
-        <v>Kmu0warcwdo7b</v>
+        <v>Kmu0wbkul0teb</v>
       </c>
       <c r="B2080" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -79617,7 +79617,7 @@
     </row>
     <row r="2081">
       <c r="A2081" t="str">
-        <v>Kmu0warcwwn9m</v>
+        <v>Kmu0wbkulm3wu</v>
       </c>
       <c r="B2081" t="str">
         <v>Asesor SDM Aparatur Ahli Muda</v>
@@ -79655,7 +79655,7 @@
     </row>
     <row r="2082">
       <c r="A2082" t="str">
-        <v>Kmu0warcwn6q0</v>
+        <v>Kmu0wbkuljpzu</v>
       </c>
       <c r="B2082" t="str">
         <v>Asesor SDM Aparatur Ahli Pertama</v>
@@ -79769,7 +79769,7 @@
     </row>
     <row r="2085">
       <c r="A2085" t="str">
-        <v>Kmu0warcw7exz</v>
+        <v>Kmu0wbkul1d4m</v>
       </c>
       <c r="B2085" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79807,7 +79807,7 @@
     </row>
     <row r="2086">
       <c r="A2086" t="str">
-        <v>Kmu0warcwe6cv</v>
+        <v>Kmu0wbkulo12a</v>
       </c>
       <c r="B2086" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79845,7 +79845,7 @@
     </row>
     <row r="2087">
       <c r="A2087" t="str">
-        <v>Kmu0warcwn54q</v>
+        <v>Kmu0wbkul99q9</v>
       </c>
       <c r="B2087" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79921,7 +79921,7 @@
     </row>
     <row r="2089">
       <c r="A2089" t="str">
-        <v>Kmu0warcw8i92</v>
+        <v>Kmu0wbkulsroy</v>
       </c>
       <c r="B2089" t="str">
         <v>Penata Layanan Operasional</v>
@@ -79959,7 +79959,7 @@
     </row>
     <row r="2090">
       <c r="A2090" t="str">
-        <v>Kmu0warcwotil</v>
+        <v>Kmu0wbkulrjkf</v>
       </c>
       <c r="B2090" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79997,7 +79997,7 @@
     </row>
     <row r="2091">
       <c r="A2091" t="str">
-        <v>Kmu0warcw1q2w</v>
+        <v>Kmu0wbkulwa61</v>
       </c>
       <c r="B2091" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80073,7 +80073,7 @@
     </row>
     <row r="2093">
       <c r="A2093" t="str">
-        <v>Kmu0warcw6vda</v>
+        <v>Kmu0wbkullx29</v>
       </c>
       <c r="B2093" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80111,7 +80111,7 @@
     </row>
     <row r="2094">
       <c r="A2094" t="str">
-        <v>Kmu0warcw6xyk</v>
+        <v>Kmu0wbkul7oan</v>
       </c>
       <c r="B2094" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80149,7 +80149,7 @@
     </row>
     <row r="2095">
       <c r="A2095" t="str">
-        <v>Kmu0warcwk95g</v>
+        <v>Kmu0wbkuldg3g</v>
       </c>
       <c r="B2095" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80187,7 +80187,7 @@
     </row>
     <row r="2096">
       <c r="A2096" t="str">
-        <v>Kmu0warcwvt28</v>
+        <v>Kmu0wbkulpsm2</v>
       </c>
       <c r="B2096" t="str">
         <v>Analis Anggaran Ahli Pertama/ Analis Keuangan Negara Ahli Pertama</v>
@@ -80225,7 +80225,7 @@
     </row>
     <row r="2097">
       <c r="A2097" t="str">
-        <v>Kmu0warcwqx42</v>
+        <v>Kmu0wbkulfvri</v>
       </c>
       <c r="B2097" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Muda/Pengawas Keuangan Negara Ahli Muda</v>
@@ -80263,7 +80263,7 @@
     </row>
     <row r="2098">
       <c r="A2098" t="str">
-        <v>Kmu0warcwtsp9</v>
+        <v>Kmu0wbkulv271</v>
       </c>
       <c r="B2098" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Pertama/Pengawas Keuangan Negara Ahli Pertama</v>
@@ -80301,7 +80301,7 @@
     </row>
     <row r="2099">
       <c r="A2099" t="str">
-        <v>Kmu0warcw34vi</v>
+        <v>Kmu0wbkulrtdh</v>
       </c>
       <c r="B2099" t="str">
         <v>Pranata Keuangan APBN Penyelia/Pengawas Keuangan Negara Penyelia</v>
@@ -80339,7 +80339,7 @@
     </row>
     <row r="2100">
       <c r="A2100" t="str">
-        <v>Kmu0warcwjdc9</v>
+        <v>Kmu0wbkulppma</v>
       </c>
       <c r="B2100" t="str">
         <v>Pranata Keuangan APBN Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -80377,7 +80377,7 @@
     </row>
     <row r="2101">
       <c r="A2101" t="str">
-        <v>Kmu0warcwg2xo</v>
+        <v>Kmu0wbkulomj3</v>
       </c>
       <c r="B2101" t="str">
         <v>Pranata Keuangan APBN Terampil/Pengawas Keuangan Negara Terampil</v>
@@ -80415,7 +80415,7 @@
     </row>
     <row r="2102">
       <c r="A2102" t="str">
-        <v>Kmu0warcwoapq</v>
+        <v>Kmu0wbkul5quz</v>
       </c>
       <c r="B2102" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -80453,7 +80453,7 @@
     </row>
     <row r="2103">
       <c r="A2103" t="str">
-        <v>Kmu0warcwcf1v</v>
+        <v>Kmu0wbkulfzy6</v>
       </c>
       <c r="B2103" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -80491,7 +80491,7 @@
     </row>
     <row r="2104">
       <c r="A2104" t="str">
-        <v>Kmu0warcwtymx</v>
+        <v>Kmu0wbkuloh5a</v>
       </c>
       <c r="B2104" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -80529,7 +80529,7 @@
     </row>
     <row r="2105">
       <c r="A2105" t="str">
-        <v>Kmu0warcw69a8</v>
+        <v>Kmu0wbkulmsv9</v>
       </c>
       <c r="B2105" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -80567,7 +80567,7 @@
     </row>
     <row r="2106">
       <c r="A2106" t="str">
-        <v>Kmu0warcw025g</v>
+        <v>Kmu0wbkul2te4</v>
       </c>
       <c r="B2106" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -80681,7 +80681,7 @@
     </row>
     <row r="2109">
       <c r="A2109" t="str">
-        <v>Kmu0warcwx4al</v>
+        <v>Kmu0wbkulpbkc</v>
       </c>
       <c r="B2109" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80719,7 +80719,7 @@
     </row>
     <row r="2110">
       <c r="A2110" t="str">
-        <v>Kmu0warcwla58</v>
+        <v>Kmu0wbkul685h</v>
       </c>
       <c r="B2110" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80757,7 +80757,7 @@
     </row>
     <row r="2111">
       <c r="A2111" t="str">
-        <v>Kmu0warcwskq6</v>
+        <v>Kmu0wbkulo201</v>
       </c>
       <c r="B2111" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80833,7 +80833,7 @@
     </row>
     <row r="2113">
       <c r="A2113" t="str">
-        <v>Kmu0warcwvmtl</v>
+        <v>Kmu0wbkul38f7</v>
       </c>
       <c r="B2113" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80871,7 +80871,7 @@
     </row>
     <row r="2114">
       <c r="A2114" t="str">
-        <v>Kmu0warcwcsjq</v>
+        <v>Kmu0wbkulwmf1</v>
       </c>
       <c r="B2114" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80909,7 +80909,7 @@
     </row>
     <row r="2115">
       <c r="A2115" t="str">
-        <v>Kmu0warcw4suv</v>
+        <v>Kmu0wbkuljan6</v>
       </c>
       <c r="B2115" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80985,7 +80985,7 @@
     </row>
     <row r="2117">
       <c r="A2117" t="str">
-        <v>Kmu0warcwlxo9</v>
+        <v>Kmu0wbkul6ao3</v>
       </c>
       <c r="B2117" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -81023,7 +81023,7 @@
     </row>
     <row r="2118">
       <c r="A2118" t="str">
-        <v>Kmu0warcwfqit</v>
+        <v>Kmu0wbkulezy7</v>
       </c>
       <c r="B2118" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81061,7 +81061,7 @@
     </row>
     <row r="2119">
       <c r="A2119" t="str">
-        <v>Kmu0warcw69c9</v>
+        <v>Kmu0wbkul7mhg</v>
       </c>
       <c r="B2119" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81099,7 +81099,7 @@
     </row>
     <row r="2120">
       <c r="A2120" t="str">
-        <v>Kmu0warcw6832</v>
+        <v>Kmu0wbkul6uh6</v>
       </c>
       <c r="B2120" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -81137,7 +81137,7 @@
     </row>
     <row r="2121">
       <c r="A2121" t="str">
-        <v>Kmu0warcwlkra</v>
+        <v>Kmu0wbkullhev</v>
       </c>
       <c r="B2121" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -81175,7 +81175,7 @@
     </row>
     <row r="2122">
       <c r="A2122" t="str">
-        <v>Kmu0warcwfc8r</v>
+        <v>Kmu0wbkulbrgg</v>
       </c>
       <c r="B2122" t="str">
         <v>Pengawas Keuangan Negara Mahir</v>
@@ -81213,7 +81213,7 @@
     </row>
     <row r="2123">
       <c r="A2123" t="str">
-        <v>Kmu0warcw2j1f</v>
+        <v>Kmu0wbkulbhac</v>
       </c>
       <c r="B2123" t="str">
         <v>Pengawas Keuangan Negara Terampil</v>
@@ -81327,7 +81327,7 @@
     </row>
     <row r="2126">
       <c r="A2126" t="str">
-        <v>Kmu0warcwemzo</v>
+        <v>Kmu0wbkulc3p3</v>
       </c>
       <c r="B2126" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81365,7 +81365,7 @@
     </row>
     <row r="2127">
       <c r="A2127" t="str">
-        <v>Kmu0warcwmge9</v>
+        <v>Kmu0wbkultgr2</v>
       </c>
       <c r="B2127" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81403,7 +81403,7 @@
     </row>
     <row r="2128">
       <c r="A2128" t="str">
-        <v>Kmu0warcwcsck</v>
+        <v>Kmu0wbkul4y24</v>
       </c>
       <c r="B2128" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81441,7 +81441,7 @@
     </row>
     <row r="2129">
       <c r="A2129" t="str">
-        <v>Kmu0warcwqd6c</v>
+        <v>Kmu0wbkullgng</v>
       </c>
       <c r="B2129" t="str">
         <v>Penata Keprotokolan*</v>
@@ -81517,7 +81517,7 @@
     </row>
     <row r="2131">
       <c r="A2131" t="str">
-        <v>Kmu0warcwmp52</v>
+        <v>Kmu0wbkulm11w</v>
       </c>
       <c r="B2131" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81555,7 +81555,7 @@
     </row>
     <row r="2132">
       <c r="A2132" t="str">
-        <v>Kmu0warcw24fu</v>
+        <v>Kmu0wbkuleoff</v>
       </c>
       <c r="B2132" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81593,7 +81593,7 @@
     </row>
     <row r="2133">
       <c r="A2133" t="str">
-        <v>Kmu0warcwixx2</v>
+        <v>Kmu0wbkulb2bm</v>
       </c>
       <c r="B2133" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81631,7 +81631,7 @@
     </row>
     <row r="2134">
       <c r="A2134" t="str">
-        <v>Kmu0warcwh9un</v>
+        <v>Kmu0wbkulx9s9</v>
       </c>
       <c r="B2134" t="str">
         <v>Penata Keprotokolan*</v>
@@ -81707,7 +81707,7 @@
     </row>
     <row r="2136">
       <c r="A2136" t="str">
-        <v>Kmu0warcwcl7j</v>
+        <v>Kmu0wbkulejy2</v>
       </c>
       <c r="B2136" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81745,7 +81745,7 @@
     </row>
     <row r="2137">
       <c r="A2137" t="str">
-        <v>Kmu0warcw2jtc</v>
+        <v>Kmu0wbkul3xmx</v>
       </c>
       <c r="B2137" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81783,7 +81783,7 @@
     </row>
     <row r="2138">
       <c r="A2138" t="str">
-        <v>Kmu0warcwof2j</v>
+        <v>Kmu0wbkul28a9</v>
       </c>
       <c r="B2138" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81821,7 +81821,7 @@
     </row>
     <row r="2139">
       <c r="A2139" t="str">
-        <v>Kmu0warcw8qa5</v>
+        <v>Kmu0wbkuln044</v>
       </c>
       <c r="B2139" t="str">
         <v>Pengawas Keuangan Negara Ahli Muda</v>
@@ -81859,7 +81859,7 @@
     </row>
     <row r="2140">
       <c r="A2140" t="str">
-        <v>Kmu0warcw0ufv</v>
+        <v>Kmu0wbkulxcza</v>
       </c>
       <c r="B2140" t="str">
         <v>Pengawas Keuangan Negara Pertama</v>
@@ -81897,7 +81897,7 @@
     </row>
     <row r="2141">
       <c r="A2141" t="str">
-        <v>Kmu0warcw8ab8</v>
+        <v>Kmu0wbkulh504</v>
       </c>
       <c r="B2141" t="str">
         <v>Penata Laksana Barang Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -81935,7 +81935,7 @@
     </row>
     <row r="2142">
       <c r="A2142" t="str">
-        <v>Kmu0warcwj15m</v>
+        <v>Kmu0wbkulvryk</v>
       </c>
       <c r="B2142" t="str">
         <v>Penata Laksana Barang Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -81973,7 +81973,7 @@
     </row>
     <row r="2143">
       <c r="A2143" t="str">
-        <v>Kmu0warcwquvg</v>
+        <v>Kmu0wbkul6gas</v>
       </c>
       <c r="B2143" t="str">
         <v>Penata Laksana Barang Terampil/ Pengawas Keuangan Negara Terampil</v>
@@ -82011,7 +82011,7 @@
     </row>
     <row r="2144">
       <c r="A2144" t="str">
-        <v>Kmu0warcw8hz3</v>
+        <v>Kmu0wbkulq72o</v>
       </c>
       <c r="B2144" t="str">
         <v>Arsiparis Ahli Muda</v>
@@ -82049,7 +82049,7 @@
     </row>
     <row r="2145">
       <c r="A2145" t="str">
-        <v>Kmu0warcwjq59</v>
+        <v>Kmu0wbkultb6z</v>
       </c>
       <c r="B2145" t="str">
         <v>Arsiparis Ahli Pertama</v>
@@ -82087,7 +82087,7 @@
     </row>
     <row r="2146">
       <c r="A2146" t="str">
-        <v>Kmu0warcwdg04</v>
+        <v>Kmu0wbkulkvkp</v>
       </c>
       <c r="B2146" t="str">
         <v>Arsiparis Penyelia</v>
@@ -82125,7 +82125,7 @@
     </row>
     <row r="2147">
       <c r="A2147" t="str">
-        <v>Kmu0warcwy8u5</v>
+        <v>Kmu0wbkulffnv</v>
       </c>
       <c r="B2147" t="str">
         <v>Arsiparis Mahir</v>
@@ -82163,7 +82163,7 @@
     </row>
     <row r="2148">
       <c r="A2148" t="str">
-        <v>Kmu0warcwqajq</v>
+        <v>Kmu0wbkulgcao</v>
       </c>
       <c r="B2148" t="str">
         <v>Arsiparis Terampil</v>
@@ -82277,7 +82277,7 @@
     </row>
     <row r="2151">
       <c r="A2151" t="str">
-        <v>Kmu0warcwlnfe</v>
+        <v>Kmu0wbkul7ls3</v>
       </c>
       <c r="B2151" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -82315,7 +82315,7 @@
     </row>
     <row r="2152">
       <c r="A2152" t="str">
-        <v>Kmu0warcwbdn1</v>
+        <v>Kmu0wbkuldutb</v>
       </c>
       <c r="B2152" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82353,7 +82353,7 @@
     </row>
     <row r="2153">
       <c r="A2153" t="str">
-        <v>Kmu0warcwyt0o</v>
+        <v>Kmu0wbkulixnm</v>
       </c>
       <c r="B2153" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82391,7 +82391,7 @@
     </row>
     <row r="2154">
       <c r="A2154" t="str">
-        <v>Kmu0warcx2ohc</v>
+        <v>Kmu0wbkulsfad</v>
       </c>
       <c r="B2154" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -82429,7 +82429,7 @@
     </row>
     <row r="2155">
       <c r="A2155" t="str">
-        <v>Kmu0warcxtgsk</v>
+        <v>Kmu0wbkulk2dk</v>
       </c>
       <c r="B2155" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -82467,7 +82467,7 @@
     </row>
     <row r="2156">
       <c r="A2156" t="str">
-        <v>Kmu0warcx2alw</v>
+        <v>Kmu0wbkulmlj1</v>
       </c>
       <c r="B2156" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -82505,7 +82505,7 @@
     </row>
     <row r="2157">
       <c r="A2157" t="str">
-        <v>Kmu0warcxmput</v>
+        <v>Kmu0wbkull1cg</v>
       </c>
       <c r="B2157" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -82581,7 +82581,7 @@
     </row>
     <row r="2159">
       <c r="A2159" t="str">
-        <v>Kmu0warcxvlth</v>
+        <v>Kmu0wbkulie74</v>
       </c>
       <c r="B2159" t="str">
         <v>Penata Layanan Operasional</v>
@@ -82619,7 +82619,7 @@
     </row>
     <row r="2160">
       <c r="A2160" t="str">
-        <v>Kmu0warcxjosu</v>
+        <v>Kmu0wbkuls5pu</v>
       </c>
       <c r="B2160" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82657,7 +82657,7 @@
     </row>
     <row r="2161">
       <c r="A2161" t="str">
-        <v>Kmu0warcxqphz</v>
+        <v>Kmu0wbkulyt81</v>
       </c>
       <c r="B2161" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82695,7 +82695,7 @@
     </row>
     <row r="2162">
       <c r="A2162" t="str">
-        <v>Kmu0warcxm7f4</v>
+        <v>Kmu0wbkulgd3j</v>
       </c>
       <c r="B2162" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -82733,7 +82733,7 @@
     </row>
     <row r="2163">
       <c r="A2163" t="str">
-        <v>Kmu0warcxsvkk</v>
+        <v>Kmu0wbkul1824</v>
       </c>
       <c r="B2163" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -82771,7 +82771,7 @@
     </row>
     <row r="2164">
       <c r="A2164" t="str">
-        <v>Kmu0warcxo9yh</v>
+        <v>Kmu0wbkulvk5g</v>
       </c>
       <c r="B2164" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -82809,7 +82809,7 @@
     </row>
     <row r="2165">
       <c r="A2165" t="str">
-        <v>Kmu0warcxedvj</v>
+        <v>Kmu0wbkuluys9</v>
       </c>
       <c r="B2165" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -82885,7 +82885,7 @@
     </row>
     <row r="2167">
       <c r="A2167" t="str">
-        <v>Kmu0warcxbjoh</v>
+        <v>Kmu0wbkul6fn8</v>
       </c>
       <c r="B2167" t="str">
         <v>Penata Layanan Operasional</v>
@@ -82923,7 +82923,7 @@
     </row>
     <row r="2168">
       <c r="A2168" t="str">
-        <v>Kmu0warcxiqrr</v>
+        <v>Kmu0wbkulj6gf</v>
       </c>
       <c r="B2168" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82961,7 +82961,7 @@
     </row>
     <row r="2169">
       <c r="A2169" t="str">
-        <v>Kmu0warcxpm3f</v>
+        <v>Kmu0wbkultjt7</v>
       </c>
       <c r="B2169" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82999,7 +82999,7 @@
     </row>
     <row r="2170">
       <c r="A2170" t="str">
-        <v>Kmu0warcxthgv</v>
+        <v>Kmu0wbkul8u24</v>
       </c>
       <c r="B2170" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -83037,7 +83037,7 @@
     </row>
     <row r="2171">
       <c r="A2171" t="str">
-        <v>Kmu0warcx5qc2</v>
+        <v>Kmu0wbkul29u1</v>
       </c>
       <c r="B2171" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -83075,7 +83075,7 @@
     </row>
     <row r="2172">
       <c r="A2172" t="str">
-        <v>Kmu0warcxi47i</v>
+        <v>Kmu0wbkul9wm0</v>
       </c>
       <c r="B2172" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -83113,7 +83113,7 @@
     </row>
     <row r="2173">
       <c r="A2173" t="str">
-        <v>Kmu0warcxbdcv</v>
+        <v>Kmu0wbkul89q4</v>
       </c>
       <c r="B2173" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -83151,7 +83151,7 @@
     </row>
     <row r="2174">
       <c r="A2174" t="str">
-        <v>Kmu0warcx887f</v>
+        <v>Kmu0wbkul1a03</v>
       </c>
       <c r="B2174" t="str">
         <v>Pranata Humas Ahli Muda</v>
@@ -83189,7 +83189,7 @@
     </row>
     <row r="2175">
       <c r="A2175" t="str">
-        <v>Kmu0warcxtfyj</v>
+        <v>Kmu0wbkul9kle</v>
       </c>
       <c r="B2175" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -83227,7 +83227,7 @@
     </row>
     <row r="2176">
       <c r="A2176" t="str">
-        <v>Kmu0warcx1c4v</v>
+        <v>Kmu0wbkulplnx</v>
       </c>
       <c r="B2176" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -83265,7 +83265,7 @@
     </row>
     <row r="2177">
       <c r="A2177" t="str">
-        <v>Kmu0warcxlepb</v>
+        <v>Kmu0wbkulfuv0</v>
       </c>
       <c r="B2177" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -83303,7 +83303,7 @@
     </row>
     <row r="2178">
       <c r="A2178" t="str">
-        <v>Kmu0warcx0yxx</v>
+        <v>Kmu0wbkulkesi</v>
       </c>
       <c r="B2178" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -83341,7 +83341,7 @@
     </row>
     <row r="2179">
       <c r="A2179" t="str">
-        <v>Kmu0warcxuiw4</v>
+        <v>Kmu0wbkul31uh</v>
       </c>
       <c r="B2179" t="str">
         <v>Pustakawan Ahli Pertama</v>
@@ -83379,7 +83379,7 @@
     </row>
     <row r="2180">
       <c r="A2180" t="str">
-        <v>Kmu0warcx02xw</v>
+        <v>Kmu0wbkulg67l</v>
       </c>
       <c r="B2180" t="str">
         <v>Asisten Perpustakaan Penyelia</v>
@@ -83417,7 +83417,7 @@
     </row>
     <row r="2181">
       <c r="A2181" t="str">
-        <v>Kmu0warcxx6vj</v>
+        <v>Kmu0wbkul3sl0</v>
       </c>
       <c r="B2181" t="str">
         <v>Asisten Perpustakaan Mahir</v>
@@ -83455,7 +83455,7 @@
     </row>
     <row r="2182">
       <c r="A2182" t="str">
-        <v>Kmu0warcxto5j</v>
+        <v>Kmu0wbkulvffd</v>
       </c>
       <c r="B2182" t="str">
         <v>Asisten Perpustakaan Terampil</v>
@@ -83493,7 +83493,7 @@
     </row>
     <row r="2183">
       <c r="A2183" t="str">
-        <v>Kmu0warcxr2u8</v>
+        <v>Kmu0wbkul13bj</v>
       </c>
       <c r="B2183" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Madya/Pengawas Keuangan Negara Ahli Madya</v>
@@ -83531,7 +83531,7 @@
     </row>
     <row r="2184">
       <c r="A2184" t="str">
-        <v>Kmu0warcxmgnz</v>
+        <v>Kmu0wbkulls78</v>
       </c>
       <c r="B2184" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Muda</v>
@@ -83569,7 +83569,7 @@
     </row>
     <row r="2185">
       <c r="A2185" t="str">
-        <v>Kmu0warcx4axz</v>
+        <v>Kmu0wbkul1db7</v>
       </c>
       <c r="B2185" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Pertama</v>
@@ -83683,7 +83683,7 @@
     </row>
     <row r="2188">
       <c r="A2188" t="str">
-        <v>Kmu0warcx5l8t</v>
+        <v>Kmu0wbkulfycv</v>
       </c>
       <c r="B2188" t="str">
         <v>Penata Layanan Operasional</v>
@@ -83721,7 +83721,7 @@
     </row>
     <row r="2189">
       <c r="A2189" t="str">
-        <v>Kmu0warcxxkz7</v>
+        <v>Kmu0wbkulpc1f</v>
       </c>
       <c r="B2189" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -83759,7 +83759,7 @@
     </row>
     <row r="2190">
       <c r="A2190" t="str">
-        <v>Kmu0warcxjjy8</v>
+        <v>Kmu0wbkul16nw</v>
       </c>
       <c r="B2190" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -83797,7 +83797,7 @@
     </row>
     <row r="2191">
       <c r="A2191" t="str">
-        <v>Kmu0warcxrheo</v>
+        <v>Kmu0wbkulmf11</v>
       </c>
       <c r="B2191" t="str">
         <v>Penata Keprotokolan*</v>
@@ -83911,7 +83911,7 @@
     </row>
     <row r="2194">
       <c r="A2194" t="str">
-        <v>Kmu0warcxx4jv</v>
+        <v>Kmu0wbkulwr43</v>
       </c>
       <c r="B2194" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -83949,7 +83949,7 @@
     </row>
     <row r="2195">
       <c r="A2195" t="str">
-        <v>Kmu0warcx5jnv</v>
+        <v>Kmu0wbkul3dzf</v>
       </c>
       <c r="B2195" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -83987,7 +83987,7 @@
     </row>
     <row r="2196">
       <c r="A2196" t="str">
-        <v>Kmu0warcxt4is</v>
+        <v>Kmu0wbkuluupe</v>
       </c>
       <c r="B2196" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84063,7 +84063,7 @@
     </row>
     <row r="2198">
       <c r="A2198" t="str">
-        <v>Kmu0warcxwocg</v>
+        <v>Kmu0wbkulrw21</v>
       </c>
       <c r="B2198" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84101,7 +84101,7 @@
     </row>
     <row r="2199">
       <c r="A2199" t="str">
-        <v>Kmu0warcxl3my</v>
+        <v>Kmu0wbkul02lf</v>
       </c>
       <c r="B2199" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84139,7 +84139,7 @@
     </row>
     <row r="2200">
       <c r="A2200" t="str">
-        <v>Kmu0warcxyew7</v>
+        <v>Kmu0wbkul731s</v>
       </c>
       <c r="B2200" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84177,7 +84177,7 @@
     </row>
     <row r="2201">
       <c r="A2201" t="str">
-        <v>Kmu0warcx5atg</v>
+        <v>Kmu0wbkulq2ir</v>
       </c>
       <c r="B2201" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -84215,7 +84215,7 @@
     </row>
     <row r="2202">
       <c r="A2202" t="str">
-        <v>Kmu0warcxntnk</v>
+        <v>Kmu0wbkulx4t7</v>
       </c>
       <c r="B2202" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -84253,7 +84253,7 @@
     </row>
     <row r="2203">
       <c r="A2203" t="str">
-        <v>Kmu0warcxe0fi</v>
+        <v>Kmu0wbkulbdf2</v>
       </c>
       <c r="B2203" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -84291,7 +84291,7 @@
     </row>
     <row r="2204">
       <c r="A2204" t="str">
-        <v>Kmu0warcx4a8d</v>
+        <v>Kmu0wbkul3kp7</v>
       </c>
       <c r="B2204" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -84405,7 +84405,7 @@
     </row>
     <row r="2207">
       <c r="A2207" t="str">
-        <v>Kmu0warcxj8t0</v>
+        <v>Kmu0wbkulhdw6</v>
       </c>
       <c r="B2207" t="str">
         <v>Penata Layanan Operasional</v>
@@ -84443,7 +84443,7 @@
     </row>
     <row r="2208">
       <c r="A2208" t="str">
-        <v>Kmu0warcx9lri</v>
+        <v>Kmu0wbkuly6dz</v>
       </c>
       <c r="B2208" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84481,7 +84481,7 @@
     </row>
     <row r="2209">
       <c r="A2209" t="str">
-        <v>Kmu0warcx7c4c</v>
+        <v>Kmu0wbkul7er3</v>
       </c>
       <c r="B2209" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84519,7 +84519,7 @@
     </row>
     <row r="2210">
       <c r="A2210" t="str">
-        <v>Kmu0warcxkgyw</v>
+        <v>Kmu0wbkulc2ep</v>
       </c>
       <c r="B2210" t="str">
         <v>Penata Keprotokolan*</v>
@@ -84633,7 +84633,7 @@
     </row>
     <row r="2213">
       <c r="A2213" t="str">
-        <v>Kmu0warcx6vic</v>
+        <v>Kmu0wbkulp8kh</v>
       </c>
       <c r="B2213" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84671,7 +84671,7 @@
     </row>
     <row r="2214">
       <c r="A2214" t="str">
-        <v>Kmu0warcxvmz6</v>
+        <v>Kmu0wbkul1ezq</v>
       </c>
       <c r="B2214" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84709,7 +84709,7 @@
     </row>
     <row r="2215">
       <c r="A2215" t="str">
-        <v>Kmu0warcxfzc2</v>
+        <v>Kmu0wbkulj32n</v>
       </c>
       <c r="B2215" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84785,7 +84785,7 @@
     </row>
     <row r="2217">
       <c r="A2217" t="str">
-        <v>Kmu0warcxm4fv</v>
+        <v>Kmu0wbkulci0y</v>
       </c>
       <c r="B2217" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84823,7 +84823,7 @@
     </row>
     <row r="2218">
       <c r="A2218" t="str">
-        <v>Kmu0warcxz8fb</v>
+        <v>Kmu0wbkuloor6</v>
       </c>
       <c r="B2218" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84861,7 +84861,7 @@
     </row>
     <row r="2219">
       <c r="A2219" t="str">
-        <v>Kmu0warcx24du</v>
+        <v>Kmu0wbkuldmmu</v>
       </c>
       <c r="B2219" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84899,7 +84899,7 @@
     </row>
     <row r="2220">
       <c r="A2220" t="str">
-        <v>Kmu0warcxh9d7</v>
+        <v>Kmu0wbkul3f5l</v>
       </c>
       <c r="B2220" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -84937,7 +84937,7 @@
     </row>
     <row r="2221">
       <c r="A2221" t="str">
-        <v>Kmu0warcxni1q</v>
+        <v>Kmu0wbkul3wmr</v>
       </c>
       <c r="B2221" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -84975,7 +84975,7 @@
     </row>
     <row r="2222">
       <c r="A2222" t="str">
-        <v>Kmu0warcxj36w</v>
+        <v>Kmu0wbkulien7</v>
       </c>
       <c r="B2222" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -85013,7 +85013,7 @@
     </row>
     <row r="2223">
       <c r="A2223" t="str">
-        <v>Kmu0warcxslgw</v>
+        <v>Kmu0wbkulw7jv</v>
       </c>
       <c r="B2223" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -85127,7 +85127,7 @@
     </row>
     <row r="2226">
       <c r="A2226" t="str">
-        <v>Kmu0warcxzxhp</v>
+        <v>Kmu0wbkul4qrb</v>
       </c>
       <c r="B2226" t="str">
         <v>Penata Layanan Operasional</v>
@@ -85165,7 +85165,7 @@
     </row>
     <row r="2227">
       <c r="A2227" t="str">
-        <v>Kmu0warcx97ct</v>
+        <v>Kmu0wbkulewlc</v>
       </c>
       <c r="B2227" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85203,7 +85203,7 @@
     </row>
     <row r="2228">
       <c r="A2228" t="str">
-        <v>Kmu0warcxb610</v>
+        <v>Kmu0wbkul8cvs</v>
       </c>
       <c r="B2228" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85241,7 +85241,7 @@
     </row>
     <row r="2229">
       <c r="A2229" t="str">
-        <v>Kmu0warcxdh61</v>
+        <v>Kmu0wbkul23ij</v>
       </c>
       <c r="B2229" t="str">
         <v>Penata Keprotokolan*</v>
@@ -85355,7 +85355,7 @@
     </row>
     <row r="2232">
       <c r="A2232" t="str">
-        <v>Kmu0warcxfqd9</v>
+        <v>Kmu0wbkul57kz</v>
       </c>
       <c r="B2232" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -85393,7 +85393,7 @@
     </row>
     <row r="2233">
       <c r="A2233" t="str">
-        <v>Kmu0warcxw65n</v>
+        <v>Kmu0wbkulcedd</v>
       </c>
       <c r="B2233" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85431,7 +85431,7 @@
     </row>
     <row r="2234">
       <c r="A2234" t="str">
-        <v>Kmu0warcx6rzr</v>
+        <v>Kmu0wbkulgfsl</v>
       </c>
       <c r="B2234" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85507,7 +85507,7 @@
     </row>
     <row r="2236">
       <c r="A2236" t="str">
-        <v>Kmu0warcx0k33</v>
+        <v>Kmu0wbkulcny4</v>
       </c>
       <c r="B2236" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -85545,7 +85545,7 @@
     </row>
     <row r="2237">
       <c r="A2237" t="str">
-        <v>Kmu0warcxv951</v>
+        <v>Kmu0wbkul35to</v>
       </c>
       <c r="B2237" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85583,7 +85583,7 @@
     </row>
     <row r="2238">
       <c r="A2238" t="str">
-        <v>Kmu0warcxv572</v>
+        <v>Kmu0wbkulvt6q</v>
       </c>
       <c r="B2238" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85621,7 +85621,7 @@
     </row>
     <row r="2239">
       <c r="A2239" t="str">
-        <v>Kmu0warcxwkye</v>
+        <v>Kmu0wbkulegj2</v>
       </c>
       <c r="B2239" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -85659,7 +85659,7 @@
     </row>
     <row r="2240">
       <c r="A2240" t="str">
-        <v>Kmu0warcxny41</v>
+        <v>Kmu0wbkulpkpd</v>
       </c>
       <c r="B2240" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -85697,7 +85697,7 @@
     </row>
     <row r="2241">
       <c r="A2241" t="str">
-        <v>Kmu0warcxl3r1</v>
+        <v>Kmu0wbkula0df</v>
       </c>
       <c r="B2241" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -85735,7 +85735,7 @@
     </row>
     <row r="2242">
       <c r="A2242" t="str">
-        <v>Kmu0warcxuab7</v>
+        <v>Kmu0wbkulc4qm</v>
       </c>
       <c r="B2242" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -85849,7 +85849,7 @@
     </row>
     <row r="2245">
       <c r="A2245" t="str">
-        <v>Kmu0warcxlfz1</v>
+        <v>Kmu0wbkul4a2t</v>
       </c>
       <c r="B2245" t="str">
         <v>Penata Layanan Operasional</v>
@@ -85887,7 +85887,7 @@
     </row>
     <row r="2246">
       <c r="A2246" t="str">
-        <v>Kmu0warcx36ui</v>
+        <v>Kmu0wbkulp263</v>
       </c>
       <c r="B2246" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85925,7 +85925,7 @@
     </row>
     <row r="2247">
       <c r="A2247" t="str">
-        <v>Kmu0warcxotly</v>
+        <v>Kmu0wbkul7a88</v>
       </c>
       <c r="B2247" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85963,7 +85963,7 @@
     </row>
     <row r="2248">
       <c r="A2248" t="str">
-        <v>Kmu0warcx4pvd</v>
+        <v>Kmu0wbkultw1j</v>
       </c>
       <c r="B2248" t="str">
         <v>Penata Keprotokolan*</v>
@@ -86039,7 +86039,7 @@
     </row>
     <row r="2250">
       <c r="A2250" t="str">
-        <v>Kmu0warcxgyux</v>
+        <v>Kmu0wbkulftsf</v>
       </c>
       <c r="B2250" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86077,7 +86077,7 @@
     </row>
     <row r="2251">
       <c r="A2251" t="str">
-        <v>Kmu0warcx9oah</v>
+        <v>Kmu0wbkullfig</v>
       </c>
       <c r="B2251" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86115,7 +86115,7 @@
     </row>
     <row r="2252">
       <c r="A2252" t="str">
-        <v>Kmu0warcx4s9e</v>
+        <v>Kmu0wbkulab7f</v>
       </c>
       <c r="B2252" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86153,7 +86153,7 @@
     </row>
     <row r="2253">
       <c r="A2253" t="str">
-        <v>Kmu0warcxh2j0</v>
+        <v>Kmu0wbkul5jk8</v>
       </c>
       <c r="B2253" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -86191,7 +86191,7 @@
     </row>
     <row r="2254">
       <c r="A2254" t="str">
-        <v>Kmu0warcxn71q</v>
+        <v>Kmu0wbkul2txa</v>
       </c>
       <c r="B2254" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -86305,7 +86305,7 @@
     </row>
     <row r="2257">
       <c r="A2257" t="str">
-        <v>Kmu0warcxabfg</v>
+        <v>Kmu0wbkulqzx6</v>
       </c>
       <c r="B2257" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86343,7 +86343,7 @@
     </row>
     <row r="2258">
       <c r="A2258" t="str">
-        <v>Kmu0warcx9pw1</v>
+        <v>Kmu0wbkululwd</v>
       </c>
       <c r="B2258" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86381,7 +86381,7 @@
     </row>
     <row r="2259">
       <c r="A2259" t="str">
-        <v>Kmu0warcxi03i</v>
+        <v>Kmu0wbkulxnnl</v>
       </c>
       <c r="B2259" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86457,7 +86457,7 @@
     </row>
     <row r="2261">
       <c r="A2261" t="str">
-        <v>Kmu0warcxxl8r</v>
+        <v>Kmu0wbkulp6kr</v>
       </c>
       <c r="B2261" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86495,7 +86495,7 @@
     </row>
     <row r="2262">
       <c r="A2262" t="str">
-        <v>Kmu0warcx0z1b</v>
+        <v>Kmu0wbkul2rtj</v>
       </c>
       <c r="B2262" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86533,7 +86533,7 @@
     </row>
     <row r="2263">
       <c r="A2263" t="str">
-        <v>Kmu0warcxospw</v>
+        <v>Kmu0wbkul9fsq</v>
       </c>
       <c r="B2263" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86571,7 +86571,7 @@
     </row>
     <row r="2264">
       <c r="A2264" t="str">
-        <v>Kmu0warcxut7o</v>
+        <v>Kmu0wbkul5kmt</v>
       </c>
       <c r="B2264" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -86609,7 +86609,7 @@
     </row>
     <row r="2265">
       <c r="A2265" t="str">
-        <v>Kmu0warcx3y0d</v>
+        <v>Kmu0wbkul0a65</v>
       </c>
       <c r="B2265" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -86647,7 +86647,7 @@
     </row>
     <row r="2266">
       <c r="A2266" t="str">
-        <v>Kmu0warcxi7l2</v>
+        <v>Kmu0wbkuln9sw</v>
       </c>
       <c r="B2266" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -86685,7 +86685,7 @@
     </row>
     <row r="2267">
       <c r="A2267" t="str">
-        <v>Kmu0warcxro7k</v>
+        <v>Kmu0wbkul8pl1</v>
       </c>
       <c r="B2267" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -86799,7 +86799,7 @@
     </row>
     <row r="2270">
       <c r="A2270" t="str">
-        <v>Kmu0warcxtha6</v>
+        <v>Kmu0wbkulz61t</v>
       </c>
       <c r="B2270" t="str">
         <v>Penata Layanan Operasional</v>
@@ -86837,7 +86837,7 @@
     </row>
     <row r="2271">
       <c r="A2271" t="str">
-        <v>Kmu0warcxzxd4</v>
+        <v>Kmu0wbkule85n</v>
       </c>
       <c r="B2271" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86875,7 +86875,7 @@
     </row>
     <row r="2272">
       <c r="A2272" t="str">
-        <v>Kmu0warcxl28u</v>
+        <v>Kmu0wbkul75da</v>
       </c>
       <c r="B2272" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86913,7 +86913,7 @@
     </row>
     <row r="2273">
       <c r="A2273" t="str">
-        <v>Kmu0warcx1k9m</v>
+        <v>Kmu0wbkulgs67</v>
       </c>
       <c r="B2273" t="str">
         <v>Penata Keprotokolan*</v>
@@ -87027,7 +87027,7 @@
     </row>
     <row r="2276">
       <c r="A2276" t="str">
-        <v>Kmu0warcxofyf</v>
+        <v>Kmu0wbkulpmh9</v>
       </c>
       <c r="B2276" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87065,7 +87065,7 @@
     </row>
     <row r="2277">
       <c r="A2277" t="str">
-        <v>Kmu0warcx16d6</v>
+        <v>Kmu0wbkull56u</v>
       </c>
       <c r="B2277" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87103,7 +87103,7 @@
     </row>
     <row r="2278">
       <c r="A2278" t="str">
-        <v>Kmu0warcxbcfi</v>
+        <v>Kmu0wbkullopb</v>
       </c>
       <c r="B2278" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87179,7 +87179,7 @@
     </row>
     <row r="2280">
       <c r="A2280" t="str">
-        <v>Kmu0warcxxt9t</v>
+        <v>Kmu0wbkulyrvi</v>
       </c>
       <c r="B2280" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87217,7 +87217,7 @@
     </row>
     <row r="2281">
       <c r="A2281" t="str">
-        <v>Kmu0warcxgyjq</v>
+        <v>Kmu0wbkulgv84</v>
       </c>
       <c r="B2281" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87255,7 +87255,7 @@
     </row>
     <row r="2282">
       <c r="A2282" t="str">
-        <v>Kmu0warcxam8k</v>
+        <v>Kmu0wbkuly8jo</v>
       </c>
       <c r="B2282" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87293,7 +87293,7 @@
     </row>
     <row r="2283">
       <c r="A2283" t="str">
-        <v>Kmu0warcxqruo</v>
+        <v>Kmu0wbkul3cy6</v>
       </c>
       <c r="B2283" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -87331,7 +87331,7 @@
     </row>
     <row r="2284">
       <c r="A2284" t="str">
-        <v>Kmu0warcxnyjq</v>
+        <v>Kmu0wbkulymhv</v>
       </c>
       <c r="B2284" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -87369,7 +87369,7 @@
     </row>
     <row r="2285">
       <c r="A2285" t="str">
-        <v>Kmu0warcxg1xz</v>
+        <v>Kmu0wbkulveq7</v>
       </c>
       <c r="B2285" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -87407,7 +87407,7 @@
     </row>
     <row r="2286">
       <c r="A2286" t="str">
-        <v>Kmu0warcx3341</v>
+        <v>Kmu0wbkulyqsd</v>
       </c>
       <c r="B2286" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -87521,7 +87521,7 @@
     </row>
     <row r="2289">
       <c r="A2289" t="str">
-        <v>Kmu0warcxzbzy</v>
+        <v>Kmu0wbkul9oqk</v>
       </c>
       <c r="B2289" t="str">
         <v>Penata Layanan Operasional</v>
@@ -87559,7 +87559,7 @@
     </row>
     <row r="2290">
       <c r="A2290" t="str">
-        <v>Kmu0warcximl4</v>
+        <v>Kmu0wbkulit4v</v>
       </c>
       <c r="B2290" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87597,7 +87597,7 @@
     </row>
     <row r="2291">
       <c r="A2291" t="str">
-        <v>Kmu0warcx8y4r</v>
+        <v>Kmu0wbkulmx2e</v>
       </c>
       <c r="B2291" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87635,7 +87635,7 @@
     </row>
     <row r="2292">
       <c r="A2292" t="str">
-        <v>Kmu0warcxmqni</v>
+        <v>Kmu0wbkulaws9</v>
       </c>
       <c r="B2292" t="str">
         <v>Penata Keprotokolan*</v>
@@ -87749,7 +87749,7 @@
     </row>
     <row r="2295">
       <c r="A2295" t="str">
-        <v>Kmu0warcx6w6u</v>
+        <v>Kmu0wbkulgkji</v>
       </c>
       <c r="B2295" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87787,7 +87787,7 @@
     </row>
     <row r="2296">
       <c r="A2296" t="str">
-        <v>Kmu0warcxsffa</v>
+        <v>Kmu0wbkulfz8d</v>
       </c>
       <c r="B2296" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87825,7 +87825,7 @@
     </row>
     <row r="2297">
       <c r="A2297" t="str">
-        <v>Kmu0warcx9r5v</v>
+        <v>Kmu0wbkulgy6u</v>
       </c>
       <c r="B2297" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87901,7 +87901,7 @@
     </row>
     <row r="2299">
       <c r="A2299" t="str">
-        <v>Kmu0warcxmk9a</v>
+        <v>Kmu0wbkul73od</v>
       </c>
       <c r="B2299" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87939,7 +87939,7 @@
     </row>
     <row r="2300">
       <c r="A2300" t="str">
-        <v>Kmu0warcxm99i</v>
+        <v>Kmu0wbkulyc8c</v>
       </c>
       <c r="B2300" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87977,7 +87977,7 @@
     </row>
     <row r="2301">
       <c r="A2301" t="str">
-        <v>Kmu0warcxv5pj</v>
+        <v>Kmu0wbkulv2wt</v>
       </c>
       <c r="B2301" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88015,7 +88015,7 @@
     </row>
     <row r="2302">
       <c r="A2302" t="str">
-        <v>Kmu0warcxbbtn</v>
+        <v>Kmu0wbkulat59</v>
       </c>
       <c r="B2302" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -88053,7 +88053,7 @@
     </row>
     <row r="2303">
       <c r="A2303" t="str">
-        <v>Kmu0warcxm72a</v>
+        <v>Kmu0wbkulw1oc</v>
       </c>
       <c r="B2303" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -88091,7 +88091,7 @@
     </row>
     <row r="2304">
       <c r="A2304" t="str">
-        <v>Kmu0warcxdy5k</v>
+        <v>Kmu0wbkul0s3o</v>
       </c>
       <c r="B2304" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -88129,7 +88129,7 @@
     </row>
     <row r="2305">
       <c r="A2305" t="str">
-        <v>Kmu0warcxpv8b</v>
+        <v>Kmu0wbkulbzkr</v>
       </c>
       <c r="B2305" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -88243,7 +88243,7 @@
     </row>
     <row r="2308">
       <c r="A2308" t="str">
-        <v>Kmu0warcxukt4</v>
+        <v>Kmu0wbkulkb0q</v>
       </c>
       <c r="B2308" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88281,7 +88281,7 @@
     </row>
     <row r="2309">
       <c r="A2309" t="str">
-        <v>Kmu0warcxpjd2</v>
+        <v>Kmu0wbkulwny5</v>
       </c>
       <c r="B2309" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88319,7 +88319,7 @@
     </row>
     <row r="2310">
       <c r="A2310" t="str">
-        <v>Kmu0warcxcrlw</v>
+        <v>Kmu0wbkulrplf</v>
       </c>
       <c r="B2310" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88357,7 +88357,7 @@
     </row>
     <row r="2311">
       <c r="A2311" t="str">
-        <v>Kmu0warcxua0m</v>
+        <v>Kmu0wbkulvmb7</v>
       </c>
       <c r="B2311" t="str">
         <v>Penata Keprotokolan*</v>
@@ -88471,7 +88471,7 @@
     </row>
     <row r="2314">
       <c r="A2314" t="str">
-        <v>Kmu0warcx3pz1</v>
+        <v>Kmu0wbkulb38d</v>
       </c>
       <c r="B2314" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88509,7 +88509,7 @@
     </row>
     <row r="2315">
       <c r="A2315" t="str">
-        <v>Kmu0warcxx84d</v>
+        <v>Kmu0wbkulcn1d</v>
       </c>
       <c r="B2315" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88547,7 +88547,7 @@
     </row>
     <row r="2316">
       <c r="A2316" t="str">
-        <v>Kmu0warcxuohe</v>
+        <v>Kmu0wbkuljyfd</v>
       </c>
       <c r="B2316" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88623,7 +88623,7 @@
     </row>
     <row r="2318">
       <c r="A2318" t="str">
-        <v>Kmu0warcxswp2</v>
+        <v>Kmu0wbkullzra</v>
       </c>
       <c r="B2318" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88661,7 +88661,7 @@
     </row>
     <row r="2319">
       <c r="A2319" t="str">
-        <v>Kmu0warcxap7x</v>
+        <v>Kmu0wbkumxv1m</v>
       </c>
       <c r="B2319" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88699,7 +88699,7 @@
     </row>
     <row r="2320">
       <c r="A2320" t="str">
-        <v>Kmu0warcxqrva</v>
+        <v>Kmu0wbkumgmpr</v>
       </c>
       <c r="B2320" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88775,7 +88775,7 @@
     </row>
     <row r="2322">
       <c r="A2322" t="str">
-        <v>Kmu0warcx2hd4</v>
+        <v>Kmu0wbkumzl02</v>
       </c>
       <c r="B2322" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88813,7 +88813,7 @@
     </row>
     <row r="2323">
       <c r="A2323" t="str">
-        <v>Kmu0warcxospp</v>
+        <v>Kmu0wbkumloo5</v>
       </c>
       <c r="B2323" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88851,7 +88851,7 @@
     </row>
     <row r="2324">
       <c r="A2324" t="str">
-        <v>Kmu0warcxfbfb</v>
+        <v>Kmu0wbkumwoli</v>
       </c>
       <c r="B2324" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88927,7 +88927,7 @@
     </row>
     <row r="2326">
       <c r="A2326" t="str">
-        <v>Kmu0warcxcvnf</v>
+        <v>Kmu0wbkumjffi</v>
       </c>
       <c r="B2326" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88965,7 +88965,7 @@
     </row>
     <row r="2327">
       <c r="A2327" t="str">
-        <v>Kmu0warcxevnv</v>
+        <v>Kmu0wbkum7obe</v>
       </c>
       <c r="B2327" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89003,7 +89003,7 @@
     </row>
     <row r="2328">
       <c r="A2328" t="str">
-        <v>Kmu0warcxcmcj</v>
+        <v>Kmu0wbkumqvid</v>
       </c>
       <c r="B2328" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89117,7 +89117,7 @@
     </row>
     <row r="2331">
       <c r="A2331" t="str">
-        <v>Kmu0warcxdzjx</v>
+        <v>Kmu0wbkumhutg</v>
       </c>
       <c r="B2331" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89155,7 +89155,7 @@
     </row>
     <row r="2332">
       <c r="A2332" t="str">
-        <v>Kmu0warcxvy0k</v>
+        <v>Kmu0wbkumib53</v>
       </c>
       <c r="B2332" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89193,7 +89193,7 @@
     </row>
     <row r="2333">
       <c r="A2333" t="str">
-        <v>Kmu0warcxkrcg</v>
+        <v>Kmu0wbkumum19</v>
       </c>
       <c r="B2333" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89269,7 +89269,7 @@
     </row>
     <row r="2335">
       <c r="A2335" t="str">
-        <v>Kmu0warcxygsq</v>
+        <v>Kmu0wbkummibv</v>
       </c>
       <c r="B2335" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89307,7 +89307,7 @@
     </row>
     <row r="2336">
       <c r="A2336" t="str">
-        <v>Kmu0warcxpdc3</v>
+        <v>Kmu0wbkumvsba</v>
       </c>
       <c r="B2336" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89345,7 +89345,7 @@
     </row>
     <row r="2337">
       <c r="A2337" t="str">
-        <v>Kmu0warcx9e22</v>
+        <v>Kmu0wbkumi91j</v>
       </c>
       <c r="B2337" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89383,7 +89383,7 @@
     </row>
     <row r="2338">
       <c r="A2338" t="str">
-        <v>Kmu0warcxarnk</v>
+        <v>Kmu0wbkumi9yn</v>
       </c>
       <c r="B2338" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -89421,7 +89421,7 @@
     </row>
     <row r="2339">
       <c r="A2339" t="str">
-        <v>Kmu0warcxm197</v>
+        <v>Kmu0wbkum88xx</v>
       </c>
       <c r="B2339" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -89459,7 +89459,7 @@
     </row>
     <row r="2340">
       <c r="A2340" t="str">
-        <v>Kmu0warcx55ca</v>
+        <v>Kmu0wbkum62bu</v>
       </c>
       <c r="B2340" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -89497,7 +89497,7 @@
     </row>
     <row r="2341">
       <c r="A2341" t="str">
-        <v>Kmu0warcxz297</v>
+        <v>Kmu0wbkumbj38</v>
       </c>
       <c r="B2341" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -89611,7 +89611,7 @@
     </row>
     <row r="2344">
       <c r="A2344" t="str">
-        <v>Kmu0warcxredm</v>
+        <v>Kmu0wbkum6ig0</v>
       </c>
       <c r="B2344" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89649,7 +89649,7 @@
     </row>
     <row r="2345">
       <c r="A2345" t="str">
-        <v>Kmu0warcx98r7</v>
+        <v>Kmu0wbkumjd4n</v>
       </c>
       <c r="B2345" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89687,7 +89687,7 @@
     </row>
     <row r="2346">
       <c r="A2346" t="str">
-        <v>Kmu0warcx5zcq</v>
+        <v>Kmu0wbkum25o4</v>
       </c>
       <c r="B2346" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89801,7 +89801,7 @@
     </row>
     <row r="2349">
       <c r="A2349" t="str">
-        <v>Kmu0warcx419k</v>
+        <v>Kmu0wbkumycb0</v>
       </c>
       <c r="B2349" t="str">
         <v>Penata Layanan Operasional</v>
@@ -89839,7 +89839,7 @@
     </row>
     <row r="2350">
       <c r="A2350" t="str">
-        <v>Kmu0warcxd3sb</v>
+        <v>Kmu0wbkumqu5h</v>
       </c>
       <c r="B2350" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89877,7 +89877,7 @@
     </row>
     <row r="2351">
       <c r="A2351" t="str">
-        <v>Kmu0warcx9xs0</v>
+        <v>Kmu0wbkum2stk</v>
       </c>
       <c r="B2351" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89953,7 +89953,7 @@
     </row>
     <row r="2353">
       <c r="A2353" t="str">
-        <v>Kmu0warcx5row</v>
+        <v>Kmu0wbkumxdtm</v>
       </c>
       <c r="B2353" t="str">
         <v>Penata Layanan Operasional</v>
@@ -89991,7 +89991,7 @@
     </row>
     <row r="2354">
       <c r="A2354" t="str">
-        <v>Kmu0warcxfm49</v>
+        <v>Kmu0wbkumt9ik</v>
       </c>
       <c r="B2354" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90029,7 +90029,7 @@
     </row>
     <row r="2355">
       <c r="A2355" t="str">
-        <v>Kmu0warcxeom5</v>
+        <v>Kmu0wbkumt0l7</v>
       </c>
       <c r="B2355" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90067,7 +90067,7 @@
     </row>
     <row r="2356">
       <c r="A2356" t="str">
-        <v>Kmu0warcx8j6a</v>
+        <v>Kmu0wbkumywxo</v>
       </c>
       <c r="B2356" t="str">
         <v>Penata Keprotokolan*</v>
@@ -90143,7 +90143,7 @@
     </row>
     <row r="2358">
       <c r="A2358" t="str">
-        <v>Kmu0warcxol6b</v>
+        <v>Kmu0wbkumcah5</v>
       </c>
       <c r="B2358" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90181,7 +90181,7 @@
     </row>
     <row r="2359">
       <c r="A2359" t="str">
-        <v>Kmu0warcxf9p4</v>
+        <v>Kmu0wbkume0gy</v>
       </c>
       <c r="B2359" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90219,7 +90219,7 @@
     </row>
     <row r="2360">
       <c r="A2360" t="str">
-        <v>Kmu0warcxv686</v>
+        <v>Kmu0wbkumy8nm</v>
       </c>
       <c r="B2360" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90333,7 +90333,7 @@
     </row>
     <row r="2363">
       <c r="A2363" t="str">
-        <v>Kmu0warcxvzq6</v>
+        <v>Kmu0wbkumdnp8</v>
       </c>
       <c r="B2363" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -90371,7 +90371,7 @@
     </row>
     <row r="2364">
       <c r="A2364" t="str">
-        <v>Kmu0warcxzc4b</v>
+        <v>Kmu0wbkumku5y</v>
       </c>
       <c r="B2364" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90409,7 +90409,7 @@
     </row>
     <row r="2365">
       <c r="A2365" t="str">
-        <v>Kmu0warcx1ale</v>
+        <v>Kmu0wbkuml99x</v>
       </c>
       <c r="B2365" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90485,7 +90485,7 @@
     </row>
     <row r="2367">
       <c r="A2367" t="str">
-        <v>Kmu0warcx2089</v>
+        <v>Kmu0wbkum0m6k</v>
       </c>
       <c r="B2367" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90523,7 +90523,7 @@
     </row>
     <row r="2368">
       <c r="A2368" t="str">
-        <v>Kmu0warcxyn6r</v>
+        <v>Kmu0wbkumwd63</v>
       </c>
       <c r="B2368" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90561,7 +90561,7 @@
     </row>
     <row r="2369">
       <c r="A2369" t="str">
-        <v>Kmu0warcxjwvc</v>
+        <v>Kmu0wbkumkgm5</v>
       </c>
       <c r="B2369" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90637,7 +90637,7 @@
     </row>
     <row r="2371">
       <c r="A2371" t="str">
-        <v>Kmu0warcxyh5w</v>
+        <v>Kmu0wbkum2a8b</v>
       </c>
       <c r="B2371" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -90675,7 +90675,7 @@
     </row>
     <row r="2372">
       <c r="A2372" t="str">
-        <v>Kmu0warcxhyec</v>
+        <v>Kmu0wbkum53bg</v>
       </c>
       <c r="B2372" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90713,7 +90713,7 @@
     </row>
     <row r="2373">
       <c r="A2373" t="str">
-        <v>Kmu0warcx0tya</v>
+        <v>Kmu0wbkumigqz</v>
       </c>
       <c r="B2373" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90789,7 +90789,7 @@
     </row>
     <row r="2375">
       <c r="A2375" t="str">
-        <v>Kmu0warcx2n3y</v>
+        <v>Kmu0wbkummif7</v>
       </c>
       <c r="B2375" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90827,7 +90827,7 @@
     </row>
     <row r="2376">
       <c r="A2376" t="str">
-        <v>Kmu0warcxndn0</v>
+        <v>Kmu0wbkumain9</v>
       </c>
       <c r="B2376" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90865,7 +90865,7 @@
     </row>
     <row r="2377">
       <c r="A2377" t="str">
-        <v>Kmu0warcx60nr</v>
+        <v>Kmu0wbkumegn6</v>
       </c>
       <c r="B2377" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90903,7 +90903,7 @@
     </row>
     <row r="2378">
       <c r="A2378" t="str">
-        <v>Kmu0warcx3h0z</v>
+        <v>Kmu0wbkum5f2k</v>
       </c>
       <c r="B2378" t="str">
         <v xml:space="preserve">Analis Pembiayaan Risiko dan Keuangan/ Analis Keuangan Negara Ahli Utama									</v>

</xml_diff>

<commit_message>
Perbarui struktur organisasi (2026-09-14T07:04:02.984Z)
</commit_message>
<xml_diff>
--- a/data/struktur-organisasi.xlsx
+++ b/data/struktur-organisasi.xlsx
@@ -78173,7 +78173,7 @@
     </row>
     <row r="2043">
       <c r="A2043" t="str">
-        <v>Kmu0wc9rujtz8</v>
+        <v>Kmu0wctkt5ir5</v>
       </c>
       <c r="B2043" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78211,7 +78211,7 @@
     </row>
     <row r="2044">
       <c r="A2044" t="str">
-        <v>Kmu0wc9rurj0c</v>
+        <v>Kmu0wctktvsxv</v>
       </c>
       <c r="B2044" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78249,7 +78249,7 @@
     </row>
     <row r="2045">
       <c r="A2045" t="str">
-        <v>Kmu0wc9ruwu2e</v>
+        <v>Kmu0wctkt2ps2</v>
       </c>
       <c r="B2045" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78325,7 +78325,7 @@
     </row>
     <row r="2047">
       <c r="A2047" t="str">
-        <v>Kmu0wc9ruod1l</v>
+        <v>Kmu0wctkt2j97</v>
       </c>
       <c r="B2047" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78363,7 +78363,7 @@
     </row>
     <row r="2048">
       <c r="A2048" t="str">
-        <v>Kmu0wc9rucmzi</v>
+        <v>Kmu0wctktjx0q</v>
       </c>
       <c r="B2048" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78401,7 +78401,7 @@
     </row>
     <row r="2049">
       <c r="A2049" t="str">
-        <v>Kmu0wc9rukc1y</v>
+        <v>Kmu0wctktdeia</v>
       </c>
       <c r="B2049" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78477,7 +78477,7 @@
     </row>
     <row r="2051">
       <c r="A2051" t="str">
-        <v>Kmu0wc9rukb73</v>
+        <v>Kmu0wctkt4u01</v>
       </c>
       <c r="B2051" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78515,7 +78515,7 @@
     </row>
     <row r="2052">
       <c r="A2052" t="str">
-        <v>Kmu0wc9ru2erp</v>
+        <v>Kmu0wctkt24z2</v>
       </c>
       <c r="B2052" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78553,7 +78553,7 @@
     </row>
     <row r="2053">
       <c r="A2053" t="str">
-        <v>Kmu0wc9rumrxv</v>
+        <v>Kmu0wctktefds</v>
       </c>
       <c r="B2053" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78591,7 +78591,7 @@
     </row>
     <row r="2054">
       <c r="A2054" t="str">
-        <v>Kmu0wc9ru36sx</v>
+        <v>Kmu0wctktlvvd</v>
       </c>
       <c r="B2054" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -78629,7 +78629,7 @@
     </row>
     <row r="2055">
       <c r="A2055" t="str">
-        <v>Kmu0wc9ruh4wk</v>
+        <v>Kmu0wctkt3evn</v>
       </c>
       <c r="B2055" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -78667,7 +78667,7 @@
     </row>
     <row r="2056">
       <c r="A2056" t="str">
-        <v>Kmu0wc9ruop4g</v>
+        <v>Kmu0wctktchu2</v>
       </c>
       <c r="B2056" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -78705,7 +78705,7 @@
     </row>
     <row r="2057">
       <c r="A2057" t="str">
-        <v>Kmu0wc9rudmjf</v>
+        <v>Kmu0wctkt28g6</v>
       </c>
       <c r="B2057" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -78743,7 +78743,7 @@
     </row>
     <row r="2058">
       <c r="A2058" t="str">
-        <v>Kmu0wc9ruaog3</v>
+        <v>Kmu0wctkt2lya</v>
       </c>
       <c r="B2058" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -78857,7 +78857,7 @@
     </row>
     <row r="2061">
       <c r="A2061" t="str">
-        <v>Kmu0wc9rub1os</v>
+        <v>Kmu0wctkt1ds6</v>
       </c>
       <c r="B2061" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78895,7 +78895,7 @@
     </row>
     <row r="2062">
       <c r="A2062" t="str">
-        <v>Kmu0wc9rurhtd</v>
+        <v>Kmu0wctktemqp</v>
       </c>
       <c r="B2062" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78933,7 +78933,7 @@
     </row>
     <row r="2063">
       <c r="A2063" t="str">
-        <v>Kmu0wc9rux9oj</v>
+        <v>Kmu0wctktp0tl</v>
       </c>
       <c r="B2063" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79009,7 +79009,7 @@
     </row>
     <row r="2065">
       <c r="A2065" t="str">
-        <v>Kmu0wc9rurp6m</v>
+        <v>Kmu0wctku4zpl</v>
       </c>
       <c r="B2065" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79047,7 +79047,7 @@
     </row>
     <row r="2066">
       <c r="A2066" t="str">
-        <v>Kmu0wc9ru2ii4</v>
+        <v>Kmu0wctku9w4e</v>
       </c>
       <c r="B2066" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79085,7 +79085,7 @@
     </row>
     <row r="2067">
       <c r="A2067" t="str">
-        <v>Kmu0wc9ruc4bl</v>
+        <v>Kmu0wctkuy6ub</v>
       </c>
       <c r="B2067" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79161,7 +79161,7 @@
     </row>
     <row r="2069">
       <c r="A2069" t="str">
-        <v>Kmu0wc9rut1u3</v>
+        <v>Kmu0wctkuupme</v>
       </c>
       <c r="B2069" t="str">
         <v>Penata Layanan Operasional</v>
@@ -79199,7 +79199,7 @@
     </row>
     <row r="2070">
       <c r="A2070" t="str">
-        <v>Kmu0wc9ru3b47</v>
+        <v>Kmu0wctkuzg2e</v>
       </c>
       <c r="B2070" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79237,7 +79237,7 @@
     </row>
     <row r="2071">
       <c r="A2071" t="str">
-        <v>Kmu0wc9ru6id1</v>
+        <v>Kmu0wctkug3ir</v>
       </c>
       <c r="B2071" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79313,7 +79313,7 @@
     </row>
     <row r="2073">
       <c r="A2073" t="str">
-        <v>Kmu0wc9rurmhg</v>
+        <v>Kmu0wctku9fum</v>
       </c>
       <c r="B2073" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79351,7 +79351,7 @@
     </row>
     <row r="2074">
       <c r="A2074" t="str">
-        <v>Kmu0wc9ruwvh6</v>
+        <v>Kmu0wctku21dy</v>
       </c>
       <c r="B2074" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79389,7 +79389,7 @@
     </row>
     <row r="2075">
       <c r="A2075" t="str">
-        <v>Kmu0wc9ru1un0</v>
+        <v>Kmu0wctkug8at</v>
       </c>
       <c r="B2075" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79427,7 +79427,7 @@
     </row>
     <row r="2076">
       <c r="A2076" t="str">
-        <v>Kmu0wc9rutg9r</v>
+        <v>Kmu0wctkuhodk</v>
       </c>
       <c r="B2076" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -79465,7 +79465,7 @@
     </row>
     <row r="2077">
       <c r="A2077" t="str">
-        <v>Kmu0wc9ruohwg</v>
+        <v>Kmu0wctku1wx9</v>
       </c>
       <c r="B2077" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -79503,7 +79503,7 @@
     </row>
     <row r="2078">
       <c r="A2078" t="str">
-        <v>Kmu0wc9ruc7fx</v>
+        <v>Kmu0wctkuv59z</v>
       </c>
       <c r="B2078" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -79541,7 +79541,7 @@
     </row>
     <row r="2079">
       <c r="A2079" t="str">
-        <v>Kmu0wc9ruc4gy</v>
+        <v>Kmu0wctkugyjy</v>
       </c>
       <c r="B2079" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -79579,7 +79579,7 @@
     </row>
     <row r="2080">
       <c r="A2080" t="str">
-        <v>Kmu0wc9rud74o</v>
+        <v>Kmu0wctkumzbk</v>
       </c>
       <c r="B2080" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -79617,7 +79617,7 @@
     </row>
     <row r="2081">
       <c r="A2081" t="str">
-        <v>Kmu0wc9ruuunp</v>
+        <v>Kmu0wctkuy3qg</v>
       </c>
       <c r="B2081" t="str">
         <v>Asesor SDM Aparatur Ahli Muda</v>
@@ -79655,7 +79655,7 @@
     </row>
     <row r="2082">
       <c r="A2082" t="str">
-        <v>Kmu0wc9rum6o5</v>
+        <v>Kmu0wctkuq2sl</v>
       </c>
       <c r="B2082" t="str">
         <v>Asesor SDM Aparatur Ahli Pertama</v>
@@ -79769,7 +79769,7 @@
     </row>
     <row r="2085">
       <c r="A2085" t="str">
-        <v>Kmu0wc9rush9e</v>
+        <v>Kmu0wctkuge2k</v>
       </c>
       <c r="B2085" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79807,7 +79807,7 @@
     </row>
     <row r="2086">
       <c r="A2086" t="str">
-        <v>Kmu0wc9rux0n8</v>
+        <v>Kmu0wctkut91j</v>
       </c>
       <c r="B2086" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79845,7 +79845,7 @@
     </row>
     <row r="2087">
       <c r="A2087" t="str">
-        <v>Kmu0wc9ruxcqv</v>
+        <v>Kmu0wctkud6gp</v>
       </c>
       <c r="B2087" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79921,7 +79921,7 @@
     </row>
     <row r="2089">
       <c r="A2089" t="str">
-        <v>Kmu0wc9runxdu</v>
+        <v>Kmu0wctkurd0q</v>
       </c>
       <c r="B2089" t="str">
         <v>Penata Layanan Operasional</v>
@@ -79959,7 +79959,7 @@
     </row>
     <row r="2090">
       <c r="A2090" t="str">
-        <v>Kmu0wc9ruoo8b</v>
+        <v>Kmu0wctkurkks</v>
       </c>
       <c r="B2090" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79997,7 +79997,7 @@
     </row>
     <row r="2091">
       <c r="A2091" t="str">
-        <v>Kmu0wc9rubs9x</v>
+        <v>Kmu0wctkul5aj</v>
       </c>
       <c r="B2091" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80073,7 +80073,7 @@
     </row>
     <row r="2093">
       <c r="A2093" t="str">
-        <v>Kmu0wc9rurwkl</v>
+        <v>Kmu0wctkuq27r</v>
       </c>
       <c r="B2093" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80111,7 +80111,7 @@
     </row>
     <row r="2094">
       <c r="A2094" t="str">
-        <v>Kmu0wc9runpak</v>
+        <v>Kmu0wctkuf6eu</v>
       </c>
       <c r="B2094" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80149,7 +80149,7 @@
     </row>
     <row r="2095">
       <c r="A2095" t="str">
-        <v>Kmu0wc9ruy6vs</v>
+        <v>Kmu0wctkuqxej</v>
       </c>
       <c r="B2095" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80187,7 +80187,7 @@
     </row>
     <row r="2096">
       <c r="A2096" t="str">
-        <v>Kmu0wc9ruiljc</v>
+        <v>Kmu0wctku8uf6</v>
       </c>
       <c r="B2096" t="str">
         <v>Analis Anggaran Ahli Pertama/ Analis Keuangan Negara Ahli Pertama</v>
@@ -80225,7 +80225,7 @@
     </row>
     <row r="2097">
       <c r="A2097" t="str">
-        <v>Kmu0wc9rucclj</v>
+        <v>Kmu0wctkuidbc</v>
       </c>
       <c r="B2097" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Muda/Pengawas Keuangan Negara Ahli Muda</v>
@@ -80263,7 +80263,7 @@
     </row>
     <row r="2098">
       <c r="A2098" t="str">
-        <v>Kmu0wc9ru291j</v>
+        <v>Kmu0wctkui8e3</v>
       </c>
       <c r="B2098" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Pertama/Pengawas Keuangan Negara Ahli Pertama</v>
@@ -80301,7 +80301,7 @@
     </row>
     <row r="2099">
       <c r="A2099" t="str">
-        <v>Kmu0wc9ruqjyi</v>
+        <v>Kmu0wctkub3ef</v>
       </c>
       <c r="B2099" t="str">
         <v>Pranata Keuangan APBN Penyelia/Pengawas Keuangan Negara Penyelia</v>
@@ -80339,7 +80339,7 @@
     </row>
     <row r="2100">
       <c r="A2100" t="str">
-        <v>Kmu0wc9run9o5</v>
+        <v>Kmu0wctku6a9g</v>
       </c>
       <c r="B2100" t="str">
         <v>Pranata Keuangan APBN Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -80377,7 +80377,7 @@
     </row>
     <row r="2101">
       <c r="A2101" t="str">
-        <v>Kmu0wc9rubjuf</v>
+        <v>Kmu0wctku01ij</v>
       </c>
       <c r="B2101" t="str">
         <v>Pranata Keuangan APBN Terampil/Pengawas Keuangan Negara Terampil</v>
@@ -80415,7 +80415,7 @@
     </row>
     <row r="2102">
       <c r="A2102" t="str">
-        <v>Kmu0wc9ruvjf0</v>
+        <v>Kmu0wctkumi5r</v>
       </c>
       <c r="B2102" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -80453,7 +80453,7 @@
     </row>
     <row r="2103">
       <c r="A2103" t="str">
-        <v>Kmu0wc9rulp9r</v>
+        <v>Kmu0wctkul5hd</v>
       </c>
       <c r="B2103" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -80491,7 +80491,7 @@
     </row>
     <row r="2104">
       <c r="A2104" t="str">
-        <v>Kmu0wc9ru0do7</v>
+        <v>Kmu0wctkuo4nn</v>
       </c>
       <c r="B2104" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -80529,7 +80529,7 @@
     </row>
     <row r="2105">
       <c r="A2105" t="str">
-        <v>Kmu0wc9ru39s5</v>
+        <v>Kmu0wctku4uae</v>
       </c>
       <c r="B2105" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -80567,7 +80567,7 @@
     </row>
     <row r="2106">
       <c r="A2106" t="str">
-        <v>Kmu0wc9ru4u0k</v>
+        <v>Kmu0wctkule2d</v>
       </c>
       <c r="B2106" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -80681,7 +80681,7 @@
     </row>
     <row r="2109">
       <c r="A2109" t="str">
-        <v>Kmu0wc9rupb4c</v>
+        <v>Kmu0wctkugbli</v>
       </c>
       <c r="B2109" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80719,7 +80719,7 @@
     </row>
     <row r="2110">
       <c r="A2110" t="str">
-        <v>Kmu0wc9ruk9lg</v>
+        <v>Kmu0wctkuy5vr</v>
       </c>
       <c r="B2110" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80757,7 +80757,7 @@
     </row>
     <row r="2111">
       <c r="A2111" t="str">
-        <v>Kmu0wc9runahm</v>
+        <v>Kmu0wctkunwyg</v>
       </c>
       <c r="B2111" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80833,7 +80833,7 @@
     </row>
     <row r="2113">
       <c r="A2113" t="str">
-        <v>Kmu0wc9ruqt1d</v>
+        <v>Kmu0wctkulmko</v>
       </c>
       <c r="B2113" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80871,7 +80871,7 @@
     </row>
     <row r="2114">
       <c r="A2114" t="str">
-        <v>Kmu0wc9ru9y1a</v>
+        <v>Kmu0wctkux6q5</v>
       </c>
       <c r="B2114" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80909,7 +80909,7 @@
     </row>
     <row r="2115">
       <c r="A2115" t="str">
-        <v>Kmu0wc9ru6vz1</v>
+        <v>Kmu0wctkuyz59</v>
       </c>
       <c r="B2115" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80985,7 +80985,7 @@
     </row>
     <row r="2117">
       <c r="A2117" t="str">
-        <v>Kmu0wc9run32d</v>
+        <v>Kmu0wctku0kpn</v>
       </c>
       <c r="B2117" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -81023,7 +81023,7 @@
     </row>
     <row r="2118">
       <c r="A2118" t="str">
-        <v>Kmu0wc9ruej1a</v>
+        <v>Kmu0wctkuei6z</v>
       </c>
       <c r="B2118" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81061,7 +81061,7 @@
     </row>
     <row r="2119">
       <c r="A2119" t="str">
-        <v>Kmu0wc9ruvivi</v>
+        <v>Kmu0wctkuyeva</v>
       </c>
       <c r="B2119" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81099,7 +81099,7 @@
     </row>
     <row r="2120">
       <c r="A2120" t="str">
-        <v>Kmu0wc9rufkc7</v>
+        <v>Kmu0wctku3ztp</v>
       </c>
       <c r="B2120" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -81137,7 +81137,7 @@
     </row>
     <row r="2121">
       <c r="A2121" t="str">
-        <v>Kmu0wc9rutr7z</v>
+        <v>Kmu0wctkucnm5</v>
       </c>
       <c r="B2121" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -81175,7 +81175,7 @@
     </row>
     <row r="2122">
       <c r="A2122" t="str">
-        <v>Kmu0wc9rubeqs</v>
+        <v>Kmu0wctkuthyt</v>
       </c>
       <c r="B2122" t="str">
         <v>Pengawas Keuangan Negara Mahir</v>
@@ -81213,7 +81213,7 @@
     </row>
     <row r="2123">
       <c r="A2123" t="str">
-        <v>Kmu0wc9ruxicw</v>
+        <v>Kmu0wctku4sop</v>
       </c>
       <c r="B2123" t="str">
         <v>Pengawas Keuangan Negara Terampil</v>
@@ -81327,7 +81327,7 @@
     </row>
     <row r="2126">
       <c r="A2126" t="str">
-        <v>Kmu0wc9ruta9e</v>
+        <v>Kmu0wctkupls0</v>
       </c>
       <c r="B2126" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81365,7 +81365,7 @@
     </row>
     <row r="2127">
       <c r="A2127" t="str">
-        <v>Kmu0wc9ruuldg</v>
+        <v>Kmu0wctkuriff</v>
       </c>
       <c r="B2127" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81403,7 +81403,7 @@
     </row>
     <row r="2128">
       <c r="A2128" t="str">
-        <v>Kmu0wc9rub4xn</v>
+        <v>Kmu0wctku76nh</v>
       </c>
       <c r="B2128" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81441,7 +81441,7 @@
     </row>
     <row r="2129">
       <c r="A2129" t="str">
-        <v>Kmu0wc9rugesh</v>
+        <v>Kmu0wctkuwf04</v>
       </c>
       <c r="B2129" t="str">
         <v>Penata Keprotokolan*</v>
@@ -81517,7 +81517,7 @@
     </row>
     <row r="2131">
       <c r="A2131" t="str">
-        <v>Kmu0wc9ruk3kr</v>
+        <v>Kmu0wctkuvquq</v>
       </c>
       <c r="B2131" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81555,7 +81555,7 @@
     </row>
     <row r="2132">
       <c r="A2132" t="str">
-        <v>Kmu0wc9ruwju1</v>
+        <v>Kmu0wctkuj4f4</v>
       </c>
       <c r="B2132" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81593,7 +81593,7 @@
     </row>
     <row r="2133">
       <c r="A2133" t="str">
-        <v>Kmu0wc9ruh84t</v>
+        <v>Kmu0wctkue309</v>
       </c>
       <c r="B2133" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81631,7 +81631,7 @@
     </row>
     <row r="2134">
       <c r="A2134" t="str">
-        <v>Kmu0wc9ru8mam</v>
+        <v>Kmu0wctku10te</v>
       </c>
       <c r="B2134" t="str">
         <v>Penata Keprotokolan*</v>
@@ -81707,7 +81707,7 @@
     </row>
     <row r="2136">
       <c r="A2136" t="str">
-        <v>Kmu0wc9ru5hk3</v>
+        <v>Kmu0wctkukia5</v>
       </c>
       <c r="B2136" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81745,7 +81745,7 @@
     </row>
     <row r="2137">
       <c r="A2137" t="str">
-        <v>Kmu0wc9ruoivv</v>
+        <v>Kmu0wctku1dna</v>
       </c>
       <c r="B2137" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81783,7 +81783,7 @@
     </row>
     <row r="2138">
       <c r="A2138" t="str">
-        <v>Kmu0wc9rujql5</v>
+        <v>Kmu0wctkuhuvv</v>
       </c>
       <c r="B2138" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81821,7 +81821,7 @@
     </row>
     <row r="2139">
       <c r="A2139" t="str">
-        <v>Kmu0wc9rux86x</v>
+        <v>Kmu0wctkum4u4</v>
       </c>
       <c r="B2139" t="str">
         <v>Pengawas Keuangan Negara Ahli Muda</v>
@@ -81859,7 +81859,7 @@
     </row>
     <row r="2140">
       <c r="A2140" t="str">
-        <v>Kmu0wc9rupac2</v>
+        <v>Kmu0wctku9p12</v>
       </c>
       <c r="B2140" t="str">
         <v>Pengawas Keuangan Negara Pertama</v>
@@ -81897,7 +81897,7 @@
     </row>
     <row r="2141">
       <c r="A2141" t="str">
-        <v>Kmu0wc9rufl0v</v>
+        <v>Kmu0wctkuhk8e</v>
       </c>
       <c r="B2141" t="str">
         <v>Penata Laksana Barang Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -81935,7 +81935,7 @@
     </row>
     <row r="2142">
       <c r="A2142" t="str">
-        <v>Kmu0wc9ru6yl5</v>
+        <v>Kmu0wctkutajo</v>
       </c>
       <c r="B2142" t="str">
         <v>Penata Laksana Barang Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -81973,7 +81973,7 @@
     </row>
     <row r="2143">
       <c r="A2143" t="str">
-        <v>Kmu0wc9ru6h6t</v>
+        <v>Kmu0wctkuwj8j</v>
       </c>
       <c r="B2143" t="str">
         <v>Penata Laksana Barang Terampil/ Pengawas Keuangan Negara Terampil</v>
@@ -82011,7 +82011,7 @@
     </row>
     <row r="2144">
       <c r="A2144" t="str">
-        <v>Kmu0wc9rujgyg</v>
+        <v>Kmu0wctku3r8t</v>
       </c>
       <c r="B2144" t="str">
         <v>Arsiparis Ahli Muda</v>
@@ -82049,7 +82049,7 @@
     </row>
     <row r="2145">
       <c r="A2145" t="str">
-        <v>Kmu0wc9ru1z8y</v>
+        <v>Kmu0wctku37fx</v>
       </c>
       <c r="B2145" t="str">
         <v>Arsiparis Ahli Pertama</v>
@@ -82087,7 +82087,7 @@
     </row>
     <row r="2146">
       <c r="A2146" t="str">
-        <v>Kmu0wc9rujrfi</v>
+        <v>Kmu0wctku2z33</v>
       </c>
       <c r="B2146" t="str">
         <v>Arsiparis Penyelia</v>
@@ -82125,7 +82125,7 @@
     </row>
     <row r="2147">
       <c r="A2147" t="str">
-        <v>Kmu0wc9rui5es</v>
+        <v>Kmu0wctku6vac</v>
       </c>
       <c r="B2147" t="str">
         <v>Arsiparis Mahir</v>
@@ -82163,7 +82163,7 @@
     </row>
     <row r="2148">
       <c r="A2148" t="str">
-        <v>Kmu0wc9ruk2fd</v>
+        <v>Kmu0wctkuy4qj</v>
       </c>
       <c r="B2148" t="str">
         <v>Arsiparis Terampil</v>
@@ -82277,7 +82277,7 @@
     </row>
     <row r="2151">
       <c r="A2151" t="str">
-        <v>Kmu0wc9ru0hse</v>
+        <v>Kmu0wctku67al</v>
       </c>
       <c r="B2151" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -82315,7 +82315,7 @@
     </row>
     <row r="2152">
       <c r="A2152" t="str">
-        <v>Kmu0wc9ru2vrj</v>
+        <v>Kmu0wctkuso64</v>
       </c>
       <c r="B2152" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82353,7 +82353,7 @@
     </row>
     <row r="2153">
       <c r="A2153" t="str">
-        <v>Kmu0wc9ruxlqp</v>
+        <v>Kmu0wctkut7ae</v>
       </c>
       <c r="B2153" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82391,7 +82391,7 @@
     </row>
     <row r="2154">
       <c r="A2154" t="str">
-        <v>Kmu0wc9ruwk5t</v>
+        <v>Kmu0wctku1tdf</v>
       </c>
       <c r="B2154" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -82429,7 +82429,7 @@
     </row>
     <row r="2155">
       <c r="A2155" t="str">
-        <v>Kmu0wc9ruhjw7</v>
+        <v>Kmu0wctku2kli</v>
       </c>
       <c r="B2155" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -82467,7 +82467,7 @@
     </row>
     <row r="2156">
       <c r="A2156" t="str">
-        <v>Kmu0wc9ruwu98</v>
+        <v>Kmu0wctkuzdoe</v>
       </c>
       <c r="B2156" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -82505,7 +82505,7 @@
     </row>
     <row r="2157">
       <c r="A2157" t="str">
-        <v>Kmu0wc9ruay2u</v>
+        <v>Kmu0wctkuunbj</v>
       </c>
       <c r="B2157" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -82581,7 +82581,7 @@
     </row>
     <row r="2159">
       <c r="A2159" t="str">
-        <v>Kmu0wc9ruw0s3</v>
+        <v>Kmu0wctkuu3dj</v>
       </c>
       <c r="B2159" t="str">
         <v>Penata Layanan Operasional</v>
@@ -82619,7 +82619,7 @@
     </row>
     <row r="2160">
       <c r="A2160" t="str">
-        <v>Kmu0wc9ruszwr</v>
+        <v>Kmu0wctku67qh</v>
       </c>
       <c r="B2160" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82657,7 +82657,7 @@
     </row>
     <row r="2161">
       <c r="A2161" t="str">
-        <v>Kmu0wc9ru3ntx</v>
+        <v>Kmu0wctkufrqr</v>
       </c>
       <c r="B2161" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82695,7 +82695,7 @@
     </row>
     <row r="2162">
       <c r="A2162" t="str">
-        <v>Kmu0wc9rullsh</v>
+        <v>Kmu0wctkupczk</v>
       </c>
       <c r="B2162" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -82733,7 +82733,7 @@
     </row>
     <row r="2163">
       <c r="A2163" t="str">
-        <v>Kmu0wc9ruvc4p</v>
+        <v>Kmu0wctku1hd1</v>
       </c>
       <c r="B2163" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -82771,7 +82771,7 @@
     </row>
     <row r="2164">
       <c r="A2164" t="str">
-        <v>Kmu0wc9rue7vo</v>
+        <v>Kmu0wctku1ruu</v>
       </c>
       <c r="B2164" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -82809,7 +82809,7 @@
     </row>
     <row r="2165">
       <c r="A2165" t="str">
-        <v>Kmu0wc9rua65j</v>
+        <v>Kmu0wctkud9je</v>
       </c>
       <c r="B2165" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -82885,7 +82885,7 @@
     </row>
     <row r="2167">
       <c r="A2167" t="str">
-        <v>Kmu0wc9ru7co1</v>
+        <v>Kmu0wctkuax5b</v>
       </c>
       <c r="B2167" t="str">
         <v>Penata Layanan Operasional</v>
@@ -82923,7 +82923,7 @@
     </row>
     <row r="2168">
       <c r="A2168" t="str">
-        <v>Kmu0wc9rulfm3</v>
+        <v>Kmu0wctkunfgp</v>
       </c>
       <c r="B2168" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82961,7 +82961,7 @@
     </row>
     <row r="2169">
       <c r="A2169" t="str">
-        <v>Kmu0wc9rusa9q</v>
+        <v>Kmu0wctkux6y3</v>
       </c>
       <c r="B2169" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82999,7 +82999,7 @@
     </row>
     <row r="2170">
       <c r="A2170" t="str">
-        <v>Kmu0wc9ruql77</v>
+        <v>Kmu0wctku9r79</v>
       </c>
       <c r="B2170" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -83037,7 +83037,7 @@
     </row>
     <row r="2171">
       <c r="A2171" t="str">
-        <v>Kmu0wc9ruhyq3</v>
+        <v>Kmu0wctkui3g1</v>
       </c>
       <c r="B2171" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -83075,7 +83075,7 @@
     </row>
     <row r="2172">
       <c r="A2172" t="str">
-        <v>Kmu0wc9ru4r7f</v>
+        <v>Kmu0wctkuddzq</v>
       </c>
       <c r="B2172" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -83113,7 +83113,7 @@
     </row>
     <row r="2173">
       <c r="A2173" t="str">
-        <v>Kmu0wc9rux1u2</v>
+        <v>Kmu0wctkuy7ed</v>
       </c>
       <c r="B2173" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -83151,7 +83151,7 @@
     </row>
     <row r="2174">
       <c r="A2174" t="str">
-        <v>Kmu0wc9ru73d3</v>
+        <v>Kmu0wctkujpn2</v>
       </c>
       <c r="B2174" t="str">
         <v>Pranata Humas Ahli Muda</v>
@@ -83189,7 +83189,7 @@
     </row>
     <row r="2175">
       <c r="A2175" t="str">
-        <v>Kmu0wc9ruv2gf</v>
+        <v>Kmu0wctkub8r6</v>
       </c>
       <c r="B2175" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -83227,7 +83227,7 @@
     </row>
     <row r="2176">
       <c r="A2176" t="str">
-        <v>Kmu0wc9rucj6l</v>
+        <v>Kmu0wctku9j39</v>
       </c>
       <c r="B2176" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -83265,7 +83265,7 @@
     </row>
     <row r="2177">
       <c r="A2177" t="str">
-        <v>Kmu0wc9ruapk4</v>
+        <v>Kmu0wctkuy1xq</v>
       </c>
       <c r="B2177" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -83303,7 +83303,7 @@
     </row>
     <row r="2178">
       <c r="A2178" t="str">
-        <v>Kmu0wc9ruhg37</v>
+        <v>Kmu0wctku21jk</v>
       </c>
       <c r="B2178" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -83341,7 +83341,7 @@
     </row>
     <row r="2179">
       <c r="A2179" t="str">
-        <v>Kmu0wc9ru6w84</v>
+        <v>Kmu0wctku7wan</v>
       </c>
       <c r="B2179" t="str">
         <v>Pustakawan Ahli Pertama</v>
@@ -83379,7 +83379,7 @@
     </row>
     <row r="2180">
       <c r="A2180" t="str">
-        <v>Kmu0wc9rujt7h</v>
+        <v>Kmu0wctku3vlk</v>
       </c>
       <c r="B2180" t="str">
         <v>Asisten Perpustakaan Penyelia</v>
@@ -83417,7 +83417,7 @@
     </row>
     <row r="2181">
       <c r="A2181" t="str">
-        <v>Kmu0wc9ru4ati</v>
+        <v>Kmu0wctkuif27</v>
       </c>
       <c r="B2181" t="str">
         <v>Asisten Perpustakaan Mahir</v>
@@ -83455,7 +83455,7 @@
     </row>
     <row r="2182">
       <c r="A2182" t="str">
-        <v>Kmu0wc9ruvw2x</v>
+        <v>Kmu0wctkude8a</v>
       </c>
       <c r="B2182" t="str">
         <v>Asisten Perpustakaan Terampil</v>
@@ -83493,7 +83493,7 @@
     </row>
     <row r="2183">
       <c r="A2183" t="str">
-        <v>Kmu0wc9rusees</v>
+        <v>Kmu0wctkuoii3</v>
       </c>
       <c r="B2183" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Madya/Pengawas Keuangan Negara Ahli Madya</v>
@@ -83531,7 +83531,7 @@
     </row>
     <row r="2184">
       <c r="A2184" t="str">
-        <v>Kmu0wc9ruq480</v>
+        <v>Kmu0wctku4p9p</v>
       </c>
       <c r="B2184" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Muda</v>
@@ -83569,7 +83569,7 @@
     </row>
     <row r="2185">
       <c r="A2185" t="str">
-        <v>Kmu0wc9ruo539</v>
+        <v>Kmu0wctkus6p7</v>
       </c>
       <c r="B2185" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Pertama</v>
@@ -83683,7 +83683,7 @@
     </row>
     <row r="2188">
       <c r="A2188" t="str">
-        <v>Kmu0wc9rupbu9</v>
+        <v>Kmu0wctkuokeg</v>
       </c>
       <c r="B2188" t="str">
         <v>Penata Layanan Operasional</v>
@@ -83721,7 +83721,7 @@
     </row>
     <row r="2189">
       <c r="A2189" t="str">
-        <v>Kmu0wc9ru4yf6</v>
+        <v>Kmu0wctkunfqg</v>
       </c>
       <c r="B2189" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -83759,7 +83759,7 @@
     </row>
     <row r="2190">
       <c r="A2190" t="str">
-        <v>Kmu0wc9ruzhbh</v>
+        <v>Kmu0wctkujhme</v>
       </c>
       <c r="B2190" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -83797,7 +83797,7 @@
     </row>
     <row r="2191">
       <c r="A2191" t="str">
-        <v>Kmu0wc9ruqhnl</v>
+        <v>Kmu0wctkua43g</v>
       </c>
       <c r="B2191" t="str">
         <v>Penata Keprotokolan*</v>
@@ -83911,7 +83911,7 @@
     </row>
     <row r="2194">
       <c r="A2194" t="str">
-        <v>Kmu0wc9ru5uf6</v>
+        <v>Kmu0wctku8dwh</v>
       </c>
       <c r="B2194" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -83949,7 +83949,7 @@
     </row>
     <row r="2195">
       <c r="A2195" t="str">
-        <v>Kmu0wc9rufx21</v>
+        <v>Kmu0wctku6lkm</v>
       </c>
       <c r="B2195" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -83987,7 +83987,7 @@
     </row>
     <row r="2196">
       <c r="A2196" t="str">
-        <v>Kmu0wc9rugbpu</v>
+        <v>Kmu0wctkubd8x</v>
       </c>
       <c r="B2196" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84063,7 +84063,7 @@
     </row>
     <row r="2198">
       <c r="A2198" t="str">
-        <v>Kmu0wc9ru78oz</v>
+        <v>Kmu0wctkufk8q</v>
       </c>
       <c r="B2198" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84101,7 +84101,7 @@
     </row>
     <row r="2199">
       <c r="A2199" t="str">
-        <v>Kmu0wc9ruii9t</v>
+        <v>Kmu0wctkuyjde</v>
       </c>
       <c r="B2199" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84139,7 +84139,7 @@
     </row>
     <row r="2200">
       <c r="A2200" t="str">
-        <v>Kmu0wc9ru6e2j</v>
+        <v>Kmu0wctku4zun</v>
       </c>
       <c r="B2200" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84177,7 +84177,7 @@
     </row>
     <row r="2201">
       <c r="A2201" t="str">
-        <v>Kmu0wc9ru1zwr</v>
+        <v>Kmu0wctku1w08</v>
       </c>
       <c r="B2201" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -84215,7 +84215,7 @@
     </row>
     <row r="2202">
       <c r="A2202" t="str">
-        <v>Kmu0wc9rukf2l</v>
+        <v>Kmu0wctkubqeu</v>
       </c>
       <c r="B2202" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -84253,7 +84253,7 @@
     </row>
     <row r="2203">
       <c r="A2203" t="str">
-        <v>Kmu0wc9ruf7p4</v>
+        <v>Kmu0wctkupuna</v>
       </c>
       <c r="B2203" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -84291,7 +84291,7 @@
     </row>
     <row r="2204">
       <c r="A2204" t="str">
-        <v>Kmu0wc9ruwwjv</v>
+        <v>Kmu0wctku8woi</v>
       </c>
       <c r="B2204" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -84405,7 +84405,7 @@
     </row>
     <row r="2207">
       <c r="A2207" t="str">
-        <v>Kmu0wc9ruj4my</v>
+        <v>Kmu0wctkurw1l</v>
       </c>
       <c r="B2207" t="str">
         <v>Penata Layanan Operasional</v>
@@ -84443,7 +84443,7 @@
     </row>
     <row r="2208">
       <c r="A2208" t="str">
-        <v>Kmu0wc9rutwo3</v>
+        <v>Kmu0wctkuhyt7</v>
       </c>
       <c r="B2208" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84481,7 +84481,7 @@
     </row>
     <row r="2209">
       <c r="A2209" t="str">
-        <v>Kmu0wc9run1p7</v>
+        <v>Kmu0wctkutday</v>
       </c>
       <c r="B2209" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84519,7 +84519,7 @@
     </row>
     <row r="2210">
       <c r="A2210" t="str">
-        <v>Kmu0wc9run2i1</v>
+        <v>Kmu0wctku5q5v</v>
       </c>
       <c r="B2210" t="str">
         <v>Penata Keprotokolan*</v>
@@ -84633,7 +84633,7 @@
     </row>
     <row r="2213">
       <c r="A2213" t="str">
-        <v>Kmu0wc9ruo11r</v>
+        <v>Kmu0wctkumtls</v>
       </c>
       <c r="B2213" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84671,7 +84671,7 @@
     </row>
     <row r="2214">
       <c r="A2214" t="str">
-        <v>Kmu0wc9ru9cwp</v>
+        <v>Kmu0wctku9ar8</v>
       </c>
       <c r="B2214" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84709,7 +84709,7 @@
     </row>
     <row r="2215">
       <c r="A2215" t="str">
-        <v>Kmu0wc9ruf0fx</v>
+        <v>Kmu0wctkuawow</v>
       </c>
       <c r="B2215" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84785,7 +84785,7 @@
     </row>
     <row r="2217">
       <c r="A2217" t="str">
-        <v>Kmu0wc9rups46</v>
+        <v>Kmu0wctku9wuz</v>
       </c>
       <c r="B2217" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84823,7 +84823,7 @@
     </row>
     <row r="2218">
       <c r="A2218" t="str">
-        <v>Kmu0wc9rui35c</v>
+        <v>Kmu0wctkui55s</v>
       </c>
       <c r="B2218" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84861,7 +84861,7 @@
     </row>
     <row r="2219">
       <c r="A2219" t="str">
-        <v>Kmu0wc9rupgnl</v>
+        <v>Kmu0wctkuyp1e</v>
       </c>
       <c r="B2219" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84899,7 +84899,7 @@
     </row>
     <row r="2220">
       <c r="A2220" t="str">
-        <v>Kmu0wc9rumvz6</v>
+        <v>Kmu0wctkuwd9z</v>
       </c>
       <c r="B2220" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -84937,7 +84937,7 @@
     </row>
     <row r="2221">
       <c r="A2221" t="str">
-        <v>Kmu0wc9ru4qtd</v>
+        <v>Kmu0wctku2xci</v>
       </c>
       <c r="B2221" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -84975,7 +84975,7 @@
     </row>
     <row r="2222">
       <c r="A2222" t="str">
-        <v>Kmu0wc9ru8hw2</v>
+        <v>Kmu0wctkuehsv</v>
       </c>
       <c r="B2222" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -85013,7 +85013,7 @@
     </row>
     <row r="2223">
       <c r="A2223" t="str">
-        <v>Kmu0wc9rujea9</v>
+        <v>Kmu0wctkuygov</v>
       </c>
       <c r="B2223" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -85127,7 +85127,7 @@
     </row>
     <row r="2226">
       <c r="A2226" t="str">
-        <v>Kmu0wc9ruere6</v>
+        <v>Kmu0wctkuv1uf</v>
       </c>
       <c r="B2226" t="str">
         <v>Penata Layanan Operasional</v>
@@ -85165,7 +85165,7 @@
     </row>
     <row r="2227">
       <c r="A2227" t="str">
-        <v>Kmu0wc9rusb13</v>
+        <v>Kmu0wctkuu6th</v>
       </c>
       <c r="B2227" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85203,7 +85203,7 @@
     </row>
     <row r="2228">
       <c r="A2228" t="str">
-        <v>Kmu0wc9rusa7k</v>
+        <v>Kmu0wctkuri7g</v>
       </c>
       <c r="B2228" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85241,7 +85241,7 @@
     </row>
     <row r="2229">
       <c r="A2229" t="str">
-        <v>Kmu0wc9rufx5e</v>
+        <v>Kmu0wctkumc44</v>
       </c>
       <c r="B2229" t="str">
         <v>Penata Keprotokolan*</v>
@@ -85355,7 +85355,7 @@
     </row>
     <row r="2232">
       <c r="A2232" t="str">
-        <v>Kmu0wc9ruow77</v>
+        <v>Kmu0wctku39a9</v>
       </c>
       <c r="B2232" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -85393,7 +85393,7 @@
     </row>
     <row r="2233">
       <c r="A2233" t="str">
-        <v>Kmu0wc9ru6l55</v>
+        <v>Kmu0wctku2hdj</v>
       </c>
       <c r="B2233" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85431,7 +85431,7 @@
     </row>
     <row r="2234">
       <c r="A2234" t="str">
-        <v>Kmu0wc9ruvgmk</v>
+        <v>Kmu0wctku4pyc</v>
       </c>
       <c r="B2234" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85507,7 +85507,7 @@
     </row>
     <row r="2236">
       <c r="A2236" t="str">
-        <v>Kmu0wc9ruahgo</v>
+        <v>Kmu0wctkuwfii</v>
       </c>
       <c r="B2236" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -85545,7 +85545,7 @@
     </row>
     <row r="2237">
       <c r="A2237" t="str">
-        <v>Kmu0wc9rulrcd</v>
+        <v>Kmu0wctkuzu64</v>
       </c>
       <c r="B2237" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85583,7 +85583,7 @@
     </row>
     <row r="2238">
       <c r="A2238" t="str">
-        <v>Kmu0wc9rupjts</v>
+        <v>Kmu0wctkuxbgm</v>
       </c>
       <c r="B2238" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85621,7 +85621,7 @@
     </row>
     <row r="2239">
       <c r="A2239" t="str">
-        <v>Kmu0wc9ruf6jj</v>
+        <v>Kmu0wctku2xeo</v>
       </c>
       <c r="B2239" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -85659,7 +85659,7 @@
     </row>
     <row r="2240">
       <c r="A2240" t="str">
-        <v>Kmu0wc9ru4ujt</v>
+        <v>Kmu0wctku2d5o</v>
       </c>
       <c r="B2240" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -85697,7 +85697,7 @@
     </row>
     <row r="2241">
       <c r="A2241" t="str">
-        <v>Kmu0wc9ruyp6k</v>
+        <v>Kmu0wctkujki4</v>
       </c>
       <c r="B2241" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -85735,7 +85735,7 @@
     </row>
     <row r="2242">
       <c r="A2242" t="str">
-        <v>Kmu0wc9ruvixx</v>
+        <v>Kmu0wctkumiq9</v>
       </c>
       <c r="B2242" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -85849,7 +85849,7 @@
     </row>
     <row r="2245">
       <c r="A2245" t="str">
-        <v>Kmu0wc9ru9yow</v>
+        <v>Kmu0wctkuvqm3</v>
       </c>
       <c r="B2245" t="str">
         <v>Penata Layanan Operasional</v>
@@ -85887,7 +85887,7 @@
     </row>
     <row r="2246">
       <c r="A2246" t="str">
-        <v>Kmu0wc9ru0osn</v>
+        <v>Kmu0wctkuod1p</v>
       </c>
       <c r="B2246" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85925,7 +85925,7 @@
     </row>
     <row r="2247">
       <c r="A2247" t="str">
-        <v>Kmu0wc9ruy20a</v>
+        <v>Kmu0wctkuhohp</v>
       </c>
       <c r="B2247" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85963,7 +85963,7 @@
     </row>
     <row r="2248">
       <c r="A2248" t="str">
-        <v>Kmu0wc9runcdt</v>
+        <v>Kmu0wctku1m46</v>
       </c>
       <c r="B2248" t="str">
         <v>Penata Keprotokolan*</v>
@@ -86039,7 +86039,7 @@
     </row>
     <row r="2250">
       <c r="A2250" t="str">
-        <v>Kmu0wc9ruc30w</v>
+        <v>Kmu0wctkud5om</v>
       </c>
       <c r="B2250" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86077,7 +86077,7 @@
     </row>
     <row r="2251">
       <c r="A2251" t="str">
-        <v>Kmu0wc9ruqdu8</v>
+        <v>Kmu0wctkumyph</v>
       </c>
       <c r="B2251" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86115,7 +86115,7 @@
     </row>
     <row r="2252">
       <c r="A2252" t="str">
-        <v>Kmu0wc9ru29tq</v>
+        <v>Kmu0wctku0dj3</v>
       </c>
       <c r="B2252" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86153,7 +86153,7 @@
     </row>
     <row r="2253">
       <c r="A2253" t="str">
-        <v>Kmu0wc9rush4e</v>
+        <v>Kmu0wctkuvgxi</v>
       </c>
       <c r="B2253" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -86191,7 +86191,7 @@
     </row>
     <row r="2254">
       <c r="A2254" t="str">
-        <v>Kmu0wc9ru8lbq</v>
+        <v>Kmu0wctkuauj0</v>
       </c>
       <c r="B2254" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -86305,7 +86305,7 @@
     </row>
     <row r="2257">
       <c r="A2257" t="str">
-        <v>Kmu0wc9ru3xek</v>
+        <v>Kmu0wctkulczd</v>
       </c>
       <c r="B2257" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86343,7 +86343,7 @@
     </row>
     <row r="2258">
       <c r="A2258" t="str">
-        <v>Kmu0wc9ruv3mz</v>
+        <v>Kmu0wctkuvi2w</v>
       </c>
       <c r="B2258" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86381,7 +86381,7 @@
     </row>
     <row r="2259">
       <c r="A2259" t="str">
-        <v>Kmu0wc9ruhttv</v>
+        <v>Kmu0wctkuwlrt</v>
       </c>
       <c r="B2259" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86457,7 +86457,7 @@
     </row>
     <row r="2261">
       <c r="A2261" t="str">
-        <v>Kmu0wc9rug5yk</v>
+        <v>Kmu0wctkudqkv</v>
       </c>
       <c r="B2261" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86495,7 +86495,7 @@
     </row>
     <row r="2262">
       <c r="A2262" t="str">
-        <v>Kmu0wc9ruo8m4</v>
+        <v>Kmu0wctkuj6gq</v>
       </c>
       <c r="B2262" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86533,7 +86533,7 @@
     </row>
     <row r="2263">
       <c r="A2263" t="str">
-        <v>Kmu0wc9rug4zc</v>
+        <v>Kmu0wctkujq4l</v>
       </c>
       <c r="B2263" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86571,7 +86571,7 @@
     </row>
     <row r="2264">
       <c r="A2264" t="str">
-        <v>Kmu0wc9ru2z7b</v>
+        <v>Kmu0wctku7ws6</v>
       </c>
       <c r="B2264" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -86609,7 +86609,7 @@
     </row>
     <row r="2265">
       <c r="A2265" t="str">
-        <v>Kmu0wc9ru04o2</v>
+        <v>Kmu0wctkuxc05</v>
       </c>
       <c r="B2265" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -86647,7 +86647,7 @@
     </row>
     <row r="2266">
       <c r="A2266" t="str">
-        <v>Kmu0wc9ruyjdp</v>
+        <v>Kmu0wctkuotuj</v>
       </c>
       <c r="B2266" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -86685,7 +86685,7 @@
     </row>
     <row r="2267">
       <c r="A2267" t="str">
-        <v>Kmu0wc9ruxl08</v>
+        <v>Kmu0wctkuj9wg</v>
       </c>
       <c r="B2267" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -86799,7 +86799,7 @@
     </row>
     <row r="2270">
       <c r="A2270" t="str">
-        <v>Kmu0wc9ru9xzh</v>
+        <v>Kmu0wctkunle7</v>
       </c>
       <c r="B2270" t="str">
         <v>Penata Layanan Operasional</v>
@@ -86837,7 +86837,7 @@
     </row>
     <row r="2271">
       <c r="A2271" t="str">
-        <v>Kmu0wc9ruo0tq</v>
+        <v>Kmu0wctku3yop</v>
       </c>
       <c r="B2271" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86875,7 +86875,7 @@
     </row>
     <row r="2272">
       <c r="A2272" t="str">
-        <v>Kmu0wc9ruz7ff</v>
+        <v>Kmu0wctku6cy3</v>
       </c>
       <c r="B2272" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86913,7 +86913,7 @@
     </row>
     <row r="2273">
       <c r="A2273" t="str">
-        <v>Kmu0wc9rum4zb</v>
+        <v>Kmu0wctku82u4</v>
       </c>
       <c r="B2273" t="str">
         <v>Penata Keprotokolan*</v>
@@ -87027,7 +87027,7 @@
     </row>
     <row r="2276">
       <c r="A2276" t="str">
-        <v>Kmu0wc9rusvra</v>
+        <v>Kmu0wctkud2io</v>
       </c>
       <c r="B2276" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87065,7 +87065,7 @@
     </row>
     <row r="2277">
       <c r="A2277" t="str">
-        <v>Kmu0wc9rugiqr</v>
+        <v>Kmu0wctku8on3</v>
       </c>
       <c r="B2277" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87103,7 +87103,7 @@
     </row>
     <row r="2278">
       <c r="A2278" t="str">
-        <v>Kmu0wc9rusnti</v>
+        <v>Kmu0wctkuwwu8</v>
       </c>
       <c r="B2278" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87179,7 +87179,7 @@
     </row>
     <row r="2280">
       <c r="A2280" t="str">
-        <v>Kmu0wc9ruhiq3</v>
+        <v>Kmu0wctkuo10m</v>
       </c>
       <c r="B2280" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87217,7 +87217,7 @@
     </row>
     <row r="2281">
       <c r="A2281" t="str">
-        <v>Kmu0wc9rugmn0</v>
+        <v>Kmu0wctku0zdl</v>
       </c>
       <c r="B2281" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87255,7 +87255,7 @@
     </row>
     <row r="2282">
       <c r="A2282" t="str">
-        <v>Kmu0wc9ruel36</v>
+        <v>Kmu0wctkul1aw</v>
       </c>
       <c r="B2282" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87293,7 +87293,7 @@
     </row>
     <row r="2283">
       <c r="A2283" t="str">
-        <v>Kmu0wc9rujxf2</v>
+        <v>Kmu0wctkuyx54</v>
       </c>
       <c r="B2283" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -87331,7 +87331,7 @@
     </row>
     <row r="2284">
       <c r="A2284" t="str">
-        <v>Kmu0wc9ru8png</v>
+        <v>Kmu0wctkubfo1</v>
       </c>
       <c r="B2284" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -87369,7 +87369,7 @@
     </row>
     <row r="2285">
       <c r="A2285" t="str">
-        <v>Kmu0wc9ru1k2m</v>
+        <v>Kmu0wctkucbca</v>
       </c>
       <c r="B2285" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -87407,7 +87407,7 @@
     </row>
     <row r="2286">
       <c r="A2286" t="str">
-        <v>Kmu0wc9ru53hm</v>
+        <v>Kmu0wctkulx35</v>
       </c>
       <c r="B2286" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -87521,7 +87521,7 @@
     </row>
     <row r="2289">
       <c r="A2289" t="str">
-        <v>Kmu0wc9ruzutl</v>
+        <v>Kmu0wctkub86l</v>
       </c>
       <c r="B2289" t="str">
         <v>Penata Layanan Operasional</v>
@@ -87559,7 +87559,7 @@
     </row>
     <row r="2290">
       <c r="A2290" t="str">
-        <v>Kmu0wc9ruk3m8</v>
+        <v>Kmu0wctku19wo</v>
       </c>
       <c r="B2290" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87597,7 +87597,7 @@
     </row>
     <row r="2291">
       <c r="A2291" t="str">
-        <v>Kmu0wc9ru6bst</v>
+        <v>Kmu0wctku8q8w</v>
       </c>
       <c r="B2291" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87635,7 +87635,7 @@
     </row>
     <row r="2292">
       <c r="A2292" t="str">
-        <v>Kmu0wc9ru19pi</v>
+        <v>Kmu0wctkurmmr</v>
       </c>
       <c r="B2292" t="str">
         <v>Penata Keprotokolan*</v>
@@ -87749,7 +87749,7 @@
     </row>
     <row r="2295">
       <c r="A2295" t="str">
-        <v>Kmu0wc9ru567z</v>
+        <v>Kmu0wctkud0e9</v>
       </c>
       <c r="B2295" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87787,7 +87787,7 @@
     </row>
     <row r="2296">
       <c r="A2296" t="str">
-        <v>Kmu0wc9ruas84</v>
+        <v>Kmu0wctkuus5n</v>
       </c>
       <c r="B2296" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87825,7 +87825,7 @@
     </row>
     <row r="2297">
       <c r="A2297" t="str">
-        <v>Kmu0wc9ruzs0r</v>
+        <v>Kmu0wctkuqkwt</v>
       </c>
       <c r="B2297" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87901,7 +87901,7 @@
     </row>
     <row r="2299">
       <c r="A2299" t="str">
-        <v>Kmu0wc9ruc6d3</v>
+        <v>Kmu0wctku9vxj</v>
       </c>
       <c r="B2299" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87939,7 +87939,7 @@
     </row>
     <row r="2300">
       <c r="A2300" t="str">
-        <v>Kmu0wc9rugov1</v>
+        <v>Kmu0wctkulzjb</v>
       </c>
       <c r="B2300" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87977,7 +87977,7 @@
     </row>
     <row r="2301">
       <c r="A2301" t="str">
-        <v>Kmu0wc9ruvncp</v>
+        <v>Kmu0wctkuvqtr</v>
       </c>
       <c r="B2301" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88015,7 +88015,7 @@
     </row>
     <row r="2302">
       <c r="A2302" t="str">
-        <v>Kmu0wc9ru7fbe</v>
+        <v>Kmu0wctku3gcl</v>
       </c>
       <c r="B2302" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -88053,7 +88053,7 @@
     </row>
     <row r="2303">
       <c r="A2303" t="str">
-        <v>Kmu0wc9ru83gg</v>
+        <v>Kmu0wctkundc7</v>
       </c>
       <c r="B2303" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -88091,7 +88091,7 @@
     </row>
     <row r="2304">
       <c r="A2304" t="str">
-        <v>Kmu0wc9ru9i3z</v>
+        <v>Kmu0wctkuizdq</v>
       </c>
       <c r="B2304" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -88129,7 +88129,7 @@
     </row>
     <row r="2305">
       <c r="A2305" t="str">
-        <v>Kmu0wc9ruz08i</v>
+        <v>Kmu0wctkumg01</v>
       </c>
       <c r="B2305" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -88243,7 +88243,7 @@
     </row>
     <row r="2308">
       <c r="A2308" t="str">
-        <v>Kmu0wc9ru1ymb</v>
+        <v>Kmu0wctkuijm6</v>
       </c>
       <c r="B2308" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88281,7 +88281,7 @@
     </row>
     <row r="2309">
       <c r="A2309" t="str">
-        <v>Kmu0wc9ruz3yd</v>
+        <v>Kmu0wctkuopkn</v>
       </c>
       <c r="B2309" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88319,7 +88319,7 @@
     </row>
     <row r="2310">
       <c r="A2310" t="str">
-        <v>Kmu0wc9ru06mh</v>
+        <v>Kmu0wctkuebmt</v>
       </c>
       <c r="B2310" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88357,7 +88357,7 @@
     </row>
     <row r="2311">
       <c r="A2311" t="str">
-        <v>Kmu0wc9rue1gm</v>
+        <v>Kmu0wctkufbkj</v>
       </c>
       <c r="B2311" t="str">
         <v>Penata Keprotokolan*</v>
@@ -88471,7 +88471,7 @@
     </row>
     <row r="2314">
       <c r="A2314" t="str">
-        <v>Kmu0wc9ru0ydd</v>
+        <v>Kmu0wctku3j7z</v>
       </c>
       <c r="B2314" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88509,7 +88509,7 @@
     </row>
     <row r="2315">
       <c r="A2315" t="str">
-        <v>Kmu0wc9ruvr3s</v>
+        <v>Kmu0wctkubdov</v>
       </c>
       <c r="B2315" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88547,7 +88547,7 @@
     </row>
     <row r="2316">
       <c r="A2316" t="str">
-        <v>Kmu0wc9ru2app</v>
+        <v>Kmu0wctku6deh</v>
       </c>
       <c r="B2316" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88623,7 +88623,7 @@
     </row>
     <row r="2318">
       <c r="A2318" t="str">
-        <v>Kmu0wc9ruhl6w</v>
+        <v>Kmu0wctkujv30</v>
       </c>
       <c r="B2318" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88661,7 +88661,7 @@
     </row>
     <row r="2319">
       <c r="A2319" t="str">
-        <v>Kmu0wc9ruzmnx</v>
+        <v>Kmu0wctkuxm86</v>
       </c>
       <c r="B2319" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88699,7 +88699,7 @@
     </row>
     <row r="2320">
       <c r="A2320" t="str">
-        <v>Kmu0wc9ru5m29</v>
+        <v>Kmu0wctkuc8l2</v>
       </c>
       <c r="B2320" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88775,7 +88775,7 @@
     </row>
     <row r="2322">
       <c r="A2322" t="str">
-        <v>Kmu0wc9rukmke</v>
+        <v>Kmu0wctkuov3c</v>
       </c>
       <c r="B2322" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88813,7 +88813,7 @@
     </row>
     <row r="2323">
       <c r="A2323" t="str">
-        <v>Kmu0wc9ru9yfs</v>
+        <v>Kmu0wctkuzuqh</v>
       </c>
       <c r="B2323" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88851,7 +88851,7 @@
     </row>
     <row r="2324">
       <c r="A2324" t="str">
-        <v>Kmu0wc9ru3jd3</v>
+        <v>Kmu0wctkux5zm</v>
       </c>
       <c r="B2324" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88927,7 +88927,7 @@
     </row>
     <row r="2326">
       <c r="A2326" t="str">
-        <v>Kmu0wc9ru7ztu</v>
+        <v>Kmu0wctku3uhs</v>
       </c>
       <c r="B2326" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88965,7 +88965,7 @@
     </row>
     <row r="2327">
       <c r="A2327" t="str">
-        <v>Kmu0wc9ruas67</v>
+        <v>Kmu0wctku1tqi</v>
       </c>
       <c r="B2327" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89003,7 +89003,7 @@
     </row>
     <row r="2328">
       <c r="A2328" t="str">
-        <v>Kmu0wc9ruodbz</v>
+        <v>Kmu0wctkujjxb</v>
       </c>
       <c r="B2328" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89117,7 +89117,7 @@
     </row>
     <row r="2331">
       <c r="A2331" t="str">
-        <v>Kmu0wc9runpra</v>
+        <v>Kmu0wctkuzvvi</v>
       </c>
       <c r="B2331" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89155,7 +89155,7 @@
     </row>
     <row r="2332">
       <c r="A2332" t="str">
-        <v>Kmu0wc9rubopm</v>
+        <v>Kmu0wctku9wo5</v>
       </c>
       <c r="B2332" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89193,7 +89193,7 @@
     </row>
     <row r="2333">
       <c r="A2333" t="str">
-        <v>Kmu0wc9ruduc5</v>
+        <v>Kmu0wctkulcis</v>
       </c>
       <c r="B2333" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89269,7 +89269,7 @@
     </row>
     <row r="2335">
       <c r="A2335" t="str">
-        <v>Kmu0wc9rubb7m</v>
+        <v>Kmu0wctkux7qi</v>
       </c>
       <c r="B2335" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89307,7 +89307,7 @@
     </row>
     <row r="2336">
       <c r="A2336" t="str">
-        <v>Kmu0wc9rudmad</v>
+        <v>Kmu0wctkus0b9</v>
       </c>
       <c r="B2336" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89345,7 +89345,7 @@
     </row>
     <row r="2337">
       <c r="A2337" t="str">
-        <v>Kmu0wc9ruto33</v>
+        <v>Kmu0wctku9jv2</v>
       </c>
       <c r="B2337" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89383,7 +89383,7 @@
     </row>
     <row r="2338">
       <c r="A2338" t="str">
-        <v>Kmu0wc9run813</v>
+        <v>Kmu0wctkupx75</v>
       </c>
       <c r="B2338" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -89421,7 +89421,7 @@
     </row>
     <row r="2339">
       <c r="A2339" t="str">
-        <v>Kmu0wc9runcrh</v>
+        <v>Kmu0wctkunnk2</v>
       </c>
       <c r="B2339" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -89459,7 +89459,7 @@
     </row>
     <row r="2340">
       <c r="A2340" t="str">
-        <v>Kmu0wc9rutqd1</v>
+        <v>Kmu0wctkurjcd</v>
       </c>
       <c r="B2340" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -89497,7 +89497,7 @@
     </row>
     <row r="2341">
       <c r="A2341" t="str">
-        <v>Kmu0wc9rurqp0</v>
+        <v>Kmu0wctku5lbw</v>
       </c>
       <c r="B2341" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -89611,7 +89611,7 @@
     </row>
     <row r="2344">
       <c r="A2344" t="str">
-        <v>Kmu0wc9rulrbc</v>
+        <v>Kmu0wctkulrg3</v>
       </c>
       <c r="B2344" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89649,7 +89649,7 @@
     </row>
     <row r="2345">
       <c r="A2345" t="str">
-        <v>Kmu0wc9ruu1zb</v>
+        <v>Kmu0wctkuhg42</v>
       </c>
       <c r="B2345" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89687,7 +89687,7 @@
     </row>
     <row r="2346">
       <c r="A2346" t="str">
-        <v>Kmu0wc9ruv7tm</v>
+        <v>Kmu0wctkuusiq</v>
       </c>
       <c r="B2346" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89801,7 +89801,7 @@
     </row>
     <row r="2349">
       <c r="A2349" t="str">
-        <v>Kmu0wc9ru8lbh</v>
+        <v>Kmu0wctku252l</v>
       </c>
       <c r="B2349" t="str">
         <v>Penata Layanan Operasional</v>
@@ -89839,7 +89839,7 @@
     </row>
     <row r="2350">
       <c r="A2350" t="str">
-        <v>Kmu0wc9rui8f0</v>
+        <v>Kmu0wctku465d</v>
       </c>
       <c r="B2350" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89877,7 +89877,7 @@
     </row>
     <row r="2351">
       <c r="A2351" t="str">
-        <v>Kmu0wc9ru4wym</v>
+        <v>Kmu0wctkux2i6</v>
       </c>
       <c r="B2351" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89953,7 +89953,7 @@
     </row>
     <row r="2353">
       <c r="A2353" t="str">
-        <v>Kmu0wc9ru8yyu</v>
+        <v>Kmu0wctku6cwe</v>
       </c>
       <c r="B2353" t="str">
         <v>Penata Layanan Operasional</v>
@@ -89991,7 +89991,7 @@
     </row>
     <row r="2354">
       <c r="A2354" t="str">
-        <v>Kmu0wc9ruk8ps</v>
+        <v>Kmu0wctku8iax</v>
       </c>
       <c r="B2354" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90029,7 +90029,7 @@
     </row>
     <row r="2355">
       <c r="A2355" t="str">
-        <v>Kmu0wc9ruhag0</v>
+        <v>Kmu0wctkuy9ej</v>
       </c>
       <c r="B2355" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90067,7 +90067,7 @@
     </row>
     <row r="2356">
       <c r="A2356" t="str">
-        <v>Kmu0wc9ru7m9j</v>
+        <v>Kmu0wctkuf885</v>
       </c>
       <c r="B2356" t="str">
         <v>Penata Keprotokolan*</v>
@@ -90143,7 +90143,7 @@
     </row>
     <row r="2358">
       <c r="A2358" t="str">
-        <v>Kmu0wc9ruldak</v>
+        <v>Kmu0wctkuh8jx</v>
       </c>
       <c r="B2358" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90181,7 +90181,7 @@
     </row>
     <row r="2359">
       <c r="A2359" t="str">
-        <v>Kmu0wc9ru5l1b</v>
+        <v>Kmu0wctkuvnxy</v>
       </c>
       <c r="B2359" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90219,7 +90219,7 @@
     </row>
     <row r="2360">
       <c r="A2360" t="str">
-        <v>Kmu0wc9rud4jb</v>
+        <v>Kmu0wctkuam89</v>
       </c>
       <c r="B2360" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90333,7 +90333,7 @@
     </row>
     <row r="2363">
       <c r="A2363" t="str">
-        <v>Kmu0wc9ruxp5p</v>
+        <v>Kmu0wctku9evv</v>
       </c>
       <c r="B2363" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -90371,7 +90371,7 @@
     </row>
     <row r="2364">
       <c r="A2364" t="str">
-        <v>Kmu0wc9ru8mok</v>
+        <v>Kmu0wctkuqi0x</v>
       </c>
       <c r="B2364" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90409,7 +90409,7 @@
     </row>
     <row r="2365">
       <c r="A2365" t="str">
-        <v>Kmu0wc9ruwkac</v>
+        <v>Kmu0wctku4v82</v>
       </c>
       <c r="B2365" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90485,7 +90485,7 @@
     </row>
     <row r="2367">
       <c r="A2367" t="str">
-        <v>Kmu0wc9ru8pqr</v>
+        <v>Kmu0wctkuwch3</v>
       </c>
       <c r="B2367" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90523,7 +90523,7 @@
     </row>
     <row r="2368">
       <c r="A2368" t="str">
-        <v>Kmu0wc9ruvcph</v>
+        <v>Kmu0wctkuexns</v>
       </c>
       <c r="B2368" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90561,7 +90561,7 @@
     </row>
     <row r="2369">
       <c r="A2369" t="str">
-        <v>Kmu0wc9ru02pf</v>
+        <v>Kmu0wctkuwhj4</v>
       </c>
       <c r="B2369" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90637,7 +90637,7 @@
     </row>
     <row r="2371">
       <c r="A2371" t="str">
-        <v>Kmu0wc9ru0qyn</v>
+        <v>Kmu0wctku1g8s</v>
       </c>
       <c r="B2371" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -90675,7 +90675,7 @@
     </row>
     <row r="2372">
       <c r="A2372" t="str">
-        <v>Kmu0wc9ru8mg1</v>
+        <v>Kmu0wctkuxwtc</v>
       </c>
       <c r="B2372" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90713,7 +90713,7 @@
     </row>
     <row r="2373">
       <c r="A2373" t="str">
-        <v>Kmu0wc9ru9mxp</v>
+        <v>Kmu0wctku1aj5</v>
       </c>
       <c r="B2373" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90789,7 +90789,7 @@
     </row>
     <row r="2375">
       <c r="A2375" t="str">
-        <v>Kmu0wc9ruap80</v>
+        <v>Kmu0wctkulapv</v>
       </c>
       <c r="B2375" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90827,7 +90827,7 @@
     </row>
     <row r="2376">
       <c r="A2376" t="str">
-        <v>Kmu0wc9rulse5</v>
+        <v>Kmu0wctkua9f5</v>
       </c>
       <c r="B2376" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90865,7 +90865,7 @@
     </row>
     <row r="2377">
       <c r="A2377" t="str">
-        <v>Kmu0wc9ruw931</v>
+        <v>Kmu0wctku1y6e</v>
       </c>
       <c r="B2377" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90903,7 +90903,7 @@
     </row>
     <row r="2378">
       <c r="A2378" t="str">
-        <v>Kmu0wc9ru3o2j</v>
+        <v>Kmu0wctkuu8za</v>
       </c>
       <c r="B2378" t="str">
         <v xml:space="preserve">Analis Pembiayaan Risiko dan Keuangan/ Analis Keuangan Negara Ahli Utama									</v>

</xml_diff>

<commit_message>
Perbarui struktur organisasi (2026-09-14T07:04:17.603Z)
</commit_message>
<xml_diff>
--- a/data/struktur-organisasi.xlsx
+++ b/data/struktur-organisasi.xlsx
@@ -78173,7 +78173,7 @@
     </row>
     <row r="2043">
       <c r="A2043" t="str">
-        <v>Kmu0wctkt5ir5</v>
+        <v>Kmu0wc9rujtz8</v>
       </c>
       <c r="B2043" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78211,7 +78211,7 @@
     </row>
     <row r="2044">
       <c r="A2044" t="str">
-        <v>Kmu0wctktvsxv</v>
+        <v>Kmu0wc9rurj0c</v>
       </c>
       <c r="B2044" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78249,7 +78249,7 @@
     </row>
     <row r="2045">
       <c r="A2045" t="str">
-        <v>Kmu0wctkt2ps2</v>
+        <v>Kmu0wc9ruwu2e</v>
       </c>
       <c r="B2045" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78325,7 +78325,7 @@
     </row>
     <row r="2047">
       <c r="A2047" t="str">
-        <v>Kmu0wctkt2j97</v>
+        <v>Kmu0wc9ruod1l</v>
       </c>
       <c r="B2047" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78363,7 +78363,7 @@
     </row>
     <row r="2048">
       <c r="A2048" t="str">
-        <v>Kmu0wctktjx0q</v>
+        <v>Kmu0wc9rucmzi</v>
       </c>
       <c r="B2048" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78401,7 +78401,7 @@
     </row>
     <row r="2049">
       <c r="A2049" t="str">
-        <v>Kmu0wctktdeia</v>
+        <v>Kmu0wc9rukc1y</v>
       </c>
       <c r="B2049" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78477,7 +78477,7 @@
     </row>
     <row r="2051">
       <c r="A2051" t="str">
-        <v>Kmu0wctkt4u01</v>
+        <v>Kmu0wc9rukb73</v>
       </c>
       <c r="B2051" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78515,7 +78515,7 @@
     </row>
     <row r="2052">
       <c r="A2052" t="str">
-        <v>Kmu0wctkt24z2</v>
+        <v>Kmu0wc9ru2erp</v>
       </c>
       <c r="B2052" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78553,7 +78553,7 @@
     </row>
     <row r="2053">
       <c r="A2053" t="str">
-        <v>Kmu0wctktefds</v>
+        <v>Kmu0wc9rumrxv</v>
       </c>
       <c r="B2053" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78591,7 +78591,7 @@
     </row>
     <row r="2054">
       <c r="A2054" t="str">
-        <v>Kmu0wctktlvvd</v>
+        <v>Kmu0wc9ru36sx</v>
       </c>
       <c r="B2054" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -78629,7 +78629,7 @@
     </row>
     <row r="2055">
       <c r="A2055" t="str">
-        <v>Kmu0wctkt3evn</v>
+        <v>Kmu0wc9ruh4wk</v>
       </c>
       <c r="B2055" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -78667,7 +78667,7 @@
     </row>
     <row r="2056">
       <c r="A2056" t="str">
-        <v>Kmu0wctktchu2</v>
+        <v>Kmu0wc9ruop4g</v>
       </c>
       <c r="B2056" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -78705,7 +78705,7 @@
     </row>
     <row r="2057">
       <c r="A2057" t="str">
-        <v>Kmu0wctkt28g6</v>
+        <v>Kmu0wc9rudmjf</v>
       </c>
       <c r="B2057" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -78743,7 +78743,7 @@
     </row>
     <row r="2058">
       <c r="A2058" t="str">
-        <v>Kmu0wctkt2lya</v>
+        <v>Kmu0wc9ruaog3</v>
       </c>
       <c r="B2058" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -78857,7 +78857,7 @@
     </row>
     <row r="2061">
       <c r="A2061" t="str">
-        <v>Kmu0wctkt1ds6</v>
+        <v>Kmu0wc9rub1os</v>
       </c>
       <c r="B2061" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78895,7 +78895,7 @@
     </row>
     <row r="2062">
       <c r="A2062" t="str">
-        <v>Kmu0wctktemqp</v>
+        <v>Kmu0wc9rurhtd</v>
       </c>
       <c r="B2062" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78933,7 +78933,7 @@
     </row>
     <row r="2063">
       <c r="A2063" t="str">
-        <v>Kmu0wctktp0tl</v>
+        <v>Kmu0wc9rux9oj</v>
       </c>
       <c r="B2063" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79009,7 +79009,7 @@
     </row>
     <row r="2065">
       <c r="A2065" t="str">
-        <v>Kmu0wctku4zpl</v>
+        <v>Kmu0wc9rurp6m</v>
       </c>
       <c r="B2065" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79047,7 +79047,7 @@
     </row>
     <row r="2066">
       <c r="A2066" t="str">
-        <v>Kmu0wctku9w4e</v>
+        <v>Kmu0wc9ru2ii4</v>
       </c>
       <c r="B2066" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79085,7 +79085,7 @@
     </row>
     <row r="2067">
       <c r="A2067" t="str">
-        <v>Kmu0wctkuy6ub</v>
+        <v>Kmu0wc9ruc4bl</v>
       </c>
       <c r="B2067" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79161,7 +79161,7 @@
     </row>
     <row r="2069">
       <c r="A2069" t="str">
-        <v>Kmu0wctkuupme</v>
+        <v>Kmu0wc9rut1u3</v>
       </c>
       <c r="B2069" t="str">
         <v>Penata Layanan Operasional</v>
@@ -79199,7 +79199,7 @@
     </row>
     <row r="2070">
       <c r="A2070" t="str">
-        <v>Kmu0wctkuzg2e</v>
+        <v>Kmu0wc9ru3b47</v>
       </c>
       <c r="B2070" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79237,7 +79237,7 @@
     </row>
     <row r="2071">
       <c r="A2071" t="str">
-        <v>Kmu0wctkug3ir</v>
+        <v>Kmu0wc9ru6id1</v>
       </c>
       <c r="B2071" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79313,7 +79313,7 @@
     </row>
     <row r="2073">
       <c r="A2073" t="str">
-        <v>Kmu0wctku9fum</v>
+        <v>Kmu0wc9rurmhg</v>
       </c>
       <c r="B2073" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79351,7 +79351,7 @@
     </row>
     <row r="2074">
       <c r="A2074" t="str">
-        <v>Kmu0wctku21dy</v>
+        <v>Kmu0wc9ruwvh6</v>
       </c>
       <c r="B2074" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79389,7 +79389,7 @@
     </row>
     <row r="2075">
       <c r="A2075" t="str">
-        <v>Kmu0wctkug8at</v>
+        <v>Kmu0wc9ru1un0</v>
       </c>
       <c r="B2075" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79427,7 +79427,7 @@
     </row>
     <row r="2076">
       <c r="A2076" t="str">
-        <v>Kmu0wctkuhodk</v>
+        <v>Kmu0wc9rutg9r</v>
       </c>
       <c r="B2076" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -79465,7 +79465,7 @@
     </row>
     <row r="2077">
       <c r="A2077" t="str">
-        <v>Kmu0wctku1wx9</v>
+        <v>Kmu0wc9ruohwg</v>
       </c>
       <c r="B2077" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -79503,7 +79503,7 @@
     </row>
     <row r="2078">
       <c r="A2078" t="str">
-        <v>Kmu0wctkuv59z</v>
+        <v>Kmu0wc9ruc7fx</v>
       </c>
       <c r="B2078" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -79541,7 +79541,7 @@
     </row>
     <row r="2079">
       <c r="A2079" t="str">
-        <v>Kmu0wctkugyjy</v>
+        <v>Kmu0wc9ruc4gy</v>
       </c>
       <c r="B2079" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -79579,7 +79579,7 @@
     </row>
     <row r="2080">
       <c r="A2080" t="str">
-        <v>Kmu0wctkumzbk</v>
+        <v>Kmu0wc9rud74o</v>
       </c>
       <c r="B2080" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -79617,7 +79617,7 @@
     </row>
     <row r="2081">
       <c r="A2081" t="str">
-        <v>Kmu0wctkuy3qg</v>
+        <v>Kmu0wc9ruuunp</v>
       </c>
       <c r="B2081" t="str">
         <v>Asesor SDM Aparatur Ahli Muda</v>
@@ -79655,7 +79655,7 @@
     </row>
     <row r="2082">
       <c r="A2082" t="str">
-        <v>Kmu0wctkuq2sl</v>
+        <v>Kmu0wc9rum6o5</v>
       </c>
       <c r="B2082" t="str">
         <v>Asesor SDM Aparatur Ahli Pertama</v>
@@ -79769,7 +79769,7 @@
     </row>
     <row r="2085">
       <c r="A2085" t="str">
-        <v>Kmu0wctkuge2k</v>
+        <v>Kmu0wc9rush9e</v>
       </c>
       <c r="B2085" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79807,7 +79807,7 @@
     </row>
     <row r="2086">
       <c r="A2086" t="str">
-        <v>Kmu0wctkut91j</v>
+        <v>Kmu0wc9rux0n8</v>
       </c>
       <c r="B2086" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79845,7 +79845,7 @@
     </row>
     <row r="2087">
       <c r="A2087" t="str">
-        <v>Kmu0wctkud6gp</v>
+        <v>Kmu0wc9ruxcqv</v>
       </c>
       <c r="B2087" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79921,7 +79921,7 @@
     </row>
     <row r="2089">
       <c r="A2089" t="str">
-        <v>Kmu0wctkurd0q</v>
+        <v>Kmu0wc9runxdu</v>
       </c>
       <c r="B2089" t="str">
         <v>Penata Layanan Operasional</v>
@@ -79959,7 +79959,7 @@
     </row>
     <row r="2090">
       <c r="A2090" t="str">
-        <v>Kmu0wctkurkks</v>
+        <v>Kmu0wc9ruoo8b</v>
       </c>
       <c r="B2090" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79997,7 +79997,7 @@
     </row>
     <row r="2091">
       <c r="A2091" t="str">
-        <v>Kmu0wctkul5aj</v>
+        <v>Kmu0wc9rubs9x</v>
       </c>
       <c r="B2091" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80073,7 +80073,7 @@
     </row>
     <row r="2093">
       <c r="A2093" t="str">
-        <v>Kmu0wctkuq27r</v>
+        <v>Kmu0wc9rurwkl</v>
       </c>
       <c r="B2093" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80111,7 +80111,7 @@
     </row>
     <row r="2094">
       <c r="A2094" t="str">
-        <v>Kmu0wctkuf6eu</v>
+        <v>Kmu0wc9runpak</v>
       </c>
       <c r="B2094" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80149,7 +80149,7 @@
     </row>
     <row r="2095">
       <c r="A2095" t="str">
-        <v>Kmu0wctkuqxej</v>
+        <v>Kmu0wc9ruy6vs</v>
       </c>
       <c r="B2095" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80187,7 +80187,7 @@
     </row>
     <row r="2096">
       <c r="A2096" t="str">
-        <v>Kmu0wctku8uf6</v>
+        <v>Kmu0wc9ruiljc</v>
       </c>
       <c r="B2096" t="str">
         <v>Analis Anggaran Ahli Pertama/ Analis Keuangan Negara Ahli Pertama</v>
@@ -80225,7 +80225,7 @@
     </row>
     <row r="2097">
       <c r="A2097" t="str">
-        <v>Kmu0wctkuidbc</v>
+        <v>Kmu0wc9rucclj</v>
       </c>
       <c r="B2097" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Muda/Pengawas Keuangan Negara Ahli Muda</v>
@@ -80263,7 +80263,7 @@
     </row>
     <row r="2098">
       <c r="A2098" t="str">
-        <v>Kmu0wctkui8e3</v>
+        <v>Kmu0wc9ru291j</v>
       </c>
       <c r="B2098" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Pertama/Pengawas Keuangan Negara Ahli Pertama</v>
@@ -80301,7 +80301,7 @@
     </row>
     <row r="2099">
       <c r="A2099" t="str">
-        <v>Kmu0wctkub3ef</v>
+        <v>Kmu0wc9ruqjyi</v>
       </c>
       <c r="B2099" t="str">
         <v>Pranata Keuangan APBN Penyelia/Pengawas Keuangan Negara Penyelia</v>
@@ -80339,7 +80339,7 @@
     </row>
     <row r="2100">
       <c r="A2100" t="str">
-        <v>Kmu0wctku6a9g</v>
+        <v>Kmu0wc9run9o5</v>
       </c>
       <c r="B2100" t="str">
         <v>Pranata Keuangan APBN Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -80377,7 +80377,7 @@
     </row>
     <row r="2101">
       <c r="A2101" t="str">
-        <v>Kmu0wctku01ij</v>
+        <v>Kmu0wc9rubjuf</v>
       </c>
       <c r="B2101" t="str">
         <v>Pranata Keuangan APBN Terampil/Pengawas Keuangan Negara Terampil</v>
@@ -80415,7 +80415,7 @@
     </row>
     <row r="2102">
       <c r="A2102" t="str">
-        <v>Kmu0wctkumi5r</v>
+        <v>Kmu0wc9ruvjf0</v>
       </c>
       <c r="B2102" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -80453,7 +80453,7 @@
     </row>
     <row r="2103">
       <c r="A2103" t="str">
-        <v>Kmu0wctkul5hd</v>
+        <v>Kmu0wc9rulp9r</v>
       </c>
       <c r="B2103" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -80491,7 +80491,7 @@
     </row>
     <row r="2104">
       <c r="A2104" t="str">
-        <v>Kmu0wctkuo4nn</v>
+        <v>Kmu0wc9ru0do7</v>
       </c>
       <c r="B2104" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -80529,7 +80529,7 @@
     </row>
     <row r="2105">
       <c r="A2105" t="str">
-        <v>Kmu0wctku4uae</v>
+        <v>Kmu0wc9ru39s5</v>
       </c>
       <c r="B2105" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -80567,7 +80567,7 @@
     </row>
     <row r="2106">
       <c r="A2106" t="str">
-        <v>Kmu0wctkule2d</v>
+        <v>Kmu0wc9ru4u0k</v>
       </c>
       <c r="B2106" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -80681,7 +80681,7 @@
     </row>
     <row r="2109">
       <c r="A2109" t="str">
-        <v>Kmu0wctkugbli</v>
+        <v>Kmu0wc9rupb4c</v>
       </c>
       <c r="B2109" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80719,7 +80719,7 @@
     </row>
     <row r="2110">
       <c r="A2110" t="str">
-        <v>Kmu0wctkuy5vr</v>
+        <v>Kmu0wc9ruk9lg</v>
       </c>
       <c r="B2110" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80757,7 +80757,7 @@
     </row>
     <row r="2111">
       <c r="A2111" t="str">
-        <v>Kmu0wctkunwyg</v>
+        <v>Kmu0wc9runahm</v>
       </c>
       <c r="B2111" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80833,7 +80833,7 @@
     </row>
     <row r="2113">
       <c r="A2113" t="str">
-        <v>Kmu0wctkulmko</v>
+        <v>Kmu0wc9ruqt1d</v>
       </c>
       <c r="B2113" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80871,7 +80871,7 @@
     </row>
     <row r="2114">
       <c r="A2114" t="str">
-        <v>Kmu0wctkux6q5</v>
+        <v>Kmu0wc9ru9y1a</v>
       </c>
       <c r="B2114" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80909,7 +80909,7 @@
     </row>
     <row r="2115">
       <c r="A2115" t="str">
-        <v>Kmu0wctkuyz59</v>
+        <v>Kmu0wc9ru6vz1</v>
       </c>
       <c r="B2115" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80985,7 +80985,7 @@
     </row>
     <row r="2117">
       <c r="A2117" t="str">
-        <v>Kmu0wctku0kpn</v>
+        <v>Kmu0wc9run32d</v>
       </c>
       <c r="B2117" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -81023,7 +81023,7 @@
     </row>
     <row r="2118">
       <c r="A2118" t="str">
-        <v>Kmu0wctkuei6z</v>
+        <v>Kmu0wc9ruej1a</v>
       </c>
       <c r="B2118" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81061,7 +81061,7 @@
     </row>
     <row r="2119">
       <c r="A2119" t="str">
-        <v>Kmu0wctkuyeva</v>
+        <v>Kmu0wc9ruvivi</v>
       </c>
       <c r="B2119" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81099,7 +81099,7 @@
     </row>
     <row r="2120">
       <c r="A2120" t="str">
-        <v>Kmu0wctku3ztp</v>
+        <v>Kmu0wc9rufkc7</v>
       </c>
       <c r="B2120" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -81137,7 +81137,7 @@
     </row>
     <row r="2121">
       <c r="A2121" t="str">
-        <v>Kmu0wctkucnm5</v>
+        <v>Kmu0wc9rutr7z</v>
       </c>
       <c r="B2121" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -81175,7 +81175,7 @@
     </row>
     <row r="2122">
       <c r="A2122" t="str">
-        <v>Kmu0wctkuthyt</v>
+        <v>Kmu0wc9rubeqs</v>
       </c>
       <c r="B2122" t="str">
         <v>Pengawas Keuangan Negara Mahir</v>
@@ -81213,7 +81213,7 @@
     </row>
     <row r="2123">
       <c r="A2123" t="str">
-        <v>Kmu0wctku4sop</v>
+        <v>Kmu0wc9ruxicw</v>
       </c>
       <c r="B2123" t="str">
         <v>Pengawas Keuangan Negara Terampil</v>
@@ -81327,7 +81327,7 @@
     </row>
     <row r="2126">
       <c r="A2126" t="str">
-        <v>Kmu0wctkupls0</v>
+        <v>Kmu0wc9ruta9e</v>
       </c>
       <c r="B2126" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81365,7 +81365,7 @@
     </row>
     <row r="2127">
       <c r="A2127" t="str">
-        <v>Kmu0wctkuriff</v>
+        <v>Kmu0wc9ruuldg</v>
       </c>
       <c r="B2127" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81403,7 +81403,7 @@
     </row>
     <row r="2128">
       <c r="A2128" t="str">
-        <v>Kmu0wctku76nh</v>
+        <v>Kmu0wc9rub4xn</v>
       </c>
       <c r="B2128" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81441,7 +81441,7 @@
     </row>
     <row r="2129">
       <c r="A2129" t="str">
-        <v>Kmu0wctkuwf04</v>
+        <v>Kmu0wc9rugesh</v>
       </c>
       <c r="B2129" t="str">
         <v>Penata Keprotokolan*</v>
@@ -81517,7 +81517,7 @@
     </row>
     <row r="2131">
       <c r="A2131" t="str">
-        <v>Kmu0wctkuvquq</v>
+        <v>Kmu0wc9ruk3kr</v>
       </c>
       <c r="B2131" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81555,7 +81555,7 @@
     </row>
     <row r="2132">
       <c r="A2132" t="str">
-        <v>Kmu0wctkuj4f4</v>
+        <v>Kmu0wc9ruwju1</v>
       </c>
       <c r="B2132" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81593,7 +81593,7 @@
     </row>
     <row r="2133">
       <c r="A2133" t="str">
-        <v>Kmu0wctkue309</v>
+        <v>Kmu0wc9ruh84t</v>
       </c>
       <c r="B2133" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81631,7 +81631,7 @@
     </row>
     <row r="2134">
       <c r="A2134" t="str">
-        <v>Kmu0wctku10te</v>
+        <v>Kmu0wc9ru8mam</v>
       </c>
       <c r="B2134" t="str">
         <v>Penata Keprotokolan*</v>
@@ -81707,7 +81707,7 @@
     </row>
     <row r="2136">
       <c r="A2136" t="str">
-        <v>Kmu0wctkukia5</v>
+        <v>Kmu0wc9ru5hk3</v>
       </c>
       <c r="B2136" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81745,7 +81745,7 @@
     </row>
     <row r="2137">
       <c r="A2137" t="str">
-        <v>Kmu0wctku1dna</v>
+        <v>Kmu0wc9ruoivv</v>
       </c>
       <c r="B2137" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81783,7 +81783,7 @@
     </row>
     <row r="2138">
       <c r="A2138" t="str">
-        <v>Kmu0wctkuhuvv</v>
+        <v>Kmu0wc9rujql5</v>
       </c>
       <c r="B2138" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81821,7 +81821,7 @@
     </row>
     <row r="2139">
       <c r="A2139" t="str">
-        <v>Kmu0wctkum4u4</v>
+        <v>Kmu0wc9rux86x</v>
       </c>
       <c r="B2139" t="str">
         <v>Pengawas Keuangan Negara Ahli Muda</v>
@@ -81859,7 +81859,7 @@
     </row>
     <row r="2140">
       <c r="A2140" t="str">
-        <v>Kmu0wctku9p12</v>
+        <v>Kmu0wc9rupac2</v>
       </c>
       <c r="B2140" t="str">
         <v>Pengawas Keuangan Negara Pertama</v>
@@ -81897,7 +81897,7 @@
     </row>
     <row r="2141">
       <c r="A2141" t="str">
-        <v>Kmu0wctkuhk8e</v>
+        <v>Kmu0wc9rufl0v</v>
       </c>
       <c r="B2141" t="str">
         <v>Penata Laksana Barang Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -81935,7 +81935,7 @@
     </row>
     <row r="2142">
       <c r="A2142" t="str">
-        <v>Kmu0wctkutajo</v>
+        <v>Kmu0wc9ru6yl5</v>
       </c>
       <c r="B2142" t="str">
         <v>Penata Laksana Barang Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -81973,7 +81973,7 @@
     </row>
     <row r="2143">
       <c r="A2143" t="str">
-        <v>Kmu0wctkuwj8j</v>
+        <v>Kmu0wc9ru6h6t</v>
       </c>
       <c r="B2143" t="str">
         <v>Penata Laksana Barang Terampil/ Pengawas Keuangan Negara Terampil</v>
@@ -82011,7 +82011,7 @@
     </row>
     <row r="2144">
       <c r="A2144" t="str">
-        <v>Kmu0wctku3r8t</v>
+        <v>Kmu0wc9rujgyg</v>
       </c>
       <c r="B2144" t="str">
         <v>Arsiparis Ahli Muda</v>
@@ -82049,7 +82049,7 @@
     </row>
     <row r="2145">
       <c r="A2145" t="str">
-        <v>Kmu0wctku37fx</v>
+        <v>Kmu0wc9ru1z8y</v>
       </c>
       <c r="B2145" t="str">
         <v>Arsiparis Ahli Pertama</v>
@@ -82087,7 +82087,7 @@
     </row>
     <row r="2146">
       <c r="A2146" t="str">
-        <v>Kmu0wctku2z33</v>
+        <v>Kmu0wc9rujrfi</v>
       </c>
       <c r="B2146" t="str">
         <v>Arsiparis Penyelia</v>
@@ -82125,7 +82125,7 @@
     </row>
     <row r="2147">
       <c r="A2147" t="str">
-        <v>Kmu0wctku6vac</v>
+        <v>Kmu0wc9rui5es</v>
       </c>
       <c r="B2147" t="str">
         <v>Arsiparis Mahir</v>
@@ -82163,7 +82163,7 @@
     </row>
     <row r="2148">
       <c r="A2148" t="str">
-        <v>Kmu0wctkuy4qj</v>
+        <v>Kmu0wc9ruk2fd</v>
       </c>
       <c r="B2148" t="str">
         <v>Arsiparis Terampil</v>
@@ -82277,7 +82277,7 @@
     </row>
     <row r="2151">
       <c r="A2151" t="str">
-        <v>Kmu0wctku67al</v>
+        <v>Kmu0wc9ru0hse</v>
       </c>
       <c r="B2151" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -82315,7 +82315,7 @@
     </row>
     <row r="2152">
       <c r="A2152" t="str">
-        <v>Kmu0wctkuso64</v>
+        <v>Kmu0wc9ru2vrj</v>
       </c>
       <c r="B2152" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82353,7 +82353,7 @@
     </row>
     <row r="2153">
       <c r="A2153" t="str">
-        <v>Kmu0wctkut7ae</v>
+        <v>Kmu0wc9ruxlqp</v>
       </c>
       <c r="B2153" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82391,7 +82391,7 @@
     </row>
     <row r="2154">
       <c r="A2154" t="str">
-        <v>Kmu0wctku1tdf</v>
+        <v>Kmu0wc9ruwk5t</v>
       </c>
       <c r="B2154" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -82429,7 +82429,7 @@
     </row>
     <row r="2155">
       <c r="A2155" t="str">
-        <v>Kmu0wctku2kli</v>
+        <v>Kmu0wc9ruhjw7</v>
       </c>
       <c r="B2155" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -82467,7 +82467,7 @@
     </row>
     <row r="2156">
       <c r="A2156" t="str">
-        <v>Kmu0wctkuzdoe</v>
+        <v>Kmu0wc9ruwu98</v>
       </c>
       <c r="B2156" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -82505,7 +82505,7 @@
     </row>
     <row r="2157">
       <c r="A2157" t="str">
-        <v>Kmu0wctkuunbj</v>
+        <v>Kmu0wc9ruay2u</v>
       </c>
       <c r="B2157" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -82581,7 +82581,7 @@
     </row>
     <row r="2159">
       <c r="A2159" t="str">
-        <v>Kmu0wctkuu3dj</v>
+        <v>Kmu0wc9ruw0s3</v>
       </c>
       <c r="B2159" t="str">
         <v>Penata Layanan Operasional</v>
@@ -82619,7 +82619,7 @@
     </row>
     <row r="2160">
       <c r="A2160" t="str">
-        <v>Kmu0wctku67qh</v>
+        <v>Kmu0wc9ruszwr</v>
       </c>
       <c r="B2160" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82657,7 +82657,7 @@
     </row>
     <row r="2161">
       <c r="A2161" t="str">
-        <v>Kmu0wctkufrqr</v>
+        <v>Kmu0wc9ru3ntx</v>
       </c>
       <c r="B2161" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82695,7 +82695,7 @@
     </row>
     <row r="2162">
       <c r="A2162" t="str">
-        <v>Kmu0wctkupczk</v>
+        <v>Kmu0wc9rullsh</v>
       </c>
       <c r="B2162" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -82733,7 +82733,7 @@
     </row>
     <row r="2163">
       <c r="A2163" t="str">
-        <v>Kmu0wctku1hd1</v>
+        <v>Kmu0wc9ruvc4p</v>
       </c>
       <c r="B2163" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -82771,7 +82771,7 @@
     </row>
     <row r="2164">
       <c r="A2164" t="str">
-        <v>Kmu0wctku1ruu</v>
+        <v>Kmu0wc9rue7vo</v>
       </c>
       <c r="B2164" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -82809,7 +82809,7 @@
     </row>
     <row r="2165">
       <c r="A2165" t="str">
-        <v>Kmu0wctkud9je</v>
+        <v>Kmu0wc9rua65j</v>
       </c>
       <c r="B2165" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -82885,7 +82885,7 @@
     </row>
     <row r="2167">
       <c r="A2167" t="str">
-        <v>Kmu0wctkuax5b</v>
+        <v>Kmu0wc9ru7co1</v>
       </c>
       <c r="B2167" t="str">
         <v>Penata Layanan Operasional</v>
@@ -82923,7 +82923,7 @@
     </row>
     <row r="2168">
       <c r="A2168" t="str">
-        <v>Kmu0wctkunfgp</v>
+        <v>Kmu0wc9rulfm3</v>
       </c>
       <c r="B2168" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82961,7 +82961,7 @@
     </row>
     <row r="2169">
       <c r="A2169" t="str">
-        <v>Kmu0wctkux6y3</v>
+        <v>Kmu0wc9rusa9q</v>
       </c>
       <c r="B2169" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82999,7 +82999,7 @@
     </row>
     <row r="2170">
       <c r="A2170" t="str">
-        <v>Kmu0wctku9r79</v>
+        <v>Kmu0wc9ruql77</v>
       </c>
       <c r="B2170" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -83037,7 +83037,7 @@
     </row>
     <row r="2171">
       <c r="A2171" t="str">
-        <v>Kmu0wctkui3g1</v>
+        <v>Kmu0wc9ruhyq3</v>
       </c>
       <c r="B2171" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -83075,7 +83075,7 @@
     </row>
     <row r="2172">
       <c r="A2172" t="str">
-        <v>Kmu0wctkuddzq</v>
+        <v>Kmu0wc9ru4r7f</v>
       </c>
       <c r="B2172" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -83113,7 +83113,7 @@
     </row>
     <row r="2173">
       <c r="A2173" t="str">
-        <v>Kmu0wctkuy7ed</v>
+        <v>Kmu0wc9rux1u2</v>
       </c>
       <c r="B2173" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -83151,7 +83151,7 @@
     </row>
     <row r="2174">
       <c r="A2174" t="str">
-        <v>Kmu0wctkujpn2</v>
+        <v>Kmu0wc9ru73d3</v>
       </c>
       <c r="B2174" t="str">
         <v>Pranata Humas Ahli Muda</v>
@@ -83189,7 +83189,7 @@
     </row>
     <row r="2175">
       <c r="A2175" t="str">
-        <v>Kmu0wctkub8r6</v>
+        <v>Kmu0wc9ruv2gf</v>
       </c>
       <c r="B2175" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -83227,7 +83227,7 @@
     </row>
     <row r="2176">
       <c r="A2176" t="str">
-        <v>Kmu0wctku9j39</v>
+        <v>Kmu0wc9rucj6l</v>
       </c>
       <c r="B2176" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -83265,7 +83265,7 @@
     </row>
     <row r="2177">
       <c r="A2177" t="str">
-        <v>Kmu0wctkuy1xq</v>
+        <v>Kmu0wc9ruapk4</v>
       </c>
       <c r="B2177" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -83303,7 +83303,7 @@
     </row>
     <row r="2178">
       <c r="A2178" t="str">
-        <v>Kmu0wctku21jk</v>
+        <v>Kmu0wc9ruhg37</v>
       </c>
       <c r="B2178" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -83341,7 +83341,7 @@
     </row>
     <row r="2179">
       <c r="A2179" t="str">
-        <v>Kmu0wctku7wan</v>
+        <v>Kmu0wc9ru6w84</v>
       </c>
       <c r="B2179" t="str">
         <v>Pustakawan Ahli Pertama</v>
@@ -83379,7 +83379,7 @@
     </row>
     <row r="2180">
       <c r="A2180" t="str">
-        <v>Kmu0wctku3vlk</v>
+        <v>Kmu0wc9rujt7h</v>
       </c>
       <c r="B2180" t="str">
         <v>Asisten Perpustakaan Penyelia</v>
@@ -83417,7 +83417,7 @@
     </row>
     <row r="2181">
       <c r="A2181" t="str">
-        <v>Kmu0wctkuif27</v>
+        <v>Kmu0wc9ru4ati</v>
       </c>
       <c r="B2181" t="str">
         <v>Asisten Perpustakaan Mahir</v>
@@ -83455,7 +83455,7 @@
     </row>
     <row r="2182">
       <c r="A2182" t="str">
-        <v>Kmu0wctkude8a</v>
+        <v>Kmu0wc9ruvw2x</v>
       </c>
       <c r="B2182" t="str">
         <v>Asisten Perpustakaan Terampil</v>
@@ -83493,7 +83493,7 @@
     </row>
     <row r="2183">
       <c r="A2183" t="str">
-        <v>Kmu0wctkuoii3</v>
+        <v>Kmu0wc9rusees</v>
       </c>
       <c r="B2183" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Madya/Pengawas Keuangan Negara Ahli Madya</v>
@@ -83531,7 +83531,7 @@
     </row>
     <row r="2184">
       <c r="A2184" t="str">
-        <v>Kmu0wctku4p9p</v>
+        <v>Kmu0wc9ruq480</v>
       </c>
       <c r="B2184" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Muda</v>
@@ -83569,7 +83569,7 @@
     </row>
     <row r="2185">
       <c r="A2185" t="str">
-        <v>Kmu0wctkus6p7</v>
+        <v>Kmu0wc9ruo539</v>
       </c>
       <c r="B2185" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Pertama</v>
@@ -83683,7 +83683,7 @@
     </row>
     <row r="2188">
       <c r="A2188" t="str">
-        <v>Kmu0wctkuokeg</v>
+        <v>Kmu0wc9rupbu9</v>
       </c>
       <c r="B2188" t="str">
         <v>Penata Layanan Operasional</v>
@@ -83721,7 +83721,7 @@
     </row>
     <row r="2189">
       <c r="A2189" t="str">
-        <v>Kmu0wctkunfqg</v>
+        <v>Kmu0wc9ru4yf6</v>
       </c>
       <c r="B2189" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -83759,7 +83759,7 @@
     </row>
     <row r="2190">
       <c r="A2190" t="str">
-        <v>Kmu0wctkujhme</v>
+        <v>Kmu0wc9ruzhbh</v>
       </c>
       <c r="B2190" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -83797,7 +83797,7 @@
     </row>
     <row r="2191">
       <c r="A2191" t="str">
-        <v>Kmu0wctkua43g</v>
+        <v>Kmu0wc9ruqhnl</v>
       </c>
       <c r="B2191" t="str">
         <v>Penata Keprotokolan*</v>
@@ -83911,7 +83911,7 @@
     </row>
     <row r="2194">
       <c r="A2194" t="str">
-        <v>Kmu0wctku8dwh</v>
+        <v>Kmu0wc9ru5uf6</v>
       </c>
       <c r="B2194" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -83949,7 +83949,7 @@
     </row>
     <row r="2195">
       <c r="A2195" t="str">
-        <v>Kmu0wctku6lkm</v>
+        <v>Kmu0wc9rufx21</v>
       </c>
       <c r="B2195" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -83987,7 +83987,7 @@
     </row>
     <row r="2196">
       <c r="A2196" t="str">
-        <v>Kmu0wctkubd8x</v>
+        <v>Kmu0wc9rugbpu</v>
       </c>
       <c r="B2196" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84063,7 +84063,7 @@
     </row>
     <row r="2198">
       <c r="A2198" t="str">
-        <v>Kmu0wctkufk8q</v>
+        <v>Kmu0wc9ru78oz</v>
       </c>
       <c r="B2198" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84101,7 +84101,7 @@
     </row>
     <row r="2199">
       <c r="A2199" t="str">
-        <v>Kmu0wctkuyjde</v>
+        <v>Kmu0wc9ruii9t</v>
       </c>
       <c r="B2199" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84139,7 +84139,7 @@
     </row>
     <row r="2200">
       <c r="A2200" t="str">
-        <v>Kmu0wctku4zun</v>
+        <v>Kmu0wc9ru6e2j</v>
       </c>
       <c r="B2200" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84177,7 +84177,7 @@
     </row>
     <row r="2201">
       <c r="A2201" t="str">
-        <v>Kmu0wctku1w08</v>
+        <v>Kmu0wc9ru1zwr</v>
       </c>
       <c r="B2201" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -84215,7 +84215,7 @@
     </row>
     <row r="2202">
       <c r="A2202" t="str">
-        <v>Kmu0wctkubqeu</v>
+        <v>Kmu0wc9rukf2l</v>
       </c>
       <c r="B2202" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -84253,7 +84253,7 @@
     </row>
     <row r="2203">
       <c r="A2203" t="str">
-        <v>Kmu0wctkupuna</v>
+        <v>Kmu0wc9ruf7p4</v>
       </c>
       <c r="B2203" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -84291,7 +84291,7 @@
     </row>
     <row r="2204">
       <c r="A2204" t="str">
-        <v>Kmu0wctku8woi</v>
+        <v>Kmu0wc9ruwwjv</v>
       </c>
       <c r="B2204" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -84405,7 +84405,7 @@
     </row>
     <row r="2207">
       <c r="A2207" t="str">
-        <v>Kmu0wctkurw1l</v>
+        <v>Kmu0wc9ruj4my</v>
       </c>
       <c r="B2207" t="str">
         <v>Penata Layanan Operasional</v>
@@ -84443,7 +84443,7 @@
     </row>
     <row r="2208">
       <c r="A2208" t="str">
-        <v>Kmu0wctkuhyt7</v>
+        <v>Kmu0wc9rutwo3</v>
       </c>
       <c r="B2208" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84481,7 +84481,7 @@
     </row>
     <row r="2209">
       <c r="A2209" t="str">
-        <v>Kmu0wctkutday</v>
+        <v>Kmu0wc9run1p7</v>
       </c>
       <c r="B2209" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84519,7 +84519,7 @@
     </row>
     <row r="2210">
       <c r="A2210" t="str">
-        <v>Kmu0wctku5q5v</v>
+        <v>Kmu0wc9run2i1</v>
       </c>
       <c r="B2210" t="str">
         <v>Penata Keprotokolan*</v>
@@ -84633,7 +84633,7 @@
     </row>
     <row r="2213">
       <c r="A2213" t="str">
-        <v>Kmu0wctkumtls</v>
+        <v>Kmu0wc9ruo11r</v>
       </c>
       <c r="B2213" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84671,7 +84671,7 @@
     </row>
     <row r="2214">
       <c r="A2214" t="str">
-        <v>Kmu0wctku9ar8</v>
+        <v>Kmu0wc9ru9cwp</v>
       </c>
       <c r="B2214" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84709,7 +84709,7 @@
     </row>
     <row r="2215">
       <c r="A2215" t="str">
-        <v>Kmu0wctkuawow</v>
+        <v>Kmu0wc9ruf0fx</v>
       </c>
       <c r="B2215" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84785,7 +84785,7 @@
     </row>
     <row r="2217">
       <c r="A2217" t="str">
-        <v>Kmu0wctku9wuz</v>
+        <v>Kmu0wc9rups46</v>
       </c>
       <c r="B2217" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84823,7 +84823,7 @@
     </row>
     <row r="2218">
       <c r="A2218" t="str">
-        <v>Kmu0wctkui55s</v>
+        <v>Kmu0wc9rui35c</v>
       </c>
       <c r="B2218" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84861,7 +84861,7 @@
     </row>
     <row r="2219">
       <c r="A2219" t="str">
-        <v>Kmu0wctkuyp1e</v>
+        <v>Kmu0wc9rupgnl</v>
       </c>
       <c r="B2219" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84899,7 +84899,7 @@
     </row>
     <row r="2220">
       <c r="A2220" t="str">
-        <v>Kmu0wctkuwd9z</v>
+        <v>Kmu0wc9rumvz6</v>
       </c>
       <c r="B2220" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -84937,7 +84937,7 @@
     </row>
     <row r="2221">
       <c r="A2221" t="str">
-        <v>Kmu0wctku2xci</v>
+        <v>Kmu0wc9ru4qtd</v>
       </c>
       <c r="B2221" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -84975,7 +84975,7 @@
     </row>
     <row r="2222">
       <c r="A2222" t="str">
-        <v>Kmu0wctkuehsv</v>
+        <v>Kmu0wc9ru8hw2</v>
       </c>
       <c r="B2222" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -85013,7 +85013,7 @@
     </row>
     <row r="2223">
       <c r="A2223" t="str">
-        <v>Kmu0wctkuygov</v>
+        <v>Kmu0wc9rujea9</v>
       </c>
       <c r="B2223" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -85127,7 +85127,7 @@
     </row>
     <row r="2226">
       <c r="A2226" t="str">
-        <v>Kmu0wctkuv1uf</v>
+        <v>Kmu0wc9ruere6</v>
       </c>
       <c r="B2226" t="str">
         <v>Penata Layanan Operasional</v>
@@ -85165,7 +85165,7 @@
     </row>
     <row r="2227">
       <c r="A2227" t="str">
-        <v>Kmu0wctkuu6th</v>
+        <v>Kmu0wc9rusb13</v>
       </c>
       <c r="B2227" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85203,7 +85203,7 @@
     </row>
     <row r="2228">
       <c r="A2228" t="str">
-        <v>Kmu0wctkuri7g</v>
+        <v>Kmu0wc9rusa7k</v>
       </c>
       <c r="B2228" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85241,7 +85241,7 @@
     </row>
     <row r="2229">
       <c r="A2229" t="str">
-        <v>Kmu0wctkumc44</v>
+        <v>Kmu0wc9rufx5e</v>
       </c>
       <c r="B2229" t="str">
         <v>Penata Keprotokolan*</v>
@@ -85355,7 +85355,7 @@
     </row>
     <row r="2232">
       <c r="A2232" t="str">
-        <v>Kmu0wctku39a9</v>
+        <v>Kmu0wc9ruow77</v>
       </c>
       <c r="B2232" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -85393,7 +85393,7 @@
     </row>
     <row r="2233">
       <c r="A2233" t="str">
-        <v>Kmu0wctku2hdj</v>
+        <v>Kmu0wc9ru6l55</v>
       </c>
       <c r="B2233" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85431,7 +85431,7 @@
     </row>
     <row r="2234">
       <c r="A2234" t="str">
-        <v>Kmu0wctku4pyc</v>
+        <v>Kmu0wc9ruvgmk</v>
       </c>
       <c r="B2234" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85507,7 +85507,7 @@
     </row>
     <row r="2236">
       <c r="A2236" t="str">
-        <v>Kmu0wctkuwfii</v>
+        <v>Kmu0wc9ruahgo</v>
       </c>
       <c r="B2236" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -85545,7 +85545,7 @@
     </row>
     <row r="2237">
       <c r="A2237" t="str">
-        <v>Kmu0wctkuzu64</v>
+        <v>Kmu0wc9rulrcd</v>
       </c>
       <c r="B2237" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85583,7 +85583,7 @@
     </row>
     <row r="2238">
       <c r="A2238" t="str">
-        <v>Kmu0wctkuxbgm</v>
+        <v>Kmu0wc9rupjts</v>
       </c>
       <c r="B2238" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85621,7 +85621,7 @@
     </row>
     <row r="2239">
       <c r="A2239" t="str">
-        <v>Kmu0wctku2xeo</v>
+        <v>Kmu0wc9ruf6jj</v>
       </c>
       <c r="B2239" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -85659,7 +85659,7 @@
     </row>
     <row r="2240">
       <c r="A2240" t="str">
-        <v>Kmu0wctku2d5o</v>
+        <v>Kmu0wc9ru4ujt</v>
       </c>
       <c r="B2240" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -85697,7 +85697,7 @@
     </row>
     <row r="2241">
       <c r="A2241" t="str">
-        <v>Kmu0wctkujki4</v>
+        <v>Kmu0wc9ruyp6k</v>
       </c>
       <c r="B2241" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -85735,7 +85735,7 @@
     </row>
     <row r="2242">
       <c r="A2242" t="str">
-        <v>Kmu0wctkumiq9</v>
+        <v>Kmu0wc9ruvixx</v>
       </c>
       <c r="B2242" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -85849,7 +85849,7 @@
     </row>
     <row r="2245">
       <c r="A2245" t="str">
-        <v>Kmu0wctkuvqm3</v>
+        <v>Kmu0wc9ru9yow</v>
       </c>
       <c r="B2245" t="str">
         <v>Penata Layanan Operasional</v>
@@ -85887,7 +85887,7 @@
     </row>
     <row r="2246">
       <c r="A2246" t="str">
-        <v>Kmu0wctkuod1p</v>
+        <v>Kmu0wc9ru0osn</v>
       </c>
       <c r="B2246" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85925,7 +85925,7 @@
     </row>
     <row r="2247">
       <c r="A2247" t="str">
-        <v>Kmu0wctkuhohp</v>
+        <v>Kmu0wc9ruy20a</v>
       </c>
       <c r="B2247" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85963,7 +85963,7 @@
     </row>
     <row r="2248">
       <c r="A2248" t="str">
-        <v>Kmu0wctku1m46</v>
+        <v>Kmu0wc9runcdt</v>
       </c>
       <c r="B2248" t="str">
         <v>Penata Keprotokolan*</v>
@@ -86039,7 +86039,7 @@
     </row>
     <row r="2250">
       <c r="A2250" t="str">
-        <v>Kmu0wctkud5om</v>
+        <v>Kmu0wc9ruc30w</v>
       </c>
       <c r="B2250" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86077,7 +86077,7 @@
     </row>
     <row r="2251">
       <c r="A2251" t="str">
-        <v>Kmu0wctkumyph</v>
+        <v>Kmu0wc9ruqdu8</v>
       </c>
       <c r="B2251" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86115,7 +86115,7 @@
     </row>
     <row r="2252">
       <c r="A2252" t="str">
-        <v>Kmu0wctku0dj3</v>
+        <v>Kmu0wc9ru29tq</v>
       </c>
       <c r="B2252" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86153,7 +86153,7 @@
     </row>
     <row r="2253">
       <c r="A2253" t="str">
-        <v>Kmu0wctkuvgxi</v>
+        <v>Kmu0wc9rush4e</v>
       </c>
       <c r="B2253" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -86191,7 +86191,7 @@
     </row>
     <row r="2254">
       <c r="A2254" t="str">
-        <v>Kmu0wctkuauj0</v>
+        <v>Kmu0wc9ru8lbq</v>
       </c>
       <c r="B2254" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -86305,7 +86305,7 @@
     </row>
     <row r="2257">
       <c r="A2257" t="str">
-        <v>Kmu0wctkulczd</v>
+        <v>Kmu0wc9ru3xek</v>
       </c>
       <c r="B2257" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86343,7 +86343,7 @@
     </row>
     <row r="2258">
       <c r="A2258" t="str">
-        <v>Kmu0wctkuvi2w</v>
+        <v>Kmu0wc9ruv3mz</v>
       </c>
       <c r="B2258" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86381,7 +86381,7 @@
     </row>
     <row r="2259">
       <c r="A2259" t="str">
-        <v>Kmu0wctkuwlrt</v>
+        <v>Kmu0wc9ruhttv</v>
       </c>
       <c r="B2259" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86457,7 +86457,7 @@
     </row>
     <row r="2261">
       <c r="A2261" t="str">
-        <v>Kmu0wctkudqkv</v>
+        <v>Kmu0wc9rug5yk</v>
       </c>
       <c r="B2261" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86495,7 +86495,7 @@
     </row>
     <row r="2262">
       <c r="A2262" t="str">
-        <v>Kmu0wctkuj6gq</v>
+        <v>Kmu0wc9ruo8m4</v>
       </c>
       <c r="B2262" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86533,7 +86533,7 @@
     </row>
     <row r="2263">
       <c r="A2263" t="str">
-        <v>Kmu0wctkujq4l</v>
+        <v>Kmu0wc9rug4zc</v>
       </c>
       <c r="B2263" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86571,7 +86571,7 @@
     </row>
     <row r="2264">
       <c r="A2264" t="str">
-        <v>Kmu0wctku7ws6</v>
+        <v>Kmu0wc9ru2z7b</v>
       </c>
       <c r="B2264" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -86609,7 +86609,7 @@
     </row>
     <row r="2265">
       <c r="A2265" t="str">
-        <v>Kmu0wctkuxc05</v>
+        <v>Kmu0wc9ru04o2</v>
       </c>
       <c r="B2265" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -86647,7 +86647,7 @@
     </row>
     <row r="2266">
       <c r="A2266" t="str">
-        <v>Kmu0wctkuotuj</v>
+        <v>Kmu0wc9ruyjdp</v>
       </c>
       <c r="B2266" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -86685,7 +86685,7 @@
     </row>
     <row r="2267">
       <c r="A2267" t="str">
-        <v>Kmu0wctkuj9wg</v>
+        <v>Kmu0wc9ruxl08</v>
       </c>
       <c r="B2267" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -86799,7 +86799,7 @@
     </row>
     <row r="2270">
       <c r="A2270" t="str">
-        <v>Kmu0wctkunle7</v>
+        <v>Kmu0wc9ru9xzh</v>
       </c>
       <c r="B2270" t="str">
         <v>Penata Layanan Operasional</v>
@@ -86837,7 +86837,7 @@
     </row>
     <row r="2271">
       <c r="A2271" t="str">
-        <v>Kmu0wctku3yop</v>
+        <v>Kmu0wc9ruo0tq</v>
       </c>
       <c r="B2271" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86875,7 +86875,7 @@
     </row>
     <row r="2272">
       <c r="A2272" t="str">
-        <v>Kmu0wctku6cy3</v>
+        <v>Kmu0wc9ruz7ff</v>
       </c>
       <c r="B2272" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86913,7 +86913,7 @@
     </row>
     <row r="2273">
       <c r="A2273" t="str">
-        <v>Kmu0wctku82u4</v>
+        <v>Kmu0wc9rum4zb</v>
       </c>
       <c r="B2273" t="str">
         <v>Penata Keprotokolan*</v>
@@ -87027,7 +87027,7 @@
     </row>
     <row r="2276">
       <c r="A2276" t="str">
-        <v>Kmu0wctkud2io</v>
+        <v>Kmu0wc9rusvra</v>
       </c>
       <c r="B2276" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87065,7 +87065,7 @@
     </row>
     <row r="2277">
       <c r="A2277" t="str">
-        <v>Kmu0wctku8on3</v>
+        <v>Kmu0wc9rugiqr</v>
       </c>
       <c r="B2277" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87103,7 +87103,7 @@
     </row>
     <row r="2278">
       <c r="A2278" t="str">
-        <v>Kmu0wctkuwwu8</v>
+        <v>Kmu0wc9rusnti</v>
       </c>
       <c r="B2278" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87179,7 +87179,7 @@
     </row>
     <row r="2280">
       <c r="A2280" t="str">
-        <v>Kmu0wctkuo10m</v>
+        <v>Kmu0wc9ruhiq3</v>
       </c>
       <c r="B2280" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87217,7 +87217,7 @@
     </row>
     <row r="2281">
       <c r="A2281" t="str">
-        <v>Kmu0wctku0zdl</v>
+        <v>Kmu0wc9rugmn0</v>
       </c>
       <c r="B2281" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87255,7 +87255,7 @@
     </row>
     <row r="2282">
       <c r="A2282" t="str">
-        <v>Kmu0wctkul1aw</v>
+        <v>Kmu0wc9ruel36</v>
       </c>
       <c r="B2282" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87293,7 +87293,7 @@
     </row>
     <row r="2283">
       <c r="A2283" t="str">
-        <v>Kmu0wctkuyx54</v>
+        <v>Kmu0wc9rujxf2</v>
       </c>
       <c r="B2283" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -87331,7 +87331,7 @@
     </row>
     <row r="2284">
       <c r="A2284" t="str">
-        <v>Kmu0wctkubfo1</v>
+        <v>Kmu0wc9ru8png</v>
       </c>
       <c r="B2284" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -87369,7 +87369,7 @@
     </row>
     <row r="2285">
       <c r="A2285" t="str">
-        <v>Kmu0wctkucbca</v>
+        <v>Kmu0wc9ru1k2m</v>
       </c>
       <c r="B2285" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -87407,7 +87407,7 @@
     </row>
     <row r="2286">
       <c r="A2286" t="str">
-        <v>Kmu0wctkulx35</v>
+        <v>Kmu0wc9ru53hm</v>
       </c>
       <c r="B2286" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -87521,7 +87521,7 @@
     </row>
     <row r="2289">
       <c r="A2289" t="str">
-        <v>Kmu0wctkub86l</v>
+        <v>Kmu0wc9ruzutl</v>
       </c>
       <c r="B2289" t="str">
         <v>Penata Layanan Operasional</v>
@@ -87559,7 +87559,7 @@
     </row>
     <row r="2290">
       <c r="A2290" t="str">
-        <v>Kmu0wctku19wo</v>
+        <v>Kmu0wc9ruk3m8</v>
       </c>
       <c r="B2290" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87597,7 +87597,7 @@
     </row>
     <row r="2291">
       <c r="A2291" t="str">
-        <v>Kmu0wctku8q8w</v>
+        <v>Kmu0wc9ru6bst</v>
       </c>
       <c r="B2291" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87635,7 +87635,7 @@
     </row>
     <row r="2292">
       <c r="A2292" t="str">
-        <v>Kmu0wctkurmmr</v>
+        <v>Kmu0wc9ru19pi</v>
       </c>
       <c r="B2292" t="str">
         <v>Penata Keprotokolan*</v>
@@ -87749,7 +87749,7 @@
     </row>
     <row r="2295">
       <c r="A2295" t="str">
-        <v>Kmu0wctkud0e9</v>
+        <v>Kmu0wc9ru567z</v>
       </c>
       <c r="B2295" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87787,7 +87787,7 @@
     </row>
     <row r="2296">
       <c r="A2296" t="str">
-        <v>Kmu0wctkuus5n</v>
+        <v>Kmu0wc9ruas84</v>
       </c>
       <c r="B2296" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87825,7 +87825,7 @@
     </row>
     <row r="2297">
       <c r="A2297" t="str">
-        <v>Kmu0wctkuqkwt</v>
+        <v>Kmu0wc9ruzs0r</v>
       </c>
       <c r="B2297" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87901,7 +87901,7 @@
     </row>
     <row r="2299">
       <c r="A2299" t="str">
-        <v>Kmu0wctku9vxj</v>
+        <v>Kmu0wc9ruc6d3</v>
       </c>
       <c r="B2299" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87939,7 +87939,7 @@
     </row>
     <row r="2300">
       <c r="A2300" t="str">
-        <v>Kmu0wctkulzjb</v>
+        <v>Kmu0wc9rugov1</v>
       </c>
       <c r="B2300" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87977,7 +87977,7 @@
     </row>
     <row r="2301">
       <c r="A2301" t="str">
-        <v>Kmu0wctkuvqtr</v>
+        <v>Kmu0wc9ruvncp</v>
       </c>
       <c r="B2301" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88015,7 +88015,7 @@
     </row>
     <row r="2302">
       <c r="A2302" t="str">
-        <v>Kmu0wctku3gcl</v>
+        <v>Kmu0wc9ru7fbe</v>
       </c>
       <c r="B2302" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -88053,7 +88053,7 @@
     </row>
     <row r="2303">
       <c r="A2303" t="str">
-        <v>Kmu0wctkundc7</v>
+        <v>Kmu0wc9ru83gg</v>
       </c>
       <c r="B2303" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -88091,7 +88091,7 @@
     </row>
     <row r="2304">
       <c r="A2304" t="str">
-        <v>Kmu0wctkuizdq</v>
+        <v>Kmu0wc9ru9i3z</v>
       </c>
       <c r="B2304" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -88129,7 +88129,7 @@
     </row>
     <row r="2305">
       <c r="A2305" t="str">
-        <v>Kmu0wctkumg01</v>
+        <v>Kmu0wc9ruz08i</v>
       </c>
       <c r="B2305" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -88243,7 +88243,7 @@
     </row>
     <row r="2308">
       <c r="A2308" t="str">
-        <v>Kmu0wctkuijm6</v>
+        <v>Kmu0wc9ru1ymb</v>
       </c>
       <c r="B2308" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88281,7 +88281,7 @@
     </row>
     <row r="2309">
       <c r="A2309" t="str">
-        <v>Kmu0wctkuopkn</v>
+        <v>Kmu0wc9ruz3yd</v>
       </c>
       <c r="B2309" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88319,7 +88319,7 @@
     </row>
     <row r="2310">
       <c r="A2310" t="str">
-        <v>Kmu0wctkuebmt</v>
+        <v>Kmu0wc9ru06mh</v>
       </c>
       <c r="B2310" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88357,7 +88357,7 @@
     </row>
     <row r="2311">
       <c r="A2311" t="str">
-        <v>Kmu0wctkufbkj</v>
+        <v>Kmu0wc9rue1gm</v>
       </c>
       <c r="B2311" t="str">
         <v>Penata Keprotokolan*</v>
@@ -88471,7 +88471,7 @@
     </row>
     <row r="2314">
       <c r="A2314" t="str">
-        <v>Kmu0wctku3j7z</v>
+        <v>Kmu0wc9ru0ydd</v>
       </c>
       <c r="B2314" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88509,7 +88509,7 @@
     </row>
     <row r="2315">
       <c r="A2315" t="str">
-        <v>Kmu0wctkubdov</v>
+        <v>Kmu0wc9ruvr3s</v>
       </c>
       <c r="B2315" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88547,7 +88547,7 @@
     </row>
     <row r="2316">
       <c r="A2316" t="str">
-        <v>Kmu0wctku6deh</v>
+        <v>Kmu0wc9ru2app</v>
       </c>
       <c r="B2316" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88623,7 +88623,7 @@
     </row>
     <row r="2318">
       <c r="A2318" t="str">
-        <v>Kmu0wctkujv30</v>
+        <v>Kmu0wc9ruhl6w</v>
       </c>
       <c r="B2318" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88661,7 +88661,7 @@
     </row>
     <row r="2319">
       <c r="A2319" t="str">
-        <v>Kmu0wctkuxm86</v>
+        <v>Kmu0wc9ruzmnx</v>
       </c>
       <c r="B2319" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88699,7 +88699,7 @@
     </row>
     <row r="2320">
       <c r="A2320" t="str">
-        <v>Kmu0wctkuc8l2</v>
+        <v>Kmu0wc9ru5m29</v>
       </c>
       <c r="B2320" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88775,7 +88775,7 @@
     </row>
     <row r="2322">
       <c r="A2322" t="str">
-        <v>Kmu0wctkuov3c</v>
+        <v>Kmu0wc9rukmke</v>
       </c>
       <c r="B2322" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88813,7 +88813,7 @@
     </row>
     <row r="2323">
       <c r="A2323" t="str">
-        <v>Kmu0wctkuzuqh</v>
+        <v>Kmu0wc9ru9yfs</v>
       </c>
       <c r="B2323" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88851,7 +88851,7 @@
     </row>
     <row r="2324">
       <c r="A2324" t="str">
-        <v>Kmu0wctkux5zm</v>
+        <v>Kmu0wc9ru3jd3</v>
       </c>
       <c r="B2324" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88927,7 +88927,7 @@
     </row>
     <row r="2326">
       <c r="A2326" t="str">
-        <v>Kmu0wctku3uhs</v>
+        <v>Kmu0wc9ru7ztu</v>
       </c>
       <c r="B2326" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88965,7 +88965,7 @@
     </row>
     <row r="2327">
       <c r="A2327" t="str">
-        <v>Kmu0wctku1tqi</v>
+        <v>Kmu0wc9ruas67</v>
       </c>
       <c r="B2327" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89003,7 +89003,7 @@
     </row>
     <row r="2328">
       <c r="A2328" t="str">
-        <v>Kmu0wctkujjxb</v>
+        <v>Kmu0wc9ruodbz</v>
       </c>
       <c r="B2328" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89117,7 +89117,7 @@
     </row>
     <row r="2331">
       <c r="A2331" t="str">
-        <v>Kmu0wctkuzvvi</v>
+        <v>Kmu0wc9runpra</v>
       </c>
       <c r="B2331" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89155,7 +89155,7 @@
     </row>
     <row r="2332">
       <c r="A2332" t="str">
-        <v>Kmu0wctku9wo5</v>
+        <v>Kmu0wc9rubopm</v>
       </c>
       <c r="B2332" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89193,7 +89193,7 @@
     </row>
     <row r="2333">
       <c r="A2333" t="str">
-        <v>Kmu0wctkulcis</v>
+        <v>Kmu0wc9ruduc5</v>
       </c>
       <c r="B2333" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89269,7 +89269,7 @@
     </row>
     <row r="2335">
       <c r="A2335" t="str">
-        <v>Kmu0wctkux7qi</v>
+        <v>Kmu0wc9rubb7m</v>
       </c>
       <c r="B2335" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89307,7 +89307,7 @@
     </row>
     <row r="2336">
       <c r="A2336" t="str">
-        <v>Kmu0wctkus0b9</v>
+        <v>Kmu0wc9rudmad</v>
       </c>
       <c r="B2336" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89345,7 +89345,7 @@
     </row>
     <row r="2337">
       <c r="A2337" t="str">
-        <v>Kmu0wctku9jv2</v>
+        <v>Kmu0wc9ruto33</v>
       </c>
       <c r="B2337" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89383,7 +89383,7 @@
     </row>
     <row r="2338">
       <c r="A2338" t="str">
-        <v>Kmu0wctkupx75</v>
+        <v>Kmu0wc9run813</v>
       </c>
       <c r="B2338" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -89421,7 +89421,7 @@
     </row>
     <row r="2339">
       <c r="A2339" t="str">
-        <v>Kmu0wctkunnk2</v>
+        <v>Kmu0wc9runcrh</v>
       </c>
       <c r="B2339" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -89459,7 +89459,7 @@
     </row>
     <row r="2340">
       <c r="A2340" t="str">
-        <v>Kmu0wctkurjcd</v>
+        <v>Kmu0wc9rutqd1</v>
       </c>
       <c r="B2340" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -89497,7 +89497,7 @@
     </row>
     <row r="2341">
       <c r="A2341" t="str">
-        <v>Kmu0wctku5lbw</v>
+        <v>Kmu0wc9rurqp0</v>
       </c>
       <c r="B2341" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -89611,7 +89611,7 @@
     </row>
     <row r="2344">
       <c r="A2344" t="str">
-        <v>Kmu0wctkulrg3</v>
+        <v>Kmu0wc9rulrbc</v>
       </c>
       <c r="B2344" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89649,7 +89649,7 @@
     </row>
     <row r="2345">
       <c r="A2345" t="str">
-        <v>Kmu0wctkuhg42</v>
+        <v>Kmu0wc9ruu1zb</v>
       </c>
       <c r="B2345" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89687,7 +89687,7 @@
     </row>
     <row r="2346">
       <c r="A2346" t="str">
-        <v>Kmu0wctkuusiq</v>
+        <v>Kmu0wc9ruv7tm</v>
       </c>
       <c r="B2346" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89801,7 +89801,7 @@
     </row>
     <row r="2349">
       <c r="A2349" t="str">
-        <v>Kmu0wctku252l</v>
+        <v>Kmu0wc9ru8lbh</v>
       </c>
       <c r="B2349" t="str">
         <v>Penata Layanan Operasional</v>
@@ -89839,7 +89839,7 @@
     </row>
     <row r="2350">
       <c r="A2350" t="str">
-        <v>Kmu0wctku465d</v>
+        <v>Kmu0wc9rui8f0</v>
       </c>
       <c r="B2350" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89877,7 +89877,7 @@
     </row>
     <row r="2351">
       <c r="A2351" t="str">
-        <v>Kmu0wctkux2i6</v>
+        <v>Kmu0wc9ru4wym</v>
       </c>
       <c r="B2351" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89953,7 +89953,7 @@
     </row>
     <row r="2353">
       <c r="A2353" t="str">
-        <v>Kmu0wctku6cwe</v>
+        <v>Kmu0wc9ru8yyu</v>
       </c>
       <c r="B2353" t="str">
         <v>Penata Layanan Operasional</v>
@@ -89991,7 +89991,7 @@
     </row>
     <row r="2354">
       <c r="A2354" t="str">
-        <v>Kmu0wctku8iax</v>
+        <v>Kmu0wc9ruk8ps</v>
       </c>
       <c r="B2354" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90029,7 +90029,7 @@
     </row>
     <row r="2355">
       <c r="A2355" t="str">
-        <v>Kmu0wctkuy9ej</v>
+        <v>Kmu0wc9ruhag0</v>
       </c>
       <c r="B2355" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90067,7 +90067,7 @@
     </row>
     <row r="2356">
       <c r="A2356" t="str">
-        <v>Kmu0wctkuf885</v>
+        <v>Kmu0wc9ru7m9j</v>
       </c>
       <c r="B2356" t="str">
         <v>Penata Keprotokolan*</v>
@@ -90143,7 +90143,7 @@
     </row>
     <row r="2358">
       <c r="A2358" t="str">
-        <v>Kmu0wctkuh8jx</v>
+        <v>Kmu0wc9ruldak</v>
       </c>
       <c r="B2358" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90181,7 +90181,7 @@
     </row>
     <row r="2359">
       <c r="A2359" t="str">
-        <v>Kmu0wctkuvnxy</v>
+        <v>Kmu0wc9ru5l1b</v>
       </c>
       <c r="B2359" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90219,7 +90219,7 @@
     </row>
     <row r="2360">
       <c r="A2360" t="str">
-        <v>Kmu0wctkuam89</v>
+        <v>Kmu0wc9rud4jb</v>
       </c>
       <c r="B2360" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90333,7 +90333,7 @@
     </row>
     <row r="2363">
       <c r="A2363" t="str">
-        <v>Kmu0wctku9evv</v>
+        <v>Kmu0wc9ruxp5p</v>
       </c>
       <c r="B2363" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -90371,7 +90371,7 @@
     </row>
     <row r="2364">
       <c r="A2364" t="str">
-        <v>Kmu0wctkuqi0x</v>
+        <v>Kmu0wc9ru8mok</v>
       </c>
       <c r="B2364" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90409,7 +90409,7 @@
     </row>
     <row r="2365">
       <c r="A2365" t="str">
-        <v>Kmu0wctku4v82</v>
+        <v>Kmu0wc9ruwkac</v>
       </c>
       <c r="B2365" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90485,7 +90485,7 @@
     </row>
     <row r="2367">
       <c r="A2367" t="str">
-        <v>Kmu0wctkuwch3</v>
+        <v>Kmu0wc9ru8pqr</v>
       </c>
       <c r="B2367" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90523,7 +90523,7 @@
     </row>
     <row r="2368">
       <c r="A2368" t="str">
-        <v>Kmu0wctkuexns</v>
+        <v>Kmu0wc9ruvcph</v>
       </c>
       <c r="B2368" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90561,7 +90561,7 @@
     </row>
     <row r="2369">
       <c r="A2369" t="str">
-        <v>Kmu0wctkuwhj4</v>
+        <v>Kmu0wc9ru02pf</v>
       </c>
       <c r="B2369" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90637,7 +90637,7 @@
     </row>
     <row r="2371">
       <c r="A2371" t="str">
-        <v>Kmu0wctku1g8s</v>
+        <v>Kmu0wc9ru0qyn</v>
       </c>
       <c r="B2371" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -90675,7 +90675,7 @@
     </row>
     <row r="2372">
       <c r="A2372" t="str">
-        <v>Kmu0wctkuxwtc</v>
+        <v>Kmu0wc9ru8mg1</v>
       </c>
       <c r="B2372" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90713,7 +90713,7 @@
     </row>
     <row r="2373">
       <c r="A2373" t="str">
-        <v>Kmu0wctku1aj5</v>
+        <v>Kmu0wc9ru9mxp</v>
       </c>
       <c r="B2373" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90789,7 +90789,7 @@
     </row>
     <row r="2375">
       <c r="A2375" t="str">
-        <v>Kmu0wctkulapv</v>
+        <v>Kmu0wc9ruap80</v>
       </c>
       <c r="B2375" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90827,7 +90827,7 @@
     </row>
     <row r="2376">
       <c r="A2376" t="str">
-        <v>Kmu0wctkua9f5</v>
+        <v>Kmu0wc9rulse5</v>
       </c>
       <c r="B2376" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90865,7 +90865,7 @@
     </row>
     <row r="2377">
       <c r="A2377" t="str">
-        <v>Kmu0wctku1y6e</v>
+        <v>Kmu0wc9ruw931</v>
       </c>
       <c r="B2377" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90903,7 +90903,7 @@
     </row>
     <row r="2378">
       <c r="A2378" t="str">
-        <v>Kmu0wctkuu8za</v>
+        <v>Kmu0wc9ru3o2j</v>
       </c>
       <c r="B2378" t="str">
         <v xml:space="preserve">Analis Pembiayaan Risiko dan Keuangan/ Analis Keuangan Negara Ahli Utama									</v>

</xml_diff>

<commit_message>
Perbarui struktur organisasi (2026-09-17T22:58:32.866Z)
</commit_message>
<xml_diff>
--- a/data/struktur-organisasi.xlsx
+++ b/data/struktur-organisasi.xlsx
@@ -78173,7 +78173,7 @@
     </row>
     <row r="2043">
       <c r="A2043" t="str">
-        <v>Kmu0wc9rujtz8</v>
+        <v>Kmu64rl7bcjz5</v>
       </c>
       <c r="B2043" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78211,7 +78211,7 @@
     </row>
     <row r="2044">
       <c r="A2044" t="str">
-        <v>Kmu0wc9rurj0c</v>
+        <v>Kmu64rl7bf34p</v>
       </c>
       <c r="B2044" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78249,7 +78249,7 @@
     </row>
     <row r="2045">
       <c r="A2045" t="str">
-        <v>Kmu0wc9ruwu2e</v>
+        <v>Kmu64rl7byrer</v>
       </c>
       <c r="B2045" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78325,7 +78325,7 @@
     </row>
     <row r="2047">
       <c r="A2047" t="str">
-        <v>Kmu0wc9ruod1l</v>
+        <v>Kmu64rl7b2pep</v>
       </c>
       <c r="B2047" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78363,7 +78363,7 @@
     </row>
     <row r="2048">
       <c r="A2048" t="str">
-        <v>Kmu0wc9rucmzi</v>
+        <v>Kmu64rl7b4jai</v>
       </c>
       <c r="B2048" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78401,7 +78401,7 @@
     </row>
     <row r="2049">
       <c r="A2049" t="str">
-        <v>Kmu0wc9rukc1y</v>
+        <v>Kmu64rl7bqkpr</v>
       </c>
       <c r="B2049" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78477,7 +78477,7 @@
     </row>
     <row r="2051">
       <c r="A2051" t="str">
-        <v>Kmu0wc9rukb73</v>
+        <v>Kmu64rl7bd874</v>
       </c>
       <c r="B2051" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78515,7 +78515,7 @@
     </row>
     <row r="2052">
       <c r="A2052" t="str">
-        <v>Kmu0wc9ru2erp</v>
+        <v>Kmu64rl7blxj6</v>
       </c>
       <c r="B2052" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78553,7 +78553,7 @@
     </row>
     <row r="2053">
       <c r="A2053" t="str">
-        <v>Kmu0wc9rumrxv</v>
+        <v>Kmu64rl7b5ig8</v>
       </c>
       <c r="B2053" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78591,7 +78591,7 @@
     </row>
     <row r="2054">
       <c r="A2054" t="str">
-        <v>Kmu0wc9ru36sx</v>
+        <v>Kmu64rl7bktr7</v>
       </c>
       <c r="B2054" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -78629,7 +78629,7 @@
     </row>
     <row r="2055">
       <c r="A2055" t="str">
-        <v>Kmu0wc9ruh4wk</v>
+        <v>Kmu64rl7bo159</v>
       </c>
       <c r="B2055" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -78667,7 +78667,7 @@
     </row>
     <row r="2056">
       <c r="A2056" t="str">
-        <v>Kmu0wc9ruop4g</v>
+        <v>Kmu64rl7bdypz</v>
       </c>
       <c r="B2056" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -78705,7 +78705,7 @@
     </row>
     <row r="2057">
       <c r="A2057" t="str">
-        <v>Kmu0wc9rudmjf</v>
+        <v>Kmu64rl7bqw16</v>
       </c>
       <c r="B2057" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -78743,7 +78743,7 @@
     </row>
     <row r="2058">
       <c r="A2058" t="str">
-        <v>Kmu0wc9ruaog3</v>
+        <v>Kmu64rl7b1xcs</v>
       </c>
       <c r="B2058" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -78857,7 +78857,7 @@
     </row>
     <row r="2061">
       <c r="A2061" t="str">
-        <v>Kmu0wc9rub1os</v>
+        <v>Kmu64rl7b2o5l</v>
       </c>
       <c r="B2061" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78895,7 +78895,7 @@
     </row>
     <row r="2062">
       <c r="A2062" t="str">
-        <v>Kmu0wc9rurhtd</v>
+        <v>Kmu64rl7bju4q</v>
       </c>
       <c r="B2062" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78933,7 +78933,7 @@
     </row>
     <row r="2063">
       <c r="A2063" t="str">
-        <v>Kmu0wc9rux9oj</v>
+        <v>Kmu64rl7b201j</v>
       </c>
       <c r="B2063" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79009,7 +79009,7 @@
     </row>
     <row r="2065">
       <c r="A2065" t="str">
-        <v>Kmu0wc9rurp6m</v>
+        <v>Kmu64rl7b4epn</v>
       </c>
       <c r="B2065" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79047,7 +79047,7 @@
     </row>
     <row r="2066">
       <c r="A2066" t="str">
-        <v>Kmu0wc9ru2ii4</v>
+        <v>Kmu64rl7byc55</v>
       </c>
       <c r="B2066" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79085,7 +79085,7 @@
     </row>
     <row r="2067">
       <c r="A2067" t="str">
-        <v>Kmu0wc9ruc4bl</v>
+        <v>Kmu64rl7byo2q</v>
       </c>
       <c r="B2067" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79161,7 +79161,7 @@
     </row>
     <row r="2069">
       <c r="A2069" t="str">
-        <v>Kmu0wc9rut1u3</v>
+        <v>Kmu64rl7bjzu2</v>
       </c>
       <c r="B2069" t="str">
         <v>Penata Layanan Operasional</v>
@@ -79199,7 +79199,7 @@
     </row>
     <row r="2070">
       <c r="A2070" t="str">
-        <v>Kmu0wc9ru3b47</v>
+        <v>Kmu64rl7bqpyb</v>
       </c>
       <c r="B2070" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79237,7 +79237,7 @@
     </row>
     <row r="2071">
       <c r="A2071" t="str">
-        <v>Kmu0wc9ru6id1</v>
+        <v>Kmu64rl7bsi1h</v>
       </c>
       <c r="B2071" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79313,7 +79313,7 @@
     </row>
     <row r="2073">
       <c r="A2073" t="str">
-        <v>Kmu0wc9rurmhg</v>
+        <v>Kmu64rl7bces6</v>
       </c>
       <c r="B2073" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79351,7 +79351,7 @@
     </row>
     <row r="2074">
       <c r="A2074" t="str">
-        <v>Kmu0wc9ruwvh6</v>
+        <v>Kmu64rl7b2gv4</v>
       </c>
       <c r="B2074" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79389,7 +79389,7 @@
     </row>
     <row r="2075">
       <c r="A2075" t="str">
-        <v>Kmu0wc9ru1un0</v>
+        <v>Kmu64rl7b3c3z</v>
       </c>
       <c r="B2075" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79427,7 +79427,7 @@
     </row>
     <row r="2076">
       <c r="A2076" t="str">
-        <v>Kmu0wc9rutg9r</v>
+        <v>Kmu64rl7bv8hm</v>
       </c>
       <c r="B2076" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -79465,7 +79465,7 @@
     </row>
     <row r="2077">
       <c r="A2077" t="str">
-        <v>Kmu0wc9ruohwg</v>
+        <v>Kmu64rl7b7fby</v>
       </c>
       <c r="B2077" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -79503,7 +79503,7 @@
     </row>
     <row r="2078">
       <c r="A2078" t="str">
-        <v>Kmu0wc9ruc7fx</v>
+        <v>Kmu64rl7btjrm</v>
       </c>
       <c r="B2078" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -79541,7 +79541,7 @@
     </row>
     <row r="2079">
       <c r="A2079" t="str">
-        <v>Kmu0wc9ruc4gy</v>
+        <v>Kmu64rl7bx9u9</v>
       </c>
       <c r="B2079" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -79579,7 +79579,7 @@
     </row>
     <row r="2080">
       <c r="A2080" t="str">
-        <v>Kmu0wc9rud74o</v>
+        <v>Kmu64rl7b55es</v>
       </c>
       <c r="B2080" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -79617,7 +79617,7 @@
     </row>
     <row r="2081">
       <c r="A2081" t="str">
-        <v>Kmu0wc9ruuunp</v>
+        <v>Kmu64rl7bumxl</v>
       </c>
       <c r="B2081" t="str">
         <v>Asesor SDM Aparatur Ahli Muda</v>
@@ -79655,7 +79655,7 @@
     </row>
     <row r="2082">
       <c r="A2082" t="str">
-        <v>Kmu0wc9rum6o5</v>
+        <v>Kmu64rl7b7fbz</v>
       </c>
       <c r="B2082" t="str">
         <v>Asesor SDM Aparatur Ahli Pertama</v>
@@ -79769,7 +79769,7 @@
     </row>
     <row r="2085">
       <c r="A2085" t="str">
-        <v>Kmu0wc9rush9e</v>
+        <v>Kmu64rl7bleij</v>
       </c>
       <c r="B2085" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79807,7 +79807,7 @@
     </row>
     <row r="2086">
       <c r="A2086" t="str">
-        <v>Kmu0wc9rux0n8</v>
+        <v>Kmu64rl7bbt3o</v>
       </c>
       <c r="B2086" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79845,7 +79845,7 @@
     </row>
     <row r="2087">
       <c r="A2087" t="str">
-        <v>Kmu0wc9ruxcqv</v>
+        <v>Kmu64rl7b1yfz</v>
       </c>
       <c r="B2087" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79921,7 +79921,7 @@
     </row>
     <row r="2089">
       <c r="A2089" t="str">
-        <v>Kmu0wc9runxdu</v>
+        <v>Kmu64rl7boxig</v>
       </c>
       <c r="B2089" t="str">
         <v>Penata Layanan Operasional</v>
@@ -79959,7 +79959,7 @@
     </row>
     <row r="2090">
       <c r="A2090" t="str">
-        <v>Kmu0wc9ruoo8b</v>
+        <v>Kmu64rl7bc170</v>
       </c>
       <c r="B2090" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79997,7 +79997,7 @@
     </row>
     <row r="2091">
       <c r="A2091" t="str">
-        <v>Kmu0wc9rubs9x</v>
+        <v>Kmu64rl7boudc</v>
       </c>
       <c r="B2091" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80073,7 +80073,7 @@
     </row>
     <row r="2093">
       <c r="A2093" t="str">
-        <v>Kmu0wc9rurwkl</v>
+        <v>Kmu64rl7bmgr8</v>
       </c>
       <c r="B2093" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80111,7 +80111,7 @@
     </row>
     <row r="2094">
       <c r="A2094" t="str">
-        <v>Kmu0wc9runpak</v>
+        <v>Kmu64rl7bizah</v>
       </c>
       <c r="B2094" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80149,7 +80149,7 @@
     </row>
     <row r="2095">
       <c r="A2095" t="str">
-        <v>Kmu0wc9ruy6vs</v>
+        <v>Kmu64rl7bgqku</v>
       </c>
       <c r="B2095" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80187,7 +80187,7 @@
     </row>
     <row r="2096">
       <c r="A2096" t="str">
-        <v>Kmu0wc9ruiljc</v>
+        <v>Kmu64rl7bbnb5</v>
       </c>
       <c r="B2096" t="str">
         <v>Analis Anggaran Ahli Pertama/ Analis Keuangan Negara Ahli Pertama</v>
@@ -80225,7 +80225,7 @@
     </row>
     <row r="2097">
       <c r="A2097" t="str">
-        <v>Kmu0wc9rucclj</v>
+        <v>Kmu64rl7b8k7o</v>
       </c>
       <c r="B2097" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Muda/Pengawas Keuangan Negara Ahli Muda</v>
@@ -80263,7 +80263,7 @@
     </row>
     <row r="2098">
       <c r="A2098" t="str">
-        <v>Kmu0wc9ru291j</v>
+        <v>Kmu64rl7bu4xy</v>
       </c>
       <c r="B2098" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Pertama/Pengawas Keuangan Negara Ahli Pertama</v>
@@ -80301,7 +80301,7 @@
     </row>
     <row r="2099">
       <c r="A2099" t="str">
-        <v>Kmu0wc9ruqjyi</v>
+        <v>Kmu64rl7bfebd</v>
       </c>
       <c r="B2099" t="str">
         <v>Pranata Keuangan APBN Penyelia/Pengawas Keuangan Negara Penyelia</v>
@@ -80339,7 +80339,7 @@
     </row>
     <row r="2100">
       <c r="A2100" t="str">
-        <v>Kmu0wc9run9o5</v>
+        <v>Kmu64rl7b8b9z</v>
       </c>
       <c r="B2100" t="str">
         <v>Pranata Keuangan APBN Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -80377,7 +80377,7 @@
     </row>
     <row r="2101">
       <c r="A2101" t="str">
-        <v>Kmu0wc9rubjuf</v>
+        <v>Kmu64rl7b4bbc</v>
       </c>
       <c r="B2101" t="str">
         <v>Pranata Keuangan APBN Terampil/Pengawas Keuangan Negara Terampil</v>
@@ -80415,7 +80415,7 @@
     </row>
     <row r="2102">
       <c r="A2102" t="str">
-        <v>Kmu0wc9ruvjf0</v>
+        <v>Kmu64rl7bqyeq</v>
       </c>
       <c r="B2102" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -80453,7 +80453,7 @@
     </row>
     <row r="2103">
       <c r="A2103" t="str">
-        <v>Kmu0wc9rulp9r</v>
+        <v>Kmu64rl7bzjyq</v>
       </c>
       <c r="B2103" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -80491,7 +80491,7 @@
     </row>
     <row r="2104">
       <c r="A2104" t="str">
-        <v>Kmu0wc9ru0do7</v>
+        <v>Kmu64rl7b6ngw</v>
       </c>
       <c r="B2104" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -80529,7 +80529,7 @@
     </row>
     <row r="2105">
       <c r="A2105" t="str">
-        <v>Kmu0wc9ru39s5</v>
+        <v>Kmu64rl7bd2qm</v>
       </c>
       <c r="B2105" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -80567,7 +80567,7 @@
     </row>
     <row r="2106">
       <c r="A2106" t="str">
-        <v>Kmu0wc9ru4u0k</v>
+        <v>Kmu64rl7b7mqa</v>
       </c>
       <c r="B2106" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -80681,7 +80681,7 @@
     </row>
     <row r="2109">
       <c r="A2109" t="str">
-        <v>Kmu0wc9rupb4c</v>
+        <v>Kmu64rl7bhdas</v>
       </c>
       <c r="B2109" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80719,7 +80719,7 @@
     </row>
     <row r="2110">
       <c r="A2110" t="str">
-        <v>Kmu0wc9ruk9lg</v>
+        <v>Kmu64rl7bbldq</v>
       </c>
       <c r="B2110" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80757,7 +80757,7 @@
     </row>
     <row r="2111">
       <c r="A2111" t="str">
-        <v>Kmu0wc9runahm</v>
+        <v>Kmu64rl7b24gt</v>
       </c>
       <c r="B2111" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80833,7 +80833,7 @@
     </row>
     <row r="2113">
       <c r="A2113" t="str">
-        <v>Kmu0wc9ruqt1d</v>
+        <v>Kmu64rl7b3zq9</v>
       </c>
       <c r="B2113" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80871,7 +80871,7 @@
     </row>
     <row r="2114">
       <c r="A2114" t="str">
-        <v>Kmu0wc9ru9y1a</v>
+        <v>Kmu64rl7b9ltw</v>
       </c>
       <c r="B2114" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80909,7 +80909,7 @@
     </row>
     <row r="2115">
       <c r="A2115" t="str">
-        <v>Kmu0wc9ru6vz1</v>
+        <v>Kmu64rl7b18x5</v>
       </c>
       <c r="B2115" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80985,7 +80985,7 @@
     </row>
     <row r="2117">
       <c r="A2117" t="str">
-        <v>Kmu0wc9run32d</v>
+        <v>Kmu64rl7b1l86</v>
       </c>
       <c r="B2117" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -81023,7 +81023,7 @@
     </row>
     <row r="2118">
       <c r="A2118" t="str">
-        <v>Kmu0wc9ruej1a</v>
+        <v>Kmu64rl7b0szt</v>
       </c>
       <c r="B2118" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81061,7 +81061,7 @@
     </row>
     <row r="2119">
       <c r="A2119" t="str">
-        <v>Kmu0wc9ruvivi</v>
+        <v>Kmu64rl7bpexk</v>
       </c>
       <c r="B2119" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81099,7 +81099,7 @@
     </row>
     <row r="2120">
       <c r="A2120" t="str">
-        <v>Kmu0wc9rufkc7</v>
+        <v>Kmu64rl7btq6t</v>
       </c>
       <c r="B2120" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -81137,7 +81137,7 @@
     </row>
     <row r="2121">
       <c r="A2121" t="str">
-        <v>Kmu0wc9rutr7z</v>
+        <v>Kmu64rl7bk2c3</v>
       </c>
       <c r="B2121" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -81175,7 +81175,7 @@
     </row>
     <row r="2122">
       <c r="A2122" t="str">
-        <v>Kmu0wc9rubeqs</v>
+        <v>Kmu64rl7bxt1k</v>
       </c>
       <c r="B2122" t="str">
         <v>Pengawas Keuangan Negara Mahir</v>
@@ -81213,7 +81213,7 @@
     </row>
     <row r="2123">
       <c r="A2123" t="str">
-        <v>Kmu0wc9ruxicw</v>
+        <v>Kmu64rl7bqtyg</v>
       </c>
       <c r="B2123" t="str">
         <v>Pengawas Keuangan Negara Terampil</v>
@@ -81327,7 +81327,7 @@
     </row>
     <row r="2126">
       <c r="A2126" t="str">
-        <v>Kmu0wc9ruta9e</v>
+        <v>Kmu64rl7btjnr</v>
       </c>
       <c r="B2126" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81365,7 +81365,7 @@
     </row>
     <row r="2127">
       <c r="A2127" t="str">
-        <v>Kmu0wc9ruuldg</v>
+        <v>Kmu64rl7bf0c7</v>
       </c>
       <c r="B2127" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81403,7 +81403,7 @@
     </row>
     <row r="2128">
       <c r="A2128" t="str">
-        <v>Kmu0wc9rub4xn</v>
+        <v>Kmu64rl7b9cu2</v>
       </c>
       <c r="B2128" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81441,7 +81441,7 @@
     </row>
     <row r="2129">
       <c r="A2129" t="str">
-        <v>Kmu0wc9rugesh</v>
+        <v>Kmu64rl7bwolg</v>
       </c>
       <c r="B2129" t="str">
         <v>Penata Keprotokolan*</v>
@@ -81517,7 +81517,7 @@
     </row>
     <row r="2131">
       <c r="A2131" t="str">
-        <v>Kmu0wc9ruk3kr</v>
+        <v>Kmu64rl7bjua6</v>
       </c>
       <c r="B2131" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81555,7 +81555,7 @@
     </row>
     <row r="2132">
       <c r="A2132" t="str">
-        <v>Kmu0wc9ruwju1</v>
+        <v>Kmu64rl7bng2s</v>
       </c>
       <c r="B2132" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81593,7 +81593,7 @@
     </row>
     <row r="2133">
       <c r="A2133" t="str">
-        <v>Kmu0wc9ruh84t</v>
+        <v>Kmu64rl7bsesi</v>
       </c>
       <c r="B2133" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81631,7 +81631,7 @@
     </row>
     <row r="2134">
       <c r="A2134" t="str">
-        <v>Kmu0wc9ru8mam</v>
+        <v>Kmu64rl7bueq4</v>
       </c>
       <c r="B2134" t="str">
         <v>Penata Keprotokolan*</v>
@@ -81707,7 +81707,7 @@
     </row>
     <row r="2136">
       <c r="A2136" t="str">
-        <v>Kmu0wc9ru5hk3</v>
+        <v>Kmu64rl7buzfk</v>
       </c>
       <c r="B2136" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81745,7 +81745,7 @@
     </row>
     <row r="2137">
       <c r="A2137" t="str">
-        <v>Kmu0wc9ruoivv</v>
+        <v>Kmu64rl7bpjju</v>
       </c>
       <c r="B2137" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81783,7 +81783,7 @@
     </row>
     <row r="2138">
       <c r="A2138" t="str">
-        <v>Kmu0wc9rujql5</v>
+        <v>Kmu64rl7bjryw</v>
       </c>
       <c r="B2138" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81821,7 +81821,7 @@
     </row>
     <row r="2139">
       <c r="A2139" t="str">
-        <v>Kmu0wc9rux86x</v>
+        <v>Kmu64rl7b9kzm</v>
       </c>
       <c r="B2139" t="str">
         <v>Pengawas Keuangan Negara Ahli Muda</v>
@@ -81859,7 +81859,7 @@
     </row>
     <row r="2140">
       <c r="A2140" t="str">
-        <v>Kmu0wc9rupac2</v>
+        <v>Kmu64rl7bhijz</v>
       </c>
       <c r="B2140" t="str">
         <v>Pengawas Keuangan Negara Pertama</v>
@@ -81897,7 +81897,7 @@
     </row>
     <row r="2141">
       <c r="A2141" t="str">
-        <v>Kmu0wc9rufl0v</v>
+        <v>Kmu64rl7bvit2</v>
       </c>
       <c r="B2141" t="str">
         <v>Penata Laksana Barang Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -81935,7 +81935,7 @@
     </row>
     <row r="2142">
       <c r="A2142" t="str">
-        <v>Kmu0wc9ru6yl5</v>
+        <v>Kmu64rl7bmii7</v>
       </c>
       <c r="B2142" t="str">
         <v>Penata Laksana Barang Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -81973,7 +81973,7 @@
     </row>
     <row r="2143">
       <c r="A2143" t="str">
-        <v>Kmu0wc9ru6h6t</v>
+        <v>Kmu64rl7bk8am</v>
       </c>
       <c r="B2143" t="str">
         <v>Penata Laksana Barang Terampil/ Pengawas Keuangan Negara Terampil</v>
@@ -82011,7 +82011,7 @@
     </row>
     <row r="2144">
       <c r="A2144" t="str">
-        <v>Kmu0wc9rujgyg</v>
+        <v>Kmu64rl7bfpy2</v>
       </c>
       <c r="B2144" t="str">
         <v>Arsiparis Ahli Muda</v>
@@ -82049,7 +82049,7 @@
     </row>
     <row r="2145">
       <c r="A2145" t="str">
-        <v>Kmu0wc9ru1z8y</v>
+        <v>Kmu64rl7bqif6</v>
       </c>
       <c r="B2145" t="str">
         <v>Arsiparis Ahli Pertama</v>
@@ -82087,7 +82087,7 @@
     </row>
     <row r="2146">
       <c r="A2146" t="str">
-        <v>Kmu0wc9rujrfi</v>
+        <v>Kmu64rl7bdowj</v>
       </c>
       <c r="B2146" t="str">
         <v>Arsiparis Penyelia</v>
@@ -82125,7 +82125,7 @@
     </row>
     <row r="2147">
       <c r="A2147" t="str">
-        <v>Kmu0wc9rui5es</v>
+        <v>Kmu64rl7bmp5f</v>
       </c>
       <c r="B2147" t="str">
         <v>Arsiparis Mahir</v>
@@ -82163,7 +82163,7 @@
     </row>
     <row r="2148">
       <c r="A2148" t="str">
-        <v>Kmu0wc9ruk2fd</v>
+        <v>Kmu64rl7btolr</v>
       </c>
       <c r="B2148" t="str">
         <v>Arsiparis Terampil</v>
@@ -82277,7 +82277,7 @@
     </row>
     <row r="2151">
       <c r="A2151" t="str">
-        <v>Kmu0wc9ru0hse</v>
+        <v>Kmu64rl7bsotk</v>
       </c>
       <c r="B2151" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -82315,7 +82315,7 @@
     </row>
     <row r="2152">
       <c r="A2152" t="str">
-        <v>Kmu0wc9ru2vrj</v>
+        <v>Kmu64rl7bgw9y</v>
       </c>
       <c r="B2152" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82353,7 +82353,7 @@
     </row>
     <row r="2153">
       <c r="A2153" t="str">
-        <v>Kmu0wc9ruxlqp</v>
+        <v>Kmu64rl7bl04x</v>
       </c>
       <c r="B2153" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82391,7 +82391,7 @@
     </row>
     <row r="2154">
       <c r="A2154" t="str">
-        <v>Kmu0wc9ruwk5t</v>
+        <v>Kmu64rl7b4gki</v>
       </c>
       <c r="B2154" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -82429,7 +82429,7 @@
     </row>
     <row r="2155">
       <c r="A2155" t="str">
-        <v>Kmu0wc9ruhjw7</v>
+        <v>Kmu64rl7ber81</v>
       </c>
       <c r="B2155" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -82467,7 +82467,7 @@
     </row>
     <row r="2156">
       <c r="A2156" t="str">
-        <v>Kmu0wc9ruwu98</v>
+        <v>Kmu64rl7b1iy7</v>
       </c>
       <c r="B2156" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -82505,7 +82505,7 @@
     </row>
     <row r="2157">
       <c r="A2157" t="str">
-        <v>Kmu0wc9ruay2u</v>
+        <v>Kmu64rl7bsowy</v>
       </c>
       <c r="B2157" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -82581,7 +82581,7 @@
     </row>
     <row r="2159">
       <c r="A2159" t="str">
-        <v>Kmu0wc9ruw0s3</v>
+        <v>Kmu64rl7bdkj6</v>
       </c>
       <c r="B2159" t="str">
         <v>Penata Layanan Operasional</v>
@@ -82619,7 +82619,7 @@
     </row>
     <row r="2160">
       <c r="A2160" t="str">
-        <v>Kmu0wc9ruszwr</v>
+        <v>Kmu64rl7bpywj</v>
       </c>
       <c r="B2160" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82657,7 +82657,7 @@
     </row>
     <row r="2161">
       <c r="A2161" t="str">
-        <v>Kmu0wc9ru3ntx</v>
+        <v>Kmu64rl7bngn4</v>
       </c>
       <c r="B2161" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82695,7 +82695,7 @@
     </row>
     <row r="2162">
       <c r="A2162" t="str">
-        <v>Kmu0wc9rullsh</v>
+        <v>Kmu64rl7bumwn</v>
       </c>
       <c r="B2162" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -82733,7 +82733,7 @@
     </row>
     <row r="2163">
       <c r="A2163" t="str">
-        <v>Kmu0wc9ruvc4p</v>
+        <v>Kmu64rl7b9ioh</v>
       </c>
       <c r="B2163" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -82771,7 +82771,7 @@
     </row>
     <row r="2164">
       <c r="A2164" t="str">
-        <v>Kmu0wc9rue7vo</v>
+        <v>Kmu64rl7bsitf</v>
       </c>
       <c r="B2164" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -82809,7 +82809,7 @@
     </row>
     <row r="2165">
       <c r="A2165" t="str">
-        <v>Kmu0wc9rua65j</v>
+        <v>Kmu64rl7bltd0</v>
       </c>
       <c r="B2165" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -82885,7 +82885,7 @@
     </row>
     <row r="2167">
       <c r="A2167" t="str">
-        <v>Kmu0wc9ru7co1</v>
+        <v>Kmu64rl7bdv09</v>
       </c>
       <c r="B2167" t="str">
         <v>Penata Layanan Operasional</v>
@@ -82923,7 +82923,7 @@
     </row>
     <row r="2168">
       <c r="A2168" t="str">
-        <v>Kmu0wc9rulfm3</v>
+        <v>Kmu64rl7bj4cw</v>
       </c>
       <c r="B2168" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82961,7 +82961,7 @@
     </row>
     <row r="2169">
       <c r="A2169" t="str">
-        <v>Kmu0wc9rusa9q</v>
+        <v>Kmu64rl7b5z4z</v>
       </c>
       <c r="B2169" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82999,7 +82999,7 @@
     </row>
     <row r="2170">
       <c r="A2170" t="str">
-        <v>Kmu0wc9ruql77</v>
+        <v>Kmu64rl7bo9p9</v>
       </c>
       <c r="B2170" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -83037,7 +83037,7 @@
     </row>
     <row r="2171">
       <c r="A2171" t="str">
-        <v>Kmu0wc9ruhyq3</v>
+        <v>Kmu64rl7bio04</v>
       </c>
       <c r="B2171" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -83075,7 +83075,7 @@
     </row>
     <row r="2172">
       <c r="A2172" t="str">
-        <v>Kmu0wc9ru4r7f</v>
+        <v>Kmu64rl7bg7xt</v>
       </c>
       <c r="B2172" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -83113,7 +83113,7 @@
     </row>
     <row r="2173">
       <c r="A2173" t="str">
-        <v>Kmu0wc9rux1u2</v>
+        <v>Kmu64rl7bpgc4</v>
       </c>
       <c r="B2173" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -83151,7 +83151,7 @@
     </row>
     <row r="2174">
       <c r="A2174" t="str">
-        <v>Kmu0wc9ru73d3</v>
+        <v>Kmu64rl7b8y4v</v>
       </c>
       <c r="B2174" t="str">
         <v>Pranata Humas Ahli Muda</v>
@@ -83189,7 +83189,7 @@
     </row>
     <row r="2175">
       <c r="A2175" t="str">
-        <v>Kmu0wc9ruv2gf</v>
+        <v>Kmu64rl7bfyqd</v>
       </c>
       <c r="B2175" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -83227,7 +83227,7 @@
     </row>
     <row r="2176">
       <c r="A2176" t="str">
-        <v>Kmu0wc9rucj6l</v>
+        <v>Kmu64rl7b2wzo</v>
       </c>
       <c r="B2176" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -83265,7 +83265,7 @@
     </row>
     <row r="2177">
       <c r="A2177" t="str">
-        <v>Kmu0wc9ruapk4</v>
+        <v>Kmu64rl7br4yx</v>
       </c>
       <c r="B2177" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -83303,7 +83303,7 @@
     </row>
     <row r="2178">
       <c r="A2178" t="str">
-        <v>Kmu0wc9ruhg37</v>
+        <v>Kmu64rl7b4nt7</v>
       </c>
       <c r="B2178" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -83341,7 +83341,7 @@
     </row>
     <row r="2179">
       <c r="A2179" t="str">
-        <v>Kmu0wc9ru6w84</v>
+        <v>Kmu64rl7bsikk</v>
       </c>
       <c r="B2179" t="str">
         <v>Pustakawan Ahli Pertama</v>
@@ -83379,7 +83379,7 @@
     </row>
     <row r="2180">
       <c r="A2180" t="str">
-        <v>Kmu0wc9rujt7h</v>
+        <v>Kmu64rl7b9qfd</v>
       </c>
       <c r="B2180" t="str">
         <v>Asisten Perpustakaan Penyelia</v>
@@ -83417,7 +83417,7 @@
     </row>
     <row r="2181">
       <c r="A2181" t="str">
-        <v>Kmu0wc9ru4ati</v>
+        <v>Kmu64rl7b282w</v>
       </c>
       <c r="B2181" t="str">
         <v>Asisten Perpustakaan Mahir</v>
@@ -83455,7 +83455,7 @@
     </row>
     <row r="2182">
       <c r="A2182" t="str">
-        <v>Kmu0wc9ruvw2x</v>
+        <v>Kmu64rl7b77fj</v>
       </c>
       <c r="B2182" t="str">
         <v>Asisten Perpustakaan Terampil</v>
@@ -83493,7 +83493,7 @@
     </row>
     <row r="2183">
       <c r="A2183" t="str">
-        <v>Kmu0wc9rusees</v>
+        <v>Kmu64rl7b5eaw</v>
       </c>
       <c r="B2183" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Madya/Pengawas Keuangan Negara Ahli Madya</v>
@@ -83531,7 +83531,7 @@
     </row>
     <row r="2184">
       <c r="A2184" t="str">
-        <v>Kmu0wc9ruq480</v>
+        <v>Kmu64rl7b4xxl</v>
       </c>
       <c r="B2184" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Muda</v>
@@ -83569,7 +83569,7 @@
     </row>
     <row r="2185">
       <c r="A2185" t="str">
-        <v>Kmu0wc9ruo539</v>
+        <v>Kmu64rl7bdo0l</v>
       </c>
       <c r="B2185" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Pertama</v>
@@ -83683,7 +83683,7 @@
     </row>
     <row r="2188">
       <c r="A2188" t="str">
-        <v>Kmu0wc9rupbu9</v>
+        <v>Kmu64rl7cgvre</v>
       </c>
       <c r="B2188" t="str">
         <v>Penata Layanan Operasional</v>
@@ -83721,7 +83721,7 @@
     </row>
     <row r="2189">
       <c r="A2189" t="str">
-        <v>Kmu0wc9ru4yf6</v>
+        <v>Kmu64rl7ckpv1</v>
       </c>
       <c r="B2189" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -83759,7 +83759,7 @@
     </row>
     <row r="2190">
       <c r="A2190" t="str">
-        <v>Kmu0wc9ruzhbh</v>
+        <v>Kmu64rl7cyz0t</v>
       </c>
       <c r="B2190" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -83797,7 +83797,7 @@
     </row>
     <row r="2191">
       <c r="A2191" t="str">
-        <v>Kmu0wc9ruqhnl</v>
+        <v>Kmu64rl7ce0zs</v>
       </c>
       <c r="B2191" t="str">
         <v>Penata Keprotokolan*</v>
@@ -83911,7 +83911,7 @@
     </row>
     <row r="2194">
       <c r="A2194" t="str">
-        <v>Kmu0wc9ru5uf6</v>
+        <v>Kmu64rl7c5lwj</v>
       </c>
       <c r="B2194" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -83949,7 +83949,7 @@
     </row>
     <row r="2195">
       <c r="A2195" t="str">
-        <v>Kmu0wc9rufx21</v>
+        <v>Kmu64rl7cs3fu</v>
       </c>
       <c r="B2195" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -83987,7 +83987,7 @@
     </row>
     <row r="2196">
       <c r="A2196" t="str">
-        <v>Kmu0wc9rugbpu</v>
+        <v>Kmu64rl7ce071</v>
       </c>
       <c r="B2196" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84063,7 +84063,7 @@
     </row>
     <row r="2198">
       <c r="A2198" t="str">
-        <v>Kmu0wc9ru78oz</v>
+        <v>Kmu64rl7caf3n</v>
       </c>
       <c r="B2198" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84101,7 +84101,7 @@
     </row>
     <row r="2199">
       <c r="A2199" t="str">
-        <v>Kmu0wc9ruii9t</v>
+        <v>Kmu64rl7cqeo8</v>
       </c>
       <c r="B2199" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84139,7 +84139,7 @@
     </row>
     <row r="2200">
       <c r="A2200" t="str">
-        <v>Kmu0wc9ru6e2j</v>
+        <v>Kmu64rl7cqxg5</v>
       </c>
       <c r="B2200" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84177,7 +84177,7 @@
     </row>
     <row r="2201">
       <c r="A2201" t="str">
-        <v>Kmu0wc9ru1zwr</v>
+        <v>Kmu64rl7covyf</v>
       </c>
       <c r="B2201" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -84215,7 +84215,7 @@
     </row>
     <row r="2202">
       <c r="A2202" t="str">
-        <v>Kmu0wc9rukf2l</v>
+        <v>Kmu64rl7cpy8u</v>
       </c>
       <c r="B2202" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -84253,7 +84253,7 @@
     </row>
     <row r="2203">
       <c r="A2203" t="str">
-        <v>Kmu0wc9ruf7p4</v>
+        <v>Kmu64rl7c10lg</v>
       </c>
       <c r="B2203" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -84291,7 +84291,7 @@
     </row>
     <row r="2204">
       <c r="A2204" t="str">
-        <v>Kmu0wc9ruwwjv</v>
+        <v>Kmu64rl7cn4h3</v>
       </c>
       <c r="B2204" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -84405,7 +84405,7 @@
     </row>
     <row r="2207">
       <c r="A2207" t="str">
-        <v>Kmu0wc9ruj4my</v>
+        <v>Kmu64rl7cyero</v>
       </c>
       <c r="B2207" t="str">
         <v>Penata Layanan Operasional</v>
@@ -84443,7 +84443,7 @@
     </row>
     <row r="2208">
       <c r="A2208" t="str">
-        <v>Kmu0wc9rutwo3</v>
+        <v>Kmu64rl7c7h1y</v>
       </c>
       <c r="B2208" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84481,7 +84481,7 @@
     </row>
     <row r="2209">
       <c r="A2209" t="str">
-        <v>Kmu0wc9run1p7</v>
+        <v>Kmu64rl7c0ale</v>
       </c>
       <c r="B2209" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84519,7 +84519,7 @@
     </row>
     <row r="2210">
       <c r="A2210" t="str">
-        <v>Kmu0wc9run2i1</v>
+        <v>Kmu64rl7ccpqs</v>
       </c>
       <c r="B2210" t="str">
         <v>Penata Keprotokolan*</v>
@@ -84633,7 +84633,7 @@
     </row>
     <row r="2213">
       <c r="A2213" t="str">
-        <v>Kmu0wc9ruo11r</v>
+        <v>Kmu64rl7crall</v>
       </c>
       <c r="B2213" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84671,7 +84671,7 @@
     </row>
     <row r="2214">
       <c r="A2214" t="str">
-        <v>Kmu0wc9ru9cwp</v>
+        <v>Kmu64rl7c8qlc</v>
       </c>
       <c r="B2214" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84709,7 +84709,7 @@
     </row>
     <row r="2215">
       <c r="A2215" t="str">
-        <v>Kmu0wc9ruf0fx</v>
+        <v>Kmu64rl7c4f6s</v>
       </c>
       <c r="B2215" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84785,7 +84785,7 @@
     </row>
     <row r="2217">
       <c r="A2217" t="str">
-        <v>Kmu0wc9rups46</v>
+        <v>Kmu64rl7cn8gq</v>
       </c>
       <c r="B2217" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84823,7 +84823,7 @@
     </row>
     <row r="2218">
       <c r="A2218" t="str">
-        <v>Kmu0wc9rui35c</v>
+        <v>Kmu64rl7c24us</v>
       </c>
       <c r="B2218" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84861,7 +84861,7 @@
     </row>
     <row r="2219">
       <c r="A2219" t="str">
-        <v>Kmu0wc9rupgnl</v>
+        <v>Kmu64rl7ckwhv</v>
       </c>
       <c r="B2219" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84899,7 +84899,7 @@
     </row>
     <row r="2220">
       <c r="A2220" t="str">
-        <v>Kmu0wc9rumvz6</v>
+        <v>Kmu64rl7cty0x</v>
       </c>
       <c r="B2220" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -84937,7 +84937,7 @@
     </row>
     <row r="2221">
       <c r="A2221" t="str">
-        <v>Kmu0wc9ru4qtd</v>
+        <v>Kmu64rl7cjkhs</v>
       </c>
       <c r="B2221" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -84975,7 +84975,7 @@
     </row>
     <row r="2222">
       <c r="A2222" t="str">
-        <v>Kmu0wc9ru8hw2</v>
+        <v>Kmu64rl7cmchx</v>
       </c>
       <c r="B2222" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -85013,7 +85013,7 @@
     </row>
     <row r="2223">
       <c r="A2223" t="str">
-        <v>Kmu0wc9rujea9</v>
+        <v>Kmu64rl7crr7d</v>
       </c>
       <c r="B2223" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -85127,7 +85127,7 @@
     </row>
     <row r="2226">
       <c r="A2226" t="str">
-        <v>Kmu0wc9ruere6</v>
+        <v>Kmu64rl7cyz1e</v>
       </c>
       <c r="B2226" t="str">
         <v>Penata Layanan Operasional</v>
@@ -85165,7 +85165,7 @@
     </row>
     <row r="2227">
       <c r="A2227" t="str">
-        <v>Kmu0wc9rusb13</v>
+        <v>Kmu64rl7c8lwf</v>
       </c>
       <c r="B2227" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85203,7 +85203,7 @@
     </row>
     <row r="2228">
       <c r="A2228" t="str">
-        <v>Kmu0wc9rusa7k</v>
+        <v>Kmu64rl7co5dy</v>
       </c>
       <c r="B2228" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85241,7 +85241,7 @@
     </row>
     <row r="2229">
       <c r="A2229" t="str">
-        <v>Kmu0wc9rufx5e</v>
+        <v>Kmu64rl7cyuxy</v>
       </c>
       <c r="B2229" t="str">
         <v>Penata Keprotokolan*</v>
@@ -85355,7 +85355,7 @@
     </row>
     <row r="2232">
       <c r="A2232" t="str">
-        <v>Kmu0wc9ruow77</v>
+        <v>Kmu64rl7cb4r2</v>
       </c>
       <c r="B2232" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -85393,7 +85393,7 @@
     </row>
     <row r="2233">
       <c r="A2233" t="str">
-        <v>Kmu0wc9ru6l55</v>
+        <v>Kmu64rl7ckvsj</v>
       </c>
       <c r="B2233" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85431,7 +85431,7 @@
     </row>
     <row r="2234">
       <c r="A2234" t="str">
-        <v>Kmu0wc9ruvgmk</v>
+        <v>Kmu64rl7cex3q</v>
       </c>
       <c r="B2234" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85507,7 +85507,7 @@
     </row>
     <row r="2236">
       <c r="A2236" t="str">
-        <v>Kmu0wc9ruahgo</v>
+        <v>Kmu64rl7cgdsj</v>
       </c>
       <c r="B2236" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -85545,7 +85545,7 @@
     </row>
     <row r="2237">
       <c r="A2237" t="str">
-        <v>Kmu0wc9rulrcd</v>
+        <v>Kmu64rl7c5lo0</v>
       </c>
       <c r="B2237" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85583,7 +85583,7 @@
     </row>
     <row r="2238">
       <c r="A2238" t="str">
-        <v>Kmu0wc9rupjts</v>
+        <v>Kmu64rl7cels9</v>
       </c>
       <c r="B2238" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85621,7 +85621,7 @@
     </row>
     <row r="2239">
       <c r="A2239" t="str">
-        <v>Kmu0wc9ruf6jj</v>
+        <v>Kmu64rl7c167i</v>
       </c>
       <c r="B2239" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -85659,7 +85659,7 @@
     </row>
     <row r="2240">
       <c r="A2240" t="str">
-        <v>Kmu0wc9ru4ujt</v>
+        <v>Kmu64rl7ccf5n</v>
       </c>
       <c r="B2240" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -85697,7 +85697,7 @@
     </row>
     <row r="2241">
       <c r="A2241" t="str">
-        <v>Kmu0wc9ruyp6k</v>
+        <v>Kmu64rl7cmuks</v>
       </c>
       <c r="B2241" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -85735,7 +85735,7 @@
     </row>
     <row r="2242">
       <c r="A2242" t="str">
-        <v>Kmu0wc9ruvixx</v>
+        <v>Kmu64rl7coxua</v>
       </c>
       <c r="B2242" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -85849,7 +85849,7 @@
     </row>
     <row r="2245">
       <c r="A2245" t="str">
-        <v>Kmu0wc9ru9yow</v>
+        <v>Kmu64rl7c921n</v>
       </c>
       <c r="B2245" t="str">
         <v>Penata Layanan Operasional</v>
@@ -85887,7 +85887,7 @@
     </row>
     <row r="2246">
       <c r="A2246" t="str">
-        <v>Kmu0wc9ru0osn</v>
+        <v>Kmu64rl7c2g7a</v>
       </c>
       <c r="B2246" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85925,7 +85925,7 @@
     </row>
     <row r="2247">
       <c r="A2247" t="str">
-        <v>Kmu0wc9ruy20a</v>
+        <v>Kmu64rl7c3o44</v>
       </c>
       <c r="B2247" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85963,7 +85963,7 @@
     </row>
     <row r="2248">
       <c r="A2248" t="str">
-        <v>Kmu0wc9runcdt</v>
+        <v>Kmu64rl7cn6kn</v>
       </c>
       <c r="B2248" t="str">
         <v>Penata Keprotokolan*</v>
@@ -86039,7 +86039,7 @@
     </row>
     <row r="2250">
       <c r="A2250" t="str">
-        <v>Kmu0wc9ruc30w</v>
+        <v>Kmu64rl7cfalc</v>
       </c>
       <c r="B2250" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86077,7 +86077,7 @@
     </row>
     <row r="2251">
       <c r="A2251" t="str">
-        <v>Kmu0wc9ruqdu8</v>
+        <v>Kmu64rl7ckwju</v>
       </c>
       <c r="B2251" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86115,7 +86115,7 @@
     </row>
     <row r="2252">
       <c r="A2252" t="str">
-        <v>Kmu0wc9ru29tq</v>
+        <v>Kmu64rl7cbknw</v>
       </c>
       <c r="B2252" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86153,7 +86153,7 @@
     </row>
     <row r="2253">
       <c r="A2253" t="str">
-        <v>Kmu0wc9rush4e</v>
+        <v>Kmu64rl7c8i32</v>
       </c>
       <c r="B2253" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -86191,7 +86191,7 @@
     </row>
     <row r="2254">
       <c r="A2254" t="str">
-        <v>Kmu0wc9ru8lbq</v>
+        <v>Kmu64rl7cwkxw</v>
       </c>
       <c r="B2254" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -86305,7 +86305,7 @@
     </row>
     <row r="2257">
       <c r="A2257" t="str">
-        <v>Kmu0wc9ru3xek</v>
+        <v>Kmu64rl7c6pkg</v>
       </c>
       <c r="B2257" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86343,7 +86343,7 @@
     </row>
     <row r="2258">
       <c r="A2258" t="str">
-        <v>Kmu0wc9ruv3mz</v>
+        <v>Kmu64rl7cri5q</v>
       </c>
       <c r="B2258" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86381,7 +86381,7 @@
     </row>
     <row r="2259">
       <c r="A2259" t="str">
-        <v>Kmu0wc9ruhttv</v>
+        <v>Kmu64rl7c0sne</v>
       </c>
       <c r="B2259" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86457,7 +86457,7 @@
     </row>
     <row r="2261">
       <c r="A2261" t="str">
-        <v>Kmu0wc9rug5yk</v>
+        <v>Kmu64rl7ckxu5</v>
       </c>
       <c r="B2261" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86495,7 +86495,7 @@
     </row>
     <row r="2262">
       <c r="A2262" t="str">
-        <v>Kmu0wc9ruo8m4</v>
+        <v>Kmu64rl7c88k3</v>
       </c>
       <c r="B2262" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86533,7 +86533,7 @@
     </row>
     <row r="2263">
       <c r="A2263" t="str">
-        <v>Kmu0wc9rug4zc</v>
+        <v>Kmu64rl7c1wsv</v>
       </c>
       <c r="B2263" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86571,7 +86571,7 @@
     </row>
     <row r="2264">
       <c r="A2264" t="str">
-        <v>Kmu0wc9ru2z7b</v>
+        <v>Kmu64rl7ca16d</v>
       </c>
       <c r="B2264" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -86609,7 +86609,7 @@
     </row>
     <row r="2265">
       <c r="A2265" t="str">
-        <v>Kmu0wc9ru04o2</v>
+        <v>Kmu64rl7cipso</v>
       </c>
       <c r="B2265" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -86647,7 +86647,7 @@
     </row>
     <row r="2266">
       <c r="A2266" t="str">
-        <v>Kmu0wc9ruyjdp</v>
+        <v>Kmu64rl7crr5p</v>
       </c>
       <c r="B2266" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -86685,7 +86685,7 @@
     </row>
     <row r="2267">
       <c r="A2267" t="str">
-        <v>Kmu0wc9ruxl08</v>
+        <v>Kmu64rl7cp2ds</v>
       </c>
       <c r="B2267" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -86799,7 +86799,7 @@
     </row>
     <row r="2270">
       <c r="A2270" t="str">
-        <v>Kmu0wc9ru9xzh</v>
+        <v>Kmu64rl7cqabl</v>
       </c>
       <c r="B2270" t="str">
         <v>Penata Layanan Operasional</v>
@@ -86837,7 +86837,7 @@
     </row>
     <row r="2271">
       <c r="A2271" t="str">
-        <v>Kmu0wc9ruo0tq</v>
+        <v>Kmu64rl7cnj9s</v>
       </c>
       <c r="B2271" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86875,7 +86875,7 @@
     </row>
     <row r="2272">
       <c r="A2272" t="str">
-        <v>Kmu0wc9ruz7ff</v>
+        <v>Kmu64rl7cgoux</v>
       </c>
       <c r="B2272" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86913,7 +86913,7 @@
     </row>
     <row r="2273">
       <c r="A2273" t="str">
-        <v>Kmu0wc9rum4zb</v>
+        <v>Kmu64rl7c0l54</v>
       </c>
       <c r="B2273" t="str">
         <v>Penata Keprotokolan*</v>
@@ -87027,7 +87027,7 @@
     </row>
     <row r="2276">
       <c r="A2276" t="str">
-        <v>Kmu0wc9rusvra</v>
+        <v>Kmu64rl7cdgdl</v>
       </c>
       <c r="B2276" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87065,7 +87065,7 @@
     </row>
     <row r="2277">
       <c r="A2277" t="str">
-        <v>Kmu0wc9rugiqr</v>
+        <v>Kmu64rl7ccobi</v>
       </c>
       <c r="B2277" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87103,7 +87103,7 @@
     </row>
     <row r="2278">
       <c r="A2278" t="str">
-        <v>Kmu0wc9rusnti</v>
+        <v>Kmu64rl7ceiv4</v>
       </c>
       <c r="B2278" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87179,7 +87179,7 @@
     </row>
     <row r="2280">
       <c r="A2280" t="str">
-        <v>Kmu0wc9ruhiq3</v>
+        <v>Kmu64rl7cckld</v>
       </c>
       <c r="B2280" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87217,7 +87217,7 @@
     </row>
     <row r="2281">
       <c r="A2281" t="str">
-        <v>Kmu0wc9rugmn0</v>
+        <v>Kmu64rl7ckhyf</v>
       </c>
       <c r="B2281" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87255,7 +87255,7 @@
     </row>
     <row r="2282">
       <c r="A2282" t="str">
-        <v>Kmu0wc9ruel36</v>
+        <v>Kmu64rl7cz4yj</v>
       </c>
       <c r="B2282" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87293,7 +87293,7 @@
     </row>
     <row r="2283">
       <c r="A2283" t="str">
-        <v>Kmu0wc9rujxf2</v>
+        <v>Kmu64rl7cehvn</v>
       </c>
       <c r="B2283" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -87331,7 +87331,7 @@
     </row>
     <row r="2284">
       <c r="A2284" t="str">
-        <v>Kmu0wc9ru8png</v>
+        <v>Kmu64rl7cmcr1</v>
       </c>
       <c r="B2284" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -87369,7 +87369,7 @@
     </row>
     <row r="2285">
       <c r="A2285" t="str">
-        <v>Kmu0wc9ru1k2m</v>
+        <v>Kmu64rl7ctsx9</v>
       </c>
       <c r="B2285" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -87407,7 +87407,7 @@
     </row>
     <row r="2286">
       <c r="A2286" t="str">
-        <v>Kmu0wc9ru53hm</v>
+        <v>Kmu64rl7cy2hj</v>
       </c>
       <c r="B2286" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -87521,7 +87521,7 @@
     </row>
     <row r="2289">
       <c r="A2289" t="str">
-        <v>Kmu0wc9ruzutl</v>
+        <v>Kmu64rl7c4w59</v>
       </c>
       <c r="B2289" t="str">
         <v>Penata Layanan Operasional</v>
@@ -87559,7 +87559,7 @@
     </row>
     <row r="2290">
       <c r="A2290" t="str">
-        <v>Kmu0wc9ruk3m8</v>
+        <v>Kmu64rl7ckttg</v>
       </c>
       <c r="B2290" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87597,7 +87597,7 @@
     </row>
     <row r="2291">
       <c r="A2291" t="str">
-        <v>Kmu0wc9ru6bst</v>
+        <v>Kmu64rl7coj5n</v>
       </c>
       <c r="B2291" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87635,7 +87635,7 @@
     </row>
     <row r="2292">
       <c r="A2292" t="str">
-        <v>Kmu0wc9ru19pi</v>
+        <v>Kmu64rl7cgv7y</v>
       </c>
       <c r="B2292" t="str">
         <v>Penata Keprotokolan*</v>
@@ -87749,7 +87749,7 @@
     </row>
     <row r="2295">
       <c r="A2295" t="str">
-        <v>Kmu0wc9ru567z</v>
+        <v>Kmu64rl7cmabi</v>
       </c>
       <c r="B2295" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87787,7 +87787,7 @@
     </row>
     <row r="2296">
       <c r="A2296" t="str">
-        <v>Kmu0wc9ruas84</v>
+        <v>Kmu64rl7cbc9e</v>
       </c>
       <c r="B2296" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87825,7 +87825,7 @@
     </row>
     <row r="2297">
       <c r="A2297" t="str">
-        <v>Kmu0wc9ruzs0r</v>
+        <v>Kmu64rl7c55ye</v>
       </c>
       <c r="B2297" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87901,7 +87901,7 @@
     </row>
     <row r="2299">
       <c r="A2299" t="str">
-        <v>Kmu0wc9ruc6d3</v>
+        <v>Kmu64rl7cxit9</v>
       </c>
       <c r="B2299" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87939,7 +87939,7 @@
     </row>
     <row r="2300">
       <c r="A2300" t="str">
-        <v>Kmu0wc9rugov1</v>
+        <v>Kmu64rl7cdm5q</v>
       </c>
       <c r="B2300" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87977,7 +87977,7 @@
     </row>
     <row r="2301">
       <c r="A2301" t="str">
-        <v>Kmu0wc9ruvncp</v>
+        <v>Kmu64rl7cgqq8</v>
       </c>
       <c r="B2301" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88015,7 +88015,7 @@
     </row>
     <row r="2302">
       <c r="A2302" t="str">
-        <v>Kmu0wc9ru7fbe</v>
+        <v>Kmu64rl7cmftb</v>
       </c>
       <c r="B2302" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -88053,7 +88053,7 @@
     </row>
     <row r="2303">
       <c r="A2303" t="str">
-        <v>Kmu0wc9ru83gg</v>
+        <v>Kmu64rl7ctc7a</v>
       </c>
       <c r="B2303" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -88091,7 +88091,7 @@
     </row>
     <row r="2304">
       <c r="A2304" t="str">
-        <v>Kmu0wc9ru9i3z</v>
+        <v>Kmu64rl7c9nj0</v>
       </c>
       <c r="B2304" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -88129,7 +88129,7 @@
     </row>
     <row r="2305">
       <c r="A2305" t="str">
-        <v>Kmu0wc9ruz08i</v>
+        <v>Kmu64rl7cafix</v>
       </c>
       <c r="B2305" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -88243,7 +88243,7 @@
     </row>
     <row r="2308">
       <c r="A2308" t="str">
-        <v>Kmu0wc9ru1ymb</v>
+        <v>Kmu64rl7ceb1f</v>
       </c>
       <c r="B2308" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88281,7 +88281,7 @@
     </row>
     <row r="2309">
       <c r="A2309" t="str">
-        <v>Kmu0wc9ruz3yd</v>
+        <v>Kmu64rl7cvoq0</v>
       </c>
       <c r="B2309" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88319,7 +88319,7 @@
     </row>
     <row r="2310">
       <c r="A2310" t="str">
-        <v>Kmu0wc9ru06mh</v>
+        <v>Kmu64rl7cseln</v>
       </c>
       <c r="B2310" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88357,7 +88357,7 @@
     </row>
     <row r="2311">
       <c r="A2311" t="str">
-        <v>Kmu0wc9rue1gm</v>
+        <v>Kmu64rl7cn71y</v>
       </c>
       <c r="B2311" t="str">
         <v>Penata Keprotokolan*</v>
@@ -88471,7 +88471,7 @@
     </row>
     <row r="2314">
       <c r="A2314" t="str">
-        <v>Kmu0wc9ru0ydd</v>
+        <v>Kmu64rl7cspdk</v>
       </c>
       <c r="B2314" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88509,7 +88509,7 @@
     </row>
     <row r="2315">
       <c r="A2315" t="str">
-        <v>Kmu0wc9ruvr3s</v>
+        <v>Kmu64rl7cx9u9</v>
       </c>
       <c r="B2315" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88547,7 +88547,7 @@
     </row>
     <row r="2316">
       <c r="A2316" t="str">
-        <v>Kmu0wc9ru2app</v>
+        <v>Kmu64rl7c46ic</v>
       </c>
       <c r="B2316" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88623,7 +88623,7 @@
     </row>
     <row r="2318">
       <c r="A2318" t="str">
-        <v>Kmu0wc9ruhl6w</v>
+        <v>Kmu64rl7ctrcq</v>
       </c>
       <c r="B2318" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88661,7 +88661,7 @@
     </row>
     <row r="2319">
       <c r="A2319" t="str">
-        <v>Kmu0wc9ruzmnx</v>
+        <v>Kmu64rl7cs2eq</v>
       </c>
       <c r="B2319" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88699,7 +88699,7 @@
     </row>
     <row r="2320">
       <c r="A2320" t="str">
-        <v>Kmu0wc9ru5m29</v>
+        <v>Kmu64rl7ctbhe</v>
       </c>
       <c r="B2320" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88775,7 +88775,7 @@
     </row>
     <row r="2322">
       <c r="A2322" t="str">
-        <v>Kmu0wc9rukmke</v>
+        <v>Kmu64rl7c40e9</v>
       </c>
       <c r="B2322" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88813,7 +88813,7 @@
     </row>
     <row r="2323">
       <c r="A2323" t="str">
-        <v>Kmu0wc9ru9yfs</v>
+        <v>Kmu64rl7ch6dx</v>
       </c>
       <c r="B2323" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88851,7 +88851,7 @@
     </row>
     <row r="2324">
       <c r="A2324" t="str">
-        <v>Kmu0wc9ru3jd3</v>
+        <v>Kmu64rl7cknh4</v>
       </c>
       <c r="B2324" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88927,7 +88927,7 @@
     </row>
     <row r="2326">
       <c r="A2326" t="str">
-        <v>Kmu0wc9ru7ztu</v>
+        <v>Kmu64rl7cbtju</v>
       </c>
       <c r="B2326" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88965,7 +88965,7 @@
     </row>
     <row r="2327">
       <c r="A2327" t="str">
-        <v>Kmu0wc9ruas67</v>
+        <v>Kmu64rl7c7eyo</v>
       </c>
       <c r="B2327" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89003,7 +89003,7 @@
     </row>
     <row r="2328">
       <c r="A2328" t="str">
-        <v>Kmu0wc9ruodbz</v>
+        <v>Kmu64rl7cpfb1</v>
       </c>
       <c r="B2328" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89117,7 +89117,7 @@
     </row>
     <row r="2331">
       <c r="A2331" t="str">
-        <v>Kmu0wc9runpra</v>
+        <v>Kmu64rl7c2i7b</v>
       </c>
       <c r="B2331" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89155,7 +89155,7 @@
     </row>
     <row r="2332">
       <c r="A2332" t="str">
-        <v>Kmu0wc9rubopm</v>
+        <v>Kmu64rl7cmtud</v>
       </c>
       <c r="B2332" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89193,7 +89193,7 @@
     </row>
     <row r="2333">
       <c r="A2333" t="str">
-        <v>Kmu0wc9ruduc5</v>
+        <v>Kmu64rl7czr6k</v>
       </c>
       <c r="B2333" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89269,7 +89269,7 @@
     </row>
     <row r="2335">
       <c r="A2335" t="str">
-        <v>Kmu0wc9rubb7m</v>
+        <v>Kmu64rl7c14s7</v>
       </c>
       <c r="B2335" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89307,7 +89307,7 @@
     </row>
     <row r="2336">
       <c r="A2336" t="str">
-        <v>Kmu0wc9rudmad</v>
+        <v>Kmu64rl7cwt7z</v>
       </c>
       <c r="B2336" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89345,7 +89345,7 @@
     </row>
     <row r="2337">
       <c r="A2337" t="str">
-        <v>Kmu0wc9ruto33</v>
+        <v>Kmu64rl7c7mf6</v>
       </c>
       <c r="B2337" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89383,7 +89383,7 @@
     </row>
     <row r="2338">
       <c r="A2338" t="str">
-        <v>Kmu0wc9run813</v>
+        <v>Kmu64rl7cgbtn</v>
       </c>
       <c r="B2338" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -89421,7 +89421,7 @@
     </row>
     <row r="2339">
       <c r="A2339" t="str">
-        <v>Kmu0wc9runcrh</v>
+        <v>Kmu64rl7cg8j6</v>
       </c>
       <c r="B2339" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -89459,7 +89459,7 @@
     </row>
     <row r="2340">
       <c r="A2340" t="str">
-        <v>Kmu0wc9rutqd1</v>
+        <v>Kmu64rl7cfsxw</v>
       </c>
       <c r="B2340" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -89497,7 +89497,7 @@
     </row>
     <row r="2341">
       <c r="A2341" t="str">
-        <v>Kmu0wc9rurqp0</v>
+        <v>Kmu64rl7c5hzv</v>
       </c>
       <c r="B2341" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -89611,7 +89611,7 @@
     </row>
     <row r="2344">
       <c r="A2344" t="str">
-        <v>Kmu0wc9rulrbc</v>
+        <v>Kmu64rl7ckc2n</v>
       </c>
       <c r="B2344" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89649,7 +89649,7 @@
     </row>
     <row r="2345">
       <c r="A2345" t="str">
-        <v>Kmu0wc9ruu1zb</v>
+        <v>Kmu64rl7cwawa</v>
       </c>
       <c r="B2345" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89687,7 +89687,7 @@
     </row>
     <row r="2346">
       <c r="A2346" t="str">
-        <v>Kmu0wc9ruv7tm</v>
+        <v>Kmu64rl7cff7m</v>
       </c>
       <c r="B2346" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89801,7 +89801,7 @@
     </row>
     <row r="2349">
       <c r="A2349" t="str">
-        <v>Kmu0wc9ru8lbh</v>
+        <v>Kmu64rl7c40cy</v>
       </c>
       <c r="B2349" t="str">
         <v>Penata Layanan Operasional</v>
@@ -89839,7 +89839,7 @@
     </row>
     <row r="2350">
       <c r="A2350" t="str">
-        <v>Kmu0wc9rui8f0</v>
+        <v>Kmu64rl7c7ydl</v>
       </c>
       <c r="B2350" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89877,7 +89877,7 @@
     </row>
     <row r="2351">
       <c r="A2351" t="str">
-        <v>Kmu0wc9ru4wym</v>
+        <v>Kmu64rl7cvbrt</v>
       </c>
       <c r="B2351" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89953,7 +89953,7 @@
     </row>
     <row r="2353">
       <c r="A2353" t="str">
-        <v>Kmu0wc9ru8yyu</v>
+        <v>Kmu64rl7cw21t</v>
       </c>
       <c r="B2353" t="str">
         <v>Penata Layanan Operasional</v>
@@ -89991,7 +89991,7 @@
     </row>
     <row r="2354">
       <c r="A2354" t="str">
-        <v>Kmu0wc9ruk8ps</v>
+        <v>Kmu64rl7cguo8</v>
       </c>
       <c r="B2354" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90029,7 +90029,7 @@
     </row>
     <row r="2355">
       <c r="A2355" t="str">
-        <v>Kmu0wc9ruhag0</v>
+        <v>Kmu64rl7cul1k</v>
       </c>
       <c r="B2355" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90067,7 +90067,7 @@
     </row>
     <row r="2356">
       <c r="A2356" t="str">
-        <v>Kmu0wc9ru7m9j</v>
+        <v>Kmu64rl7c7w03</v>
       </c>
       <c r="B2356" t="str">
         <v>Penata Keprotokolan*</v>
@@ -90143,7 +90143,7 @@
     </row>
     <row r="2358">
       <c r="A2358" t="str">
-        <v>Kmu0wc9ruldak</v>
+        <v>Kmu64rl7cr4ra</v>
       </c>
       <c r="B2358" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90181,7 +90181,7 @@
     </row>
     <row r="2359">
       <c r="A2359" t="str">
-        <v>Kmu0wc9ru5l1b</v>
+        <v>Kmu64rl7c6oxi</v>
       </c>
       <c r="B2359" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90219,7 +90219,7 @@
     </row>
     <row r="2360">
       <c r="A2360" t="str">
-        <v>Kmu0wc9rud4jb</v>
+        <v>Kmu64rl7cvqtn</v>
       </c>
       <c r="B2360" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90333,7 +90333,7 @@
     </row>
     <row r="2363">
       <c r="A2363" t="str">
-        <v>Kmu0wc9ruxp5p</v>
+        <v>Kmu64rl7chwmz</v>
       </c>
       <c r="B2363" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -90371,7 +90371,7 @@
     </row>
     <row r="2364">
       <c r="A2364" t="str">
-        <v>Kmu0wc9ru8mok</v>
+        <v>Kmu64rl7cmbou</v>
       </c>
       <c r="B2364" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90409,7 +90409,7 @@
     </row>
     <row r="2365">
       <c r="A2365" t="str">
-        <v>Kmu0wc9ruwkac</v>
+        <v>Kmu64rl7cs7mr</v>
       </c>
       <c r="B2365" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90485,7 +90485,7 @@
     </row>
     <row r="2367">
       <c r="A2367" t="str">
-        <v>Kmu0wc9ru8pqr</v>
+        <v>Kmu64rl7c0ojn</v>
       </c>
       <c r="B2367" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90523,7 +90523,7 @@
     </row>
     <row r="2368">
       <c r="A2368" t="str">
-        <v>Kmu0wc9ruvcph</v>
+        <v>Kmu64rl7cx1ah</v>
       </c>
       <c r="B2368" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90561,7 +90561,7 @@
     </row>
     <row r="2369">
       <c r="A2369" t="str">
-        <v>Kmu0wc9ru02pf</v>
+        <v>Kmu64rl7cjp1y</v>
       </c>
       <c r="B2369" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90637,7 +90637,7 @@
     </row>
     <row r="2371">
       <c r="A2371" t="str">
-        <v>Kmu0wc9ru0qyn</v>
+        <v>Kmu64rl7ck04f</v>
       </c>
       <c r="B2371" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -90675,7 +90675,7 @@
     </row>
     <row r="2372">
       <c r="A2372" t="str">
-        <v>Kmu0wc9ru8mg1</v>
+        <v>Kmu64rl7cxvom</v>
       </c>
       <c r="B2372" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90713,7 +90713,7 @@
     </row>
     <row r="2373">
       <c r="A2373" t="str">
-        <v>Kmu0wc9ru9mxp</v>
+        <v>Kmu64rl7cm0zv</v>
       </c>
       <c r="B2373" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90789,7 +90789,7 @@
     </row>
     <row r="2375">
       <c r="A2375" t="str">
-        <v>Kmu0wc9ruap80</v>
+        <v>Kmu64rl7czjo9</v>
       </c>
       <c r="B2375" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90827,7 +90827,7 @@
     </row>
     <row r="2376">
       <c r="A2376" t="str">
-        <v>Kmu0wc9rulse5</v>
+        <v>Kmu64rl7cjaud</v>
       </c>
       <c r="B2376" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90865,7 +90865,7 @@
     </row>
     <row r="2377">
       <c r="A2377" t="str">
-        <v>Kmu0wc9ruw931</v>
+        <v>Kmu64rl7ckcyo</v>
       </c>
       <c r="B2377" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90903,7 +90903,7 @@
     </row>
     <row r="2378">
       <c r="A2378" t="str">
-        <v>Kmu0wc9ru3o2j</v>
+        <v>Kmu64rl7ch3p7</v>
       </c>
       <c r="B2378" t="str">
         <v xml:space="preserve">Analis Pembiayaan Risiko dan Keuangan/ Analis Keuangan Negara Ahli Utama									</v>

</xml_diff>

<commit_message>
Perbarui struktur organisasi (2026-09-17T22:59:34.464Z)
</commit_message>
<xml_diff>
--- a/data/struktur-organisasi.xlsx
+++ b/data/struktur-organisasi.xlsx
@@ -78173,7 +78173,7 @@
     </row>
     <row r="2043">
       <c r="A2043" t="str">
-        <v>Kmu64rl7bcjz5</v>
+        <v>Kmu64t06ab5lc</v>
       </c>
       <c r="B2043" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78211,7 +78211,7 @@
     </row>
     <row r="2044">
       <c r="A2044" t="str">
-        <v>Kmu64rl7bf34p</v>
+        <v>Kmu64t06a0dyt</v>
       </c>
       <c r="B2044" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78249,7 +78249,7 @@
     </row>
     <row r="2045">
       <c r="A2045" t="str">
-        <v>Kmu64rl7byrer</v>
+        <v>Kmu64t06a9pgd</v>
       </c>
       <c r="B2045" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78325,7 +78325,7 @@
     </row>
     <row r="2047">
       <c r="A2047" t="str">
-        <v>Kmu64rl7b2pep</v>
+        <v>Kmu64t06a3y9n</v>
       </c>
       <c r="B2047" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78363,7 +78363,7 @@
     </row>
     <row r="2048">
       <c r="A2048" t="str">
-        <v>Kmu64rl7b4jai</v>
+        <v>Kmu64t06au4xi</v>
       </c>
       <c r="B2048" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78401,7 +78401,7 @@
     </row>
     <row r="2049">
       <c r="A2049" t="str">
-        <v>Kmu64rl7bqkpr</v>
+        <v>Kmu64t06ay5wc</v>
       </c>
       <c r="B2049" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78477,7 +78477,7 @@
     </row>
     <row r="2051">
       <c r="A2051" t="str">
-        <v>Kmu64rl7bd874</v>
+        <v>Kmu64t06ajdw4</v>
       </c>
       <c r="B2051" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78515,7 +78515,7 @@
     </row>
     <row r="2052">
       <c r="A2052" t="str">
-        <v>Kmu64rl7blxj6</v>
+        <v>Kmu64t06azn5y</v>
       </c>
       <c r="B2052" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78553,7 +78553,7 @@
     </row>
     <row r="2053">
       <c r="A2053" t="str">
-        <v>Kmu64rl7b5ig8</v>
+        <v>Kmu64t06acf1c</v>
       </c>
       <c r="B2053" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -78591,7 +78591,7 @@
     </row>
     <row r="2054">
       <c r="A2054" t="str">
-        <v>Kmu64rl7bktr7</v>
+        <v>Kmu64t06ac7nh</v>
       </c>
       <c r="B2054" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -78629,7 +78629,7 @@
     </row>
     <row r="2055">
       <c r="A2055" t="str">
-        <v>Kmu64rl7bo159</v>
+        <v>Kmu64t06abxkj</v>
       </c>
       <c r="B2055" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -78667,7 +78667,7 @@
     </row>
     <row r="2056">
       <c r="A2056" t="str">
-        <v>Kmu64rl7bdypz</v>
+        <v>Kmu64t06azkkp</v>
       </c>
       <c r="B2056" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -78705,7 +78705,7 @@
     </row>
     <row r="2057">
       <c r="A2057" t="str">
-        <v>Kmu64rl7bqw16</v>
+        <v>Kmu64t06auq1u</v>
       </c>
       <c r="B2057" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -78743,7 +78743,7 @@
     </row>
     <row r="2058">
       <c r="A2058" t="str">
-        <v>Kmu64rl7b1xcs</v>
+        <v>Kmu64t06a0vaa</v>
       </c>
       <c r="B2058" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -78857,7 +78857,7 @@
     </row>
     <row r="2061">
       <c r="A2061" t="str">
-        <v>Kmu64rl7b2o5l</v>
+        <v>Kmu64t06au05d</v>
       </c>
       <c r="B2061" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -78895,7 +78895,7 @@
     </row>
     <row r="2062">
       <c r="A2062" t="str">
-        <v>Kmu64rl7bju4q</v>
+        <v>Kmu64t06a2utt</v>
       </c>
       <c r="B2062" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -78933,7 +78933,7 @@
     </row>
     <row r="2063">
       <c r="A2063" t="str">
-        <v>Kmu64rl7b201j</v>
+        <v>Kmu64t06aw0e7</v>
       </c>
       <c r="B2063" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79009,7 +79009,7 @@
     </row>
     <row r="2065">
       <c r="A2065" t="str">
-        <v>Kmu64rl7b4epn</v>
+        <v>Kmu64t06a9js6</v>
       </c>
       <c r="B2065" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79047,7 +79047,7 @@
     </row>
     <row r="2066">
       <c r="A2066" t="str">
-        <v>Kmu64rl7byc55</v>
+        <v>Kmu64t06ay52d</v>
       </c>
       <c r="B2066" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79085,7 +79085,7 @@
     </row>
     <row r="2067">
       <c r="A2067" t="str">
-        <v>Kmu64rl7byo2q</v>
+        <v>Kmu64t06be7dg</v>
       </c>
       <c r="B2067" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79161,7 +79161,7 @@
     </row>
     <row r="2069">
       <c r="A2069" t="str">
-        <v>Kmu64rl7bjzu2</v>
+        <v>Kmu64t06bapsg</v>
       </c>
       <c r="B2069" t="str">
         <v>Penata Layanan Operasional</v>
@@ -79199,7 +79199,7 @@
     </row>
     <row r="2070">
       <c r="A2070" t="str">
-        <v>Kmu64rl7bqpyb</v>
+        <v>Kmu64t06by8ee</v>
       </c>
       <c r="B2070" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79237,7 +79237,7 @@
     </row>
     <row r="2071">
       <c r="A2071" t="str">
-        <v>Kmu64rl7bsi1h</v>
+        <v>Kmu64t06b730b</v>
       </c>
       <c r="B2071" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79313,7 +79313,7 @@
     </row>
     <row r="2073">
       <c r="A2073" t="str">
-        <v>Kmu64rl7bces6</v>
+        <v>Kmu64t06brgbs</v>
       </c>
       <c r="B2073" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79351,7 +79351,7 @@
     </row>
     <row r="2074">
       <c r="A2074" t="str">
-        <v>Kmu64rl7b2gv4</v>
+        <v>Kmu64t06b1na2</v>
       </c>
       <c r="B2074" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79389,7 +79389,7 @@
     </row>
     <row r="2075">
       <c r="A2075" t="str">
-        <v>Kmu64rl7b3c3z</v>
+        <v>Kmu64t06b9xcw</v>
       </c>
       <c r="B2075" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79427,7 +79427,7 @@
     </row>
     <row r="2076">
       <c r="A2076" t="str">
-        <v>Kmu64rl7bv8hm</v>
+        <v>Kmu64t06bbyie</v>
       </c>
       <c r="B2076" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -79465,7 +79465,7 @@
     </row>
     <row r="2077">
       <c r="A2077" t="str">
-        <v>Kmu64rl7b7fby</v>
+        <v>Kmu64t06bfhs1</v>
       </c>
       <c r="B2077" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -79503,7 +79503,7 @@
     </row>
     <row r="2078">
       <c r="A2078" t="str">
-        <v>Kmu64rl7btjrm</v>
+        <v>Kmu64t06b5e63</v>
       </c>
       <c r="B2078" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -79541,7 +79541,7 @@
     </row>
     <row r="2079">
       <c r="A2079" t="str">
-        <v>Kmu64rl7bx9u9</v>
+        <v>Kmu64t06bn99e</v>
       </c>
       <c r="B2079" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -79579,7 +79579,7 @@
     </row>
     <row r="2080">
       <c r="A2080" t="str">
-        <v>Kmu64rl7b55es</v>
+        <v>Kmu64t06bs9uh</v>
       </c>
       <c r="B2080" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -79617,7 +79617,7 @@
     </row>
     <row r="2081">
       <c r="A2081" t="str">
-        <v>Kmu64rl7bumxl</v>
+        <v>Kmu64t06bkbu7</v>
       </c>
       <c r="B2081" t="str">
         <v>Asesor SDM Aparatur Ahli Muda</v>
@@ -79655,7 +79655,7 @@
     </row>
     <row r="2082">
       <c r="A2082" t="str">
-        <v>Kmu64rl7b7fbz</v>
+        <v>Kmu64t06bhqa7</v>
       </c>
       <c r="B2082" t="str">
         <v>Asesor SDM Aparatur Ahli Pertama</v>
@@ -79769,7 +79769,7 @@
     </row>
     <row r="2085">
       <c r="A2085" t="str">
-        <v>Kmu64rl7bleij</v>
+        <v>Kmu64t06bwbec</v>
       </c>
       <c r="B2085" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -79807,7 +79807,7 @@
     </row>
     <row r="2086">
       <c r="A2086" t="str">
-        <v>Kmu64rl7bbt3o</v>
+        <v>Kmu64t06bnxah</v>
       </c>
       <c r="B2086" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79845,7 +79845,7 @@
     </row>
     <row r="2087">
       <c r="A2087" t="str">
-        <v>Kmu64rl7b1yfz</v>
+        <v>Kmu64t06b4ofi</v>
       </c>
       <c r="B2087" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -79921,7 +79921,7 @@
     </row>
     <row r="2089">
       <c r="A2089" t="str">
-        <v>Kmu64rl7boxig</v>
+        <v>Kmu64t06bzs44</v>
       </c>
       <c r="B2089" t="str">
         <v>Penata Layanan Operasional</v>
@@ -79959,7 +79959,7 @@
     </row>
     <row r="2090">
       <c r="A2090" t="str">
-        <v>Kmu64rl7bc170</v>
+        <v>Kmu64t06bei8q</v>
       </c>
       <c r="B2090" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -79997,7 +79997,7 @@
     </row>
     <row r="2091">
       <c r="A2091" t="str">
-        <v>Kmu64rl7boudc</v>
+        <v>Kmu64t06b87m8</v>
       </c>
       <c r="B2091" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80073,7 +80073,7 @@
     </row>
     <row r="2093">
       <c r="A2093" t="str">
-        <v>Kmu64rl7bmgr8</v>
+        <v>Kmu64t06bng9y</v>
       </c>
       <c r="B2093" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80111,7 +80111,7 @@
     </row>
     <row r="2094">
       <c r="A2094" t="str">
-        <v>Kmu64rl7bizah</v>
+        <v>Kmu64t06bdu08</v>
       </c>
       <c r="B2094" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80149,7 +80149,7 @@
     </row>
     <row r="2095">
       <c r="A2095" t="str">
-        <v>Kmu64rl7bgqku</v>
+        <v>Kmu64t06be8vm</v>
       </c>
       <c r="B2095" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80187,7 +80187,7 @@
     </row>
     <row r="2096">
       <c r="A2096" t="str">
-        <v>Kmu64rl7bbnb5</v>
+        <v>Kmu64t06bh6ek</v>
       </c>
       <c r="B2096" t="str">
         <v>Analis Anggaran Ahli Pertama/ Analis Keuangan Negara Ahli Pertama</v>
@@ -80225,7 +80225,7 @@
     </row>
     <row r="2097">
       <c r="A2097" t="str">
-        <v>Kmu64rl7b8k7o</v>
+        <v>Kmu64t06b2cqu</v>
       </c>
       <c r="B2097" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Muda/Pengawas Keuangan Negara Ahli Muda</v>
@@ -80263,7 +80263,7 @@
     </row>
     <row r="2098">
       <c r="A2098" t="str">
-        <v>Kmu64rl7bu4xy</v>
+        <v>Kmu64t06buicx</v>
       </c>
       <c r="B2098" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Pertama/Pengawas Keuangan Negara Ahli Pertama</v>
@@ -80301,7 +80301,7 @@
     </row>
     <row r="2099">
       <c r="A2099" t="str">
-        <v>Kmu64rl7bfebd</v>
+        <v>Kmu64t06b0a4g</v>
       </c>
       <c r="B2099" t="str">
         <v>Pranata Keuangan APBN Penyelia/Pengawas Keuangan Negara Penyelia</v>
@@ -80339,7 +80339,7 @@
     </row>
     <row r="2100">
       <c r="A2100" t="str">
-        <v>Kmu64rl7b8b9z</v>
+        <v>Kmu64t06bokek</v>
       </c>
       <c r="B2100" t="str">
         <v>Pranata Keuangan APBN Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -80377,7 +80377,7 @@
     </row>
     <row r="2101">
       <c r="A2101" t="str">
-        <v>Kmu64rl7b4bbc</v>
+        <v>Kmu64t06b8iew</v>
       </c>
       <c r="B2101" t="str">
         <v>Pranata Keuangan APBN Terampil/Pengawas Keuangan Negara Terampil</v>
@@ -80415,7 +80415,7 @@
     </row>
     <row r="2102">
       <c r="A2102" t="str">
-        <v>Kmu64rl7bqyeq</v>
+        <v>Kmu64t06bnngb</v>
       </c>
       <c r="B2102" t="str">
         <v>Analis SDM Aparatur Ahli Muda</v>
@@ -80453,7 +80453,7 @@
     </row>
     <row r="2103">
       <c r="A2103" t="str">
-        <v>Kmu64rl7bzjyq</v>
+        <v>Kmu64t06bz4xh</v>
       </c>
       <c r="B2103" t="str">
         <v>Analis SDM Aparatur Ahli Pertama</v>
@@ -80491,7 +80491,7 @@
     </row>
     <row r="2104">
       <c r="A2104" t="str">
-        <v>Kmu64rl7b6ngw</v>
+        <v>Kmu64t06by4w5</v>
       </c>
       <c r="B2104" t="str">
         <v>Pranata SDM Aparatur Penyelia</v>
@@ -80529,7 +80529,7 @@
     </row>
     <row r="2105">
       <c r="A2105" t="str">
-        <v>Kmu64rl7bd2qm</v>
+        <v>Kmu64t06bo65y</v>
       </c>
       <c r="B2105" t="str">
         <v>Pranata SDM Aparatur Mahir</v>
@@ -80567,7 +80567,7 @@
     </row>
     <row r="2106">
       <c r="A2106" t="str">
-        <v>Kmu64rl7b7mqa</v>
+        <v>Kmu64t06b0edr</v>
       </c>
       <c r="B2106" t="str">
         <v>Pranata SDM Aparatur Terampil</v>
@@ -80681,7 +80681,7 @@
     </row>
     <row r="2109">
       <c r="A2109" t="str">
-        <v>Kmu64rl7bhdas</v>
+        <v>Kmu64t06bjo3j</v>
       </c>
       <c r="B2109" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80719,7 +80719,7 @@
     </row>
     <row r="2110">
       <c r="A2110" t="str">
-        <v>Kmu64rl7bbldq</v>
+        <v>Kmu64t06bellr</v>
       </c>
       <c r="B2110" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80757,7 +80757,7 @@
     </row>
     <row r="2111">
       <c r="A2111" t="str">
-        <v>Kmu64rl7b24gt</v>
+        <v>Kmu64t06bh8m9</v>
       </c>
       <c r="B2111" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80833,7 +80833,7 @@
     </row>
     <row r="2113">
       <c r="A2113" t="str">
-        <v>Kmu64rl7b3zq9</v>
+        <v>Kmu64t06b0qk2</v>
       </c>
       <c r="B2113" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -80871,7 +80871,7 @@
     </row>
     <row r="2114">
       <c r="A2114" t="str">
-        <v>Kmu64rl7b9ltw</v>
+        <v>Kmu64t06b6zfl</v>
       </c>
       <c r="B2114" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -80909,7 +80909,7 @@
     </row>
     <row r="2115">
       <c r="A2115" t="str">
-        <v>Kmu64rl7b18x5</v>
+        <v>Kmu64t06b7ki2</v>
       </c>
       <c r="B2115" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -80985,7 +80985,7 @@
     </row>
     <row r="2117">
       <c r="A2117" t="str">
-        <v>Kmu64rl7b1l86</v>
+        <v>Kmu64t06bsxq5</v>
       </c>
       <c r="B2117" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -81023,7 +81023,7 @@
     </row>
     <row r="2118">
       <c r="A2118" t="str">
-        <v>Kmu64rl7b0szt</v>
+        <v>Kmu64t06b7zoi</v>
       </c>
       <c r="B2118" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81061,7 +81061,7 @@
     </row>
     <row r="2119">
       <c r="A2119" t="str">
-        <v>Kmu64rl7bpexk</v>
+        <v>Kmu64t06b1a8n</v>
       </c>
       <c r="B2119" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81099,7 +81099,7 @@
     </row>
     <row r="2120">
       <c r="A2120" t="str">
-        <v>Kmu64rl7btq6t</v>
+        <v>Kmu64t06bjour</v>
       </c>
       <c r="B2120" t="str">
         <v>Pengawas Keuangan Negara Ahli Pertama</v>
@@ -81137,7 +81137,7 @@
     </row>
     <row r="2121">
       <c r="A2121" t="str">
-        <v>Kmu64rl7bk2c3</v>
+        <v>Kmu64t06bhh5z</v>
       </c>
       <c r="B2121" t="str">
         <v>Pengawas Keuangan Negara Penyelia</v>
@@ -81175,7 +81175,7 @@
     </row>
     <row r="2122">
       <c r="A2122" t="str">
-        <v>Kmu64rl7bxt1k</v>
+        <v>Kmu64t06bgp46</v>
       </c>
       <c r="B2122" t="str">
         <v>Pengawas Keuangan Negara Mahir</v>
@@ -81213,7 +81213,7 @@
     </row>
     <row r="2123">
       <c r="A2123" t="str">
-        <v>Kmu64rl7bqtyg</v>
+        <v>Kmu64t06b6514</v>
       </c>
       <c r="B2123" t="str">
         <v>Pengawas Keuangan Negara Terampil</v>
@@ -81327,7 +81327,7 @@
     </row>
     <row r="2126">
       <c r="A2126" t="str">
-        <v>Kmu64rl7btjnr</v>
+        <v>Kmu64t06byijf</v>
       </c>
       <c r="B2126" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81365,7 +81365,7 @@
     </row>
     <row r="2127">
       <c r="A2127" t="str">
-        <v>Kmu64rl7bf0c7</v>
+        <v>Kmu64t06b87ql</v>
       </c>
       <c r="B2127" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81403,7 +81403,7 @@
     </row>
     <row r="2128">
       <c r="A2128" t="str">
-        <v>Kmu64rl7b9cu2</v>
+        <v>Kmu64t06bjr39</v>
       </c>
       <c r="B2128" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81441,7 +81441,7 @@
     </row>
     <row r="2129">
       <c r="A2129" t="str">
-        <v>Kmu64rl7bwolg</v>
+        <v>Kmu64t06b67y4</v>
       </c>
       <c r="B2129" t="str">
         <v>Penata Keprotokolan*</v>
@@ -81517,7 +81517,7 @@
     </row>
     <row r="2131">
       <c r="A2131" t="str">
-        <v>Kmu64rl7bjua6</v>
+        <v>Kmu64t06brq7q</v>
       </c>
       <c r="B2131" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81555,7 +81555,7 @@
     </row>
     <row r="2132">
       <c r="A2132" t="str">
-        <v>Kmu64rl7bng2s</v>
+        <v>Kmu64t06bar6p</v>
       </c>
       <c r="B2132" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81593,7 +81593,7 @@
     </row>
     <row r="2133">
       <c r="A2133" t="str">
-        <v>Kmu64rl7bsesi</v>
+        <v>Kmu64t06bsbno</v>
       </c>
       <c r="B2133" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81631,7 +81631,7 @@
     </row>
     <row r="2134">
       <c r="A2134" t="str">
-        <v>Kmu64rl7bueq4</v>
+        <v>Kmu64t06b9sm6</v>
       </c>
       <c r="B2134" t="str">
         <v>Penata Keprotokolan*</v>
@@ -81707,7 +81707,7 @@
     </row>
     <row r="2136">
       <c r="A2136" t="str">
-        <v>Kmu64rl7buzfk</v>
+        <v>Kmu64t06b9ymd</v>
       </c>
       <c r="B2136" t="str">
         <v>Penata Layanan Operasional</v>
@@ -81745,7 +81745,7 @@
     </row>
     <row r="2137">
       <c r="A2137" t="str">
-        <v>Kmu64rl7bpjju</v>
+        <v>Kmu64t06bxs93</v>
       </c>
       <c r="B2137" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -81783,7 +81783,7 @@
     </row>
     <row r="2138">
       <c r="A2138" t="str">
-        <v>Kmu64rl7bjryw</v>
+        <v>Kmu64t06b1uze</v>
       </c>
       <c r="B2138" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -81821,7 +81821,7 @@
     </row>
     <row r="2139">
       <c r="A2139" t="str">
-        <v>Kmu64rl7b9kzm</v>
+        <v>Kmu64t06bszo9</v>
       </c>
       <c r="B2139" t="str">
         <v>Pengawas Keuangan Negara Ahli Muda</v>
@@ -81859,7 +81859,7 @@
     </row>
     <row r="2140">
       <c r="A2140" t="str">
-        <v>Kmu64rl7bhijz</v>
+        <v>Kmu64t06bzsu4</v>
       </c>
       <c r="B2140" t="str">
         <v>Pengawas Keuangan Negara Pertama</v>
@@ -81897,7 +81897,7 @@
     </row>
     <row r="2141">
       <c r="A2141" t="str">
-        <v>Kmu64rl7bvit2</v>
+        <v>Kmu64t06brvte</v>
       </c>
       <c r="B2141" t="str">
         <v>Penata Laksana Barang Penyelia/ Pengawas Keuangan Negara Penyelia</v>
@@ -81935,7 +81935,7 @@
     </row>
     <row r="2142">
       <c r="A2142" t="str">
-        <v>Kmu64rl7bmii7</v>
+        <v>Kmu64t06bm5g7</v>
       </c>
       <c r="B2142" t="str">
         <v>Penata Laksana Barang Mahir/ Pengawas Keuangan Negara Mahir</v>
@@ -81973,7 +81973,7 @@
     </row>
     <row r="2143">
       <c r="A2143" t="str">
-        <v>Kmu64rl7bk8am</v>
+        <v>Kmu64t06bisk6</v>
       </c>
       <c r="B2143" t="str">
         <v>Penata Laksana Barang Terampil/ Pengawas Keuangan Negara Terampil</v>
@@ -82011,7 +82011,7 @@
     </row>
     <row r="2144">
       <c r="A2144" t="str">
-        <v>Kmu64rl7bfpy2</v>
+        <v>Kmu64t06bwwlr</v>
       </c>
       <c r="B2144" t="str">
         <v>Arsiparis Ahli Muda</v>
@@ -82049,7 +82049,7 @@
     </row>
     <row r="2145">
       <c r="A2145" t="str">
-        <v>Kmu64rl7bqif6</v>
+        <v>Kmu64t06b3tue</v>
       </c>
       <c r="B2145" t="str">
         <v>Arsiparis Ahli Pertama</v>
@@ -82087,7 +82087,7 @@
     </row>
     <row r="2146">
       <c r="A2146" t="str">
-        <v>Kmu64rl7bdowj</v>
+        <v>Kmu64t06bsm4g</v>
       </c>
       <c r="B2146" t="str">
         <v>Arsiparis Penyelia</v>
@@ -82125,7 +82125,7 @@
     </row>
     <row r="2147">
       <c r="A2147" t="str">
-        <v>Kmu64rl7bmp5f</v>
+        <v>Kmu64t06bmeca</v>
       </c>
       <c r="B2147" t="str">
         <v>Arsiparis Mahir</v>
@@ -82163,7 +82163,7 @@
     </row>
     <row r="2148">
       <c r="A2148" t="str">
-        <v>Kmu64rl7btolr</v>
+        <v>Kmu64t06bcn01</v>
       </c>
       <c r="B2148" t="str">
         <v>Arsiparis Terampil</v>
@@ -82277,7 +82277,7 @@
     </row>
     <row r="2151">
       <c r="A2151" t="str">
-        <v>Kmu64rl7bsotk</v>
+        <v>Kmu64t06b32u5</v>
       </c>
       <c r="B2151" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -82315,7 +82315,7 @@
     </row>
     <row r="2152">
       <c r="A2152" t="str">
-        <v>Kmu64rl7bgw9y</v>
+        <v>Kmu64t06b6a7w</v>
       </c>
       <c r="B2152" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82353,7 +82353,7 @@
     </row>
     <row r="2153">
       <c r="A2153" t="str">
-        <v>Kmu64rl7bl04x</v>
+        <v>Kmu64t06bnah5</v>
       </c>
       <c r="B2153" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82391,7 +82391,7 @@
     </row>
     <row r="2154">
       <c r="A2154" t="str">
-        <v>Kmu64rl7b4gki</v>
+        <v>Kmu64t06b8b1m</v>
       </c>
       <c r="B2154" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -82429,7 +82429,7 @@
     </row>
     <row r="2155">
       <c r="A2155" t="str">
-        <v>Kmu64rl7ber81</v>
+        <v>Kmu64t06bz6yg</v>
       </c>
       <c r="B2155" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -82467,7 +82467,7 @@
     </row>
     <row r="2156">
       <c r="A2156" t="str">
-        <v>Kmu64rl7b1iy7</v>
+        <v>Kmu64t06bnald</v>
       </c>
       <c r="B2156" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -82505,7 +82505,7 @@
     </row>
     <row r="2157">
       <c r="A2157" t="str">
-        <v>Kmu64rl7bsowy</v>
+        <v>Kmu64t06b36mm</v>
       </c>
       <c r="B2157" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -82581,7 +82581,7 @@
     </row>
     <row r="2159">
       <c r="A2159" t="str">
-        <v>Kmu64rl7bdkj6</v>
+        <v>Kmu64t06bf7fu</v>
       </c>
       <c r="B2159" t="str">
         <v>Penata Layanan Operasional</v>
@@ -82619,7 +82619,7 @@
     </row>
     <row r="2160">
       <c r="A2160" t="str">
-        <v>Kmu64rl7bpywj</v>
+        <v>Kmu64t06bjvs3</v>
       </c>
       <c r="B2160" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82657,7 +82657,7 @@
     </row>
     <row r="2161">
       <c r="A2161" t="str">
-        <v>Kmu64rl7bngn4</v>
+        <v>Kmu64t06b2ve7</v>
       </c>
       <c r="B2161" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82695,7 +82695,7 @@
     </row>
     <row r="2162">
       <c r="A2162" t="str">
-        <v>Kmu64rl7bumwn</v>
+        <v>Kmu64t06bdzy8</v>
       </c>
       <c r="B2162" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -82733,7 +82733,7 @@
     </row>
     <row r="2163">
       <c r="A2163" t="str">
-        <v>Kmu64rl7b9ioh</v>
+        <v>Kmu64t06bc4gn</v>
       </c>
       <c r="B2163" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -82771,7 +82771,7 @@
     </row>
     <row r="2164">
       <c r="A2164" t="str">
-        <v>Kmu64rl7bsitf</v>
+        <v>Kmu64t06b2ei6</v>
       </c>
       <c r="B2164" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -82809,7 +82809,7 @@
     </row>
     <row r="2165">
       <c r="A2165" t="str">
-        <v>Kmu64rl7bltd0</v>
+        <v>Kmu64t06bcxxq</v>
       </c>
       <c r="B2165" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -82885,7 +82885,7 @@
     </row>
     <row r="2167">
       <c r="A2167" t="str">
-        <v>Kmu64rl7bdv09</v>
+        <v>Kmu64t06bdziz</v>
       </c>
       <c r="B2167" t="str">
         <v>Penata Layanan Operasional</v>
@@ -82923,7 +82923,7 @@
     </row>
     <row r="2168">
       <c r="A2168" t="str">
-        <v>Kmu64rl7bj4cw</v>
+        <v>Kmu64t06b8izt</v>
       </c>
       <c r="B2168" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -82961,7 +82961,7 @@
     </row>
     <row r="2169">
       <c r="A2169" t="str">
-        <v>Kmu64rl7b5z4z</v>
+        <v>Kmu64t06bo68w</v>
       </c>
       <c r="B2169" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -82999,7 +82999,7 @@
     </row>
     <row r="2170">
       <c r="A2170" t="str">
-        <v>Kmu64rl7bo9p9</v>
+        <v>Kmu64t06bvqi6</v>
       </c>
       <c r="B2170" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -83037,7 +83037,7 @@
     </row>
     <row r="2171">
       <c r="A2171" t="str">
-        <v>Kmu64rl7bio04</v>
+        <v>Kmu64t06bte5m</v>
       </c>
       <c r="B2171" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -83075,7 +83075,7 @@
     </row>
     <row r="2172">
       <c r="A2172" t="str">
-        <v>Kmu64rl7bg7xt</v>
+        <v>Kmu64t06bqo56</v>
       </c>
       <c r="B2172" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -83113,7 +83113,7 @@
     </row>
     <row r="2173">
       <c r="A2173" t="str">
-        <v>Kmu64rl7bpgc4</v>
+        <v>Kmu64t06bfn80</v>
       </c>
       <c r="B2173" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -83151,7 +83151,7 @@
     </row>
     <row r="2174">
       <c r="A2174" t="str">
-        <v>Kmu64rl7b8y4v</v>
+        <v>Kmu64t06bzcc4</v>
       </c>
       <c r="B2174" t="str">
         <v>Pranata Humas Ahli Muda</v>
@@ -83189,7 +83189,7 @@
     </row>
     <row r="2175">
       <c r="A2175" t="str">
-        <v>Kmu64rl7bfyqd</v>
+        <v>Kmu64t06bgqjx</v>
       </c>
       <c r="B2175" t="str">
         <v>Pranata Humas Ahli Pertama**</v>
@@ -83227,7 +83227,7 @@
     </row>
     <row r="2176">
       <c r="A2176" t="str">
-        <v>Kmu64rl7b2wzo</v>
+        <v>Kmu64t06bk41m</v>
       </c>
       <c r="B2176" t="str">
         <v>Pranata Humas Penyelia**</v>
@@ -83265,7 +83265,7 @@
     </row>
     <row r="2177">
       <c r="A2177" t="str">
-        <v>Kmu64rl7br4yx</v>
+        <v>Kmu64t06b472w</v>
       </c>
       <c r="B2177" t="str">
         <v>Pranata Humas Mahir**</v>
@@ -83303,7 +83303,7 @@
     </row>
     <row r="2178">
       <c r="A2178" t="str">
-        <v>Kmu64rl7b4nt7</v>
+        <v>Kmu64t06bw35n</v>
       </c>
       <c r="B2178" t="str">
         <v>Pranata Humas Terampil**</v>
@@ -83341,7 +83341,7 @@
     </row>
     <row r="2179">
       <c r="A2179" t="str">
-        <v>Kmu64rl7bsikk</v>
+        <v>Kmu64t06b5qxp</v>
       </c>
       <c r="B2179" t="str">
         <v>Pustakawan Ahli Pertama</v>
@@ -83379,7 +83379,7 @@
     </row>
     <row r="2180">
       <c r="A2180" t="str">
-        <v>Kmu64rl7b9qfd</v>
+        <v>Kmu64t06b4hcl</v>
       </c>
       <c r="B2180" t="str">
         <v>Asisten Perpustakaan Penyelia</v>
@@ -83417,7 +83417,7 @@
     </row>
     <row r="2181">
       <c r="A2181" t="str">
-        <v>Kmu64rl7b282w</v>
+        <v>Kmu64t06bdf5d</v>
       </c>
       <c r="B2181" t="str">
         <v>Asisten Perpustakaan Mahir</v>
@@ -83455,7 +83455,7 @@
     </row>
     <row r="2182">
       <c r="A2182" t="str">
-        <v>Kmu64rl7b77fj</v>
+        <v>Kmu64t06bj2eh</v>
       </c>
       <c r="B2182" t="str">
         <v>Asisten Perpustakaan Terampil</v>
@@ -83493,7 +83493,7 @@
     </row>
     <row r="2183">
       <c r="A2183" t="str">
-        <v>Kmu64rl7b5eaw</v>
+        <v>Kmu64t06bphnu</v>
       </c>
       <c r="B2183" t="str">
         <v>Analis Pengelolaan Keuangan APBN Ahli Madya/Pengawas Keuangan Negara Ahli Madya</v>
@@ -83531,7 +83531,7 @@
     </row>
     <row r="2184">
       <c r="A2184" t="str">
-        <v>Kmu64rl7b4xxl</v>
+        <v>Kmu64t06bw9pc</v>
       </c>
       <c r="B2184" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Muda</v>
@@ -83569,7 +83569,7 @@
     </row>
     <row r="2185">
       <c r="A2185" t="str">
-        <v>Kmu64rl7bdo0l</v>
+        <v>Kmu64t06bl6gs</v>
       </c>
       <c r="B2185" t="str">
         <v>Perancang Peraturan Perundang-Undangan Ahli Pertama</v>
@@ -83683,7 +83683,7 @@
     </row>
     <row r="2188">
       <c r="A2188" t="str">
-        <v>Kmu64rl7cgvre</v>
+        <v>Kmu64t06bc51q</v>
       </c>
       <c r="B2188" t="str">
         <v>Penata Layanan Operasional</v>
@@ -83721,7 +83721,7 @@
     </row>
     <row r="2189">
       <c r="A2189" t="str">
-        <v>Kmu64rl7ckpv1</v>
+        <v>Kmu64t06b94aq</v>
       </c>
       <c r="B2189" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -83759,7 +83759,7 @@
     </row>
     <row r="2190">
       <c r="A2190" t="str">
-        <v>Kmu64rl7cyz0t</v>
+        <v>Kmu64t06bl704</v>
       </c>
       <c r="B2190" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -83797,7 +83797,7 @@
     </row>
     <row r="2191">
       <c r="A2191" t="str">
-        <v>Kmu64rl7ce0zs</v>
+        <v>Kmu64t06bxdos</v>
       </c>
       <c r="B2191" t="str">
         <v>Penata Keprotokolan*</v>
@@ -83911,7 +83911,7 @@
     </row>
     <row r="2194">
       <c r="A2194" t="str">
-        <v>Kmu64rl7c5lwj</v>
+        <v>Kmu64t06bnpwm</v>
       </c>
       <c r="B2194" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -83949,7 +83949,7 @@
     </row>
     <row r="2195">
       <c r="A2195" t="str">
-        <v>Kmu64rl7cs3fu</v>
+        <v>Kmu64t06bg7mf</v>
       </c>
       <c r="B2195" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -83987,7 +83987,7 @@
     </row>
     <row r="2196">
       <c r="A2196" t="str">
-        <v>Kmu64rl7ce071</v>
+        <v>Kmu64t06bdijb</v>
       </c>
       <c r="B2196" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84063,7 +84063,7 @@
     </row>
     <row r="2198">
       <c r="A2198" t="str">
-        <v>Kmu64rl7caf3n</v>
+        <v>Kmu64t06bpt7w</v>
       </c>
       <c r="B2198" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84101,7 +84101,7 @@
     </row>
     <row r="2199">
       <c r="A2199" t="str">
-        <v>Kmu64rl7cqeo8</v>
+        <v>Kmu64t06by6am</v>
       </c>
       <c r="B2199" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84139,7 +84139,7 @@
     </row>
     <row r="2200">
       <c r="A2200" t="str">
-        <v>Kmu64rl7cqxg5</v>
+        <v>Kmu64t06blr1b</v>
       </c>
       <c r="B2200" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84177,7 +84177,7 @@
     </row>
     <row r="2201">
       <c r="A2201" t="str">
-        <v>Kmu64rl7covyf</v>
+        <v>Kmu64t06b83vg</v>
       </c>
       <c r="B2201" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -84215,7 +84215,7 @@
     </row>
     <row r="2202">
       <c r="A2202" t="str">
-        <v>Kmu64rl7cpy8u</v>
+        <v>Kmu64t06bnqd6</v>
       </c>
       <c r="B2202" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -84253,7 +84253,7 @@
     </row>
     <row r="2203">
       <c r="A2203" t="str">
-        <v>Kmu64rl7c10lg</v>
+        <v>Kmu64t06buv9i</v>
       </c>
       <c r="B2203" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -84291,7 +84291,7 @@
     </row>
     <row r="2204">
       <c r="A2204" t="str">
-        <v>Kmu64rl7cn4h3</v>
+        <v>Kmu64t06b89jv</v>
       </c>
       <c r="B2204" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -84405,7 +84405,7 @@
     </row>
     <row r="2207">
       <c r="A2207" t="str">
-        <v>Kmu64rl7cyero</v>
+        <v>Kmu64t06bqq8l</v>
       </c>
       <c r="B2207" t="str">
         <v>Penata Layanan Operasional</v>
@@ -84443,7 +84443,7 @@
     </row>
     <row r="2208">
       <c r="A2208" t="str">
-        <v>Kmu64rl7c7h1y</v>
+        <v>Kmu64t06bpe5i</v>
       </c>
       <c r="B2208" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84481,7 +84481,7 @@
     </row>
     <row r="2209">
       <c r="A2209" t="str">
-        <v>Kmu64rl7c0ale</v>
+        <v>Kmu64t06bvxay</v>
       </c>
       <c r="B2209" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84519,7 +84519,7 @@
     </row>
     <row r="2210">
       <c r="A2210" t="str">
-        <v>Kmu64rl7ccpqs</v>
+        <v>Kmu64t06b0l2t</v>
       </c>
       <c r="B2210" t="str">
         <v>Penata Keprotokolan*</v>
@@ -84633,7 +84633,7 @@
     </row>
     <row r="2213">
       <c r="A2213" t="str">
-        <v>Kmu64rl7crall</v>
+        <v>Kmu64t06b5tw3</v>
       </c>
       <c r="B2213" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84671,7 +84671,7 @@
     </row>
     <row r="2214">
       <c r="A2214" t="str">
-        <v>Kmu64rl7c8qlc</v>
+        <v>Kmu64t06bum5x</v>
       </c>
       <c r="B2214" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84709,7 +84709,7 @@
     </row>
     <row r="2215">
       <c r="A2215" t="str">
-        <v>Kmu64rl7c4f6s</v>
+        <v>Kmu64t06bjx5c</v>
       </c>
       <c r="B2215" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84785,7 +84785,7 @@
     </row>
     <row r="2217">
       <c r="A2217" t="str">
-        <v>Kmu64rl7cn8gq</v>
+        <v>Kmu64t06bk8bz</v>
       </c>
       <c r="B2217" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -84823,7 +84823,7 @@
     </row>
     <row r="2218">
       <c r="A2218" t="str">
-        <v>Kmu64rl7c24us</v>
+        <v>Kmu64t06bcdkp</v>
       </c>
       <c r="B2218" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -84861,7 +84861,7 @@
     </row>
     <row r="2219">
       <c r="A2219" t="str">
-        <v>Kmu64rl7ckwhv</v>
+        <v>Kmu64t06brniy</v>
       </c>
       <c r="B2219" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -84899,7 +84899,7 @@
     </row>
     <row r="2220">
       <c r="A2220" t="str">
-        <v>Kmu64rl7cty0x</v>
+        <v>Kmu64t06b02th</v>
       </c>
       <c r="B2220" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -84937,7 +84937,7 @@
     </row>
     <row r="2221">
       <c r="A2221" t="str">
-        <v>Kmu64rl7cjkhs</v>
+        <v>Kmu64t06bavk4</v>
       </c>
       <c r="B2221" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -84975,7 +84975,7 @@
     </row>
     <row r="2222">
       <c r="A2222" t="str">
-        <v>Kmu64rl7cmchx</v>
+        <v>Kmu64t06bzhyj</v>
       </c>
       <c r="B2222" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -85013,7 +85013,7 @@
     </row>
     <row r="2223">
       <c r="A2223" t="str">
-        <v>Kmu64rl7crr7d</v>
+        <v>Kmu64t06bb1mi</v>
       </c>
       <c r="B2223" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -85127,7 +85127,7 @@
     </row>
     <row r="2226">
       <c r="A2226" t="str">
-        <v>Kmu64rl7cyz1e</v>
+        <v>Kmu64t06bq0wb</v>
       </c>
       <c r="B2226" t="str">
         <v>Penata Layanan Operasional</v>
@@ -85165,7 +85165,7 @@
     </row>
     <row r="2227">
       <c r="A2227" t="str">
-        <v>Kmu64rl7c8lwf</v>
+        <v>Kmu64t06b89v7</v>
       </c>
       <c r="B2227" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85203,7 +85203,7 @@
     </row>
     <row r="2228">
       <c r="A2228" t="str">
-        <v>Kmu64rl7co5dy</v>
+        <v>Kmu64t06bmpjw</v>
       </c>
       <c r="B2228" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85241,7 +85241,7 @@
     </row>
     <row r="2229">
       <c r="A2229" t="str">
-        <v>Kmu64rl7cyuxy</v>
+        <v>Kmu64t06btsgf</v>
       </c>
       <c r="B2229" t="str">
         <v>Penata Keprotokolan*</v>
@@ -85355,7 +85355,7 @@
     </row>
     <row r="2232">
       <c r="A2232" t="str">
-        <v>Kmu64rl7cb4r2</v>
+        <v>Kmu64t06bai4a</v>
       </c>
       <c r="B2232" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -85393,7 +85393,7 @@
     </row>
     <row r="2233">
       <c r="A2233" t="str">
-        <v>Kmu64rl7ckvsj</v>
+        <v>Kmu64t06bqk2u</v>
       </c>
       <c r="B2233" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85431,7 +85431,7 @@
     </row>
     <row r="2234">
       <c r="A2234" t="str">
-        <v>Kmu64rl7cex3q</v>
+        <v>Kmu64t06b5ylu</v>
       </c>
       <c r="B2234" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85507,7 +85507,7 @@
     </row>
     <row r="2236">
       <c r="A2236" t="str">
-        <v>Kmu64rl7cgdsj</v>
+        <v>Kmu64t06bjl9n</v>
       </c>
       <c r="B2236" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -85545,7 +85545,7 @@
     </row>
     <row r="2237">
       <c r="A2237" t="str">
-        <v>Kmu64rl7c5lo0</v>
+        <v>Kmu64t06bk5ei</v>
       </c>
       <c r="B2237" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85583,7 +85583,7 @@
     </row>
     <row r="2238">
       <c r="A2238" t="str">
-        <v>Kmu64rl7cels9</v>
+        <v>Kmu64t06b1oai</v>
       </c>
       <c r="B2238" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85621,7 +85621,7 @@
     </row>
     <row r="2239">
       <c r="A2239" t="str">
-        <v>Kmu64rl7c167i</v>
+        <v>Kmu64t06b940o</v>
       </c>
       <c r="B2239" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -85659,7 +85659,7 @@
     </row>
     <row r="2240">
       <c r="A2240" t="str">
-        <v>Kmu64rl7ccf5n</v>
+        <v>Kmu64t06bfx4n</v>
       </c>
       <c r="B2240" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -85697,7 +85697,7 @@
     </row>
     <row r="2241">
       <c r="A2241" t="str">
-        <v>Kmu64rl7cmuks</v>
+        <v>Kmu64t06bszgy</v>
       </c>
       <c r="B2241" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -85735,7 +85735,7 @@
     </row>
     <row r="2242">
       <c r="A2242" t="str">
-        <v>Kmu64rl7coxua</v>
+        <v>Kmu64t06bryfy</v>
       </c>
       <c r="B2242" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -85849,7 +85849,7 @@
     </row>
     <row r="2245">
       <c r="A2245" t="str">
-        <v>Kmu64rl7c921n</v>
+        <v>Kmu64t06blq2d</v>
       </c>
       <c r="B2245" t="str">
         <v>Penata Layanan Operasional</v>
@@ -85887,7 +85887,7 @@
     </row>
     <row r="2246">
       <c r="A2246" t="str">
-        <v>Kmu64rl7c2g7a</v>
+        <v>Kmu64t06bac21</v>
       </c>
       <c r="B2246" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -85925,7 +85925,7 @@
     </row>
     <row r="2247">
       <c r="A2247" t="str">
-        <v>Kmu64rl7c3o44</v>
+        <v>Kmu64t06bidcp</v>
       </c>
       <c r="B2247" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -85963,7 +85963,7 @@
     </row>
     <row r="2248">
       <c r="A2248" t="str">
-        <v>Kmu64rl7cn6kn</v>
+        <v>Kmu64t06b9dg1</v>
       </c>
       <c r="B2248" t="str">
         <v>Penata Keprotokolan*</v>
@@ -86039,7 +86039,7 @@
     </row>
     <row r="2250">
       <c r="A2250" t="str">
-        <v>Kmu64rl7cfalc</v>
+        <v>Kmu64t06bj8fn</v>
       </c>
       <c r="B2250" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86077,7 +86077,7 @@
     </row>
     <row r="2251">
       <c r="A2251" t="str">
-        <v>Kmu64rl7ckwju</v>
+        <v>Kmu64t06bywpa</v>
       </c>
       <c r="B2251" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86115,7 +86115,7 @@
     </row>
     <row r="2252">
       <c r="A2252" t="str">
-        <v>Kmu64rl7cbknw</v>
+        <v>Kmu64t06bup2i</v>
       </c>
       <c r="B2252" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86153,7 +86153,7 @@
     </row>
     <row r="2253">
       <c r="A2253" t="str">
-        <v>Kmu64rl7c8i32</v>
+        <v>Kmu64t06buzjq</v>
       </c>
       <c r="B2253" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -86191,7 +86191,7 @@
     </row>
     <row r="2254">
       <c r="A2254" t="str">
-        <v>Kmu64rl7cwkxw</v>
+        <v>Kmu64t06b8sbi</v>
       </c>
       <c r="B2254" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -86305,7 +86305,7 @@
     </row>
     <row r="2257">
       <c r="A2257" t="str">
-        <v>Kmu64rl7c6pkg</v>
+        <v>Kmu64t06bg24u</v>
       </c>
       <c r="B2257" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86343,7 +86343,7 @@
     </row>
     <row r="2258">
       <c r="A2258" t="str">
-        <v>Kmu64rl7cri5q</v>
+        <v>Kmu64t06bmsm5</v>
       </c>
       <c r="B2258" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86381,7 +86381,7 @@
     </row>
     <row r="2259">
       <c r="A2259" t="str">
-        <v>Kmu64rl7c0sne</v>
+        <v>Kmu64t06b63ej</v>
       </c>
       <c r="B2259" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86457,7 +86457,7 @@
     </row>
     <row r="2261">
       <c r="A2261" t="str">
-        <v>Kmu64rl7ckxu5</v>
+        <v>Kmu64t06b6i7y</v>
       </c>
       <c r="B2261" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -86495,7 +86495,7 @@
     </row>
     <row r="2262">
       <c r="A2262" t="str">
-        <v>Kmu64rl7c88k3</v>
+        <v>Kmu64t06bb0um</v>
       </c>
       <c r="B2262" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86533,7 +86533,7 @@
     </row>
     <row r="2263">
       <c r="A2263" t="str">
-        <v>Kmu64rl7c1wsv</v>
+        <v>Kmu64t06bm693</v>
       </c>
       <c r="B2263" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86571,7 +86571,7 @@
     </row>
     <row r="2264">
       <c r="A2264" t="str">
-        <v>Kmu64rl7ca16d</v>
+        <v>Kmu64t06bwkwz</v>
       </c>
       <c r="B2264" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -86609,7 +86609,7 @@
     </row>
     <row r="2265">
       <c r="A2265" t="str">
-        <v>Kmu64rl7cipso</v>
+        <v>Kmu64t06bzqg3</v>
       </c>
       <c r="B2265" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -86647,7 +86647,7 @@
     </row>
     <row r="2266">
       <c r="A2266" t="str">
-        <v>Kmu64rl7crr5p</v>
+        <v>Kmu64t06bmdzp</v>
       </c>
       <c r="B2266" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -86685,7 +86685,7 @@
     </row>
     <row r="2267">
       <c r="A2267" t="str">
-        <v>Kmu64rl7cp2ds</v>
+        <v>Kmu64t06bvy0y</v>
       </c>
       <c r="B2267" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -86799,7 +86799,7 @@
     </row>
     <row r="2270">
       <c r="A2270" t="str">
-        <v>Kmu64rl7cqabl</v>
+        <v>Kmu64t06baoa0</v>
       </c>
       <c r="B2270" t="str">
         <v>Penata Layanan Operasional</v>
@@ -86837,7 +86837,7 @@
     </row>
     <row r="2271">
       <c r="A2271" t="str">
-        <v>Kmu64rl7cnj9s</v>
+        <v>Kmu64t06bfstw</v>
       </c>
       <c r="B2271" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -86875,7 +86875,7 @@
     </row>
     <row r="2272">
       <c r="A2272" t="str">
-        <v>Kmu64rl7cgoux</v>
+        <v>Kmu64t06bv8yb</v>
       </c>
       <c r="B2272" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -86913,7 +86913,7 @@
     </row>
     <row r="2273">
       <c r="A2273" t="str">
-        <v>Kmu64rl7c0l54</v>
+        <v>Kmu64t06bgdt4</v>
       </c>
       <c r="B2273" t="str">
         <v>Penata Keprotokolan*</v>
@@ -87027,7 +87027,7 @@
     </row>
     <row r="2276">
       <c r="A2276" t="str">
-        <v>Kmu64rl7cdgdl</v>
+        <v>Kmu64t06be9ut</v>
       </c>
       <c r="B2276" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87065,7 +87065,7 @@
     </row>
     <row r="2277">
       <c r="A2277" t="str">
-        <v>Kmu64rl7ccobi</v>
+        <v>Kmu64t06b66pb</v>
       </c>
       <c r="B2277" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87103,7 +87103,7 @@
     </row>
     <row r="2278">
       <c r="A2278" t="str">
-        <v>Kmu64rl7ceiv4</v>
+        <v>Kmu64t06b51o7</v>
       </c>
       <c r="B2278" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87179,7 +87179,7 @@
     </row>
     <row r="2280">
       <c r="A2280" t="str">
-        <v>Kmu64rl7cckld</v>
+        <v>Kmu64t06by384</v>
       </c>
       <c r="B2280" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87217,7 +87217,7 @@
     </row>
     <row r="2281">
       <c r="A2281" t="str">
-        <v>Kmu64rl7ckhyf</v>
+        <v>Kmu64t06b1axf</v>
       </c>
       <c r="B2281" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87255,7 +87255,7 @@
     </row>
     <row r="2282">
       <c r="A2282" t="str">
-        <v>Kmu64rl7cz4yj</v>
+        <v>Kmu64t06b2y6x</v>
       </c>
       <c r="B2282" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87293,7 +87293,7 @@
     </row>
     <row r="2283">
       <c r="A2283" t="str">
-        <v>Kmu64rl7cehvn</v>
+        <v>Kmu64t06bkmxb</v>
       </c>
       <c r="B2283" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -87331,7 +87331,7 @@
     </row>
     <row r="2284">
       <c r="A2284" t="str">
-        <v>Kmu64rl7cmcr1</v>
+        <v>Kmu64t06bere2</v>
       </c>
       <c r="B2284" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -87369,7 +87369,7 @@
     </row>
     <row r="2285">
       <c r="A2285" t="str">
-        <v>Kmu64rl7ctsx9</v>
+        <v>Kmu64t06bern5</v>
       </c>
       <c r="B2285" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -87407,7 +87407,7 @@
     </row>
     <row r="2286">
       <c r="A2286" t="str">
-        <v>Kmu64rl7cy2hj</v>
+        <v>Kmu64t06bugn8</v>
       </c>
       <c r="B2286" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -87521,7 +87521,7 @@
     </row>
     <row r="2289">
       <c r="A2289" t="str">
-        <v>Kmu64rl7c4w59</v>
+        <v>Kmu64t06bx8qb</v>
       </c>
       <c r="B2289" t="str">
         <v>Penata Layanan Operasional</v>
@@ -87559,7 +87559,7 @@
     </row>
     <row r="2290">
       <c r="A2290" t="str">
-        <v>Kmu64rl7ckttg</v>
+        <v>Kmu64t06b9f4m</v>
       </c>
       <c r="B2290" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87597,7 +87597,7 @@
     </row>
     <row r="2291">
       <c r="A2291" t="str">
-        <v>Kmu64rl7coj5n</v>
+        <v>Kmu64t06bo600</v>
       </c>
       <c r="B2291" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87635,7 +87635,7 @@
     </row>
     <row r="2292">
       <c r="A2292" t="str">
-        <v>Kmu64rl7cgv7y</v>
+        <v>Kmu64t06bmvqd</v>
       </c>
       <c r="B2292" t="str">
         <v>Penata Keprotokolan*</v>
@@ -87749,7 +87749,7 @@
     </row>
     <row r="2295">
       <c r="A2295" t="str">
-        <v>Kmu64rl7cmabi</v>
+        <v>Kmu64t06b0k3m</v>
       </c>
       <c r="B2295" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87787,7 +87787,7 @@
     </row>
     <row r="2296">
       <c r="A2296" t="str">
-        <v>Kmu64rl7cbc9e</v>
+        <v>Kmu64t06bqyzm</v>
       </c>
       <c r="B2296" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87825,7 +87825,7 @@
     </row>
     <row r="2297">
       <c r="A2297" t="str">
-        <v>Kmu64rl7c55ye</v>
+        <v>Kmu64t06b0p59</v>
       </c>
       <c r="B2297" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -87901,7 +87901,7 @@
     </row>
     <row r="2299">
       <c r="A2299" t="str">
-        <v>Kmu64rl7cxit9</v>
+        <v>Kmu64t06bhm0q</v>
       </c>
       <c r="B2299" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -87939,7 +87939,7 @@
     </row>
     <row r="2300">
       <c r="A2300" t="str">
-        <v>Kmu64rl7cdm5q</v>
+        <v>Kmu64t06b9k5v</v>
       </c>
       <c r="B2300" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -87977,7 +87977,7 @@
     </row>
     <row r="2301">
       <c r="A2301" t="str">
-        <v>Kmu64rl7cgqq8</v>
+        <v>Kmu64t06bbdlb</v>
       </c>
       <c r="B2301" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88015,7 +88015,7 @@
     </row>
     <row r="2302">
       <c r="A2302" t="str">
-        <v>Kmu64rl7cmftb</v>
+        <v>Kmu64t06bjueg</v>
       </c>
       <c r="B2302" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -88053,7 +88053,7 @@
     </row>
     <row r="2303">
       <c r="A2303" t="str">
-        <v>Kmu64rl7ctc7a</v>
+        <v>Kmu64t06b7z2i</v>
       </c>
       <c r="B2303" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -88091,7 +88091,7 @@
     </row>
     <row r="2304">
       <c r="A2304" t="str">
-        <v>Kmu64rl7c9nj0</v>
+        <v>Kmu64t06bkpaj</v>
       </c>
       <c r="B2304" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -88129,7 +88129,7 @@
     </row>
     <row r="2305">
       <c r="A2305" t="str">
-        <v>Kmu64rl7cafix</v>
+        <v>Kmu64t06bx214</v>
       </c>
       <c r="B2305" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -88243,7 +88243,7 @@
     </row>
     <row r="2308">
       <c r="A2308" t="str">
-        <v>Kmu64rl7ceb1f</v>
+        <v>Kmu64t06bj766</v>
       </c>
       <c r="B2308" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88281,7 +88281,7 @@
     </row>
     <row r="2309">
       <c r="A2309" t="str">
-        <v>Kmu64rl7cvoq0</v>
+        <v>Kmu64t06bz4sq</v>
       </c>
       <c r="B2309" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88319,7 +88319,7 @@
     </row>
     <row r="2310">
       <c r="A2310" t="str">
-        <v>Kmu64rl7cseln</v>
+        <v>Kmu64t06bil53</v>
       </c>
       <c r="B2310" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88357,7 +88357,7 @@
     </row>
     <row r="2311">
       <c r="A2311" t="str">
-        <v>Kmu64rl7cn71y</v>
+        <v>Kmu64t06b52jk</v>
       </c>
       <c r="B2311" t="str">
         <v>Penata Keprotokolan*</v>
@@ -88471,7 +88471,7 @@
     </row>
     <row r="2314">
       <c r="A2314" t="str">
-        <v>Kmu64rl7cspdk</v>
+        <v>Kmu64t06basgs</v>
       </c>
       <c r="B2314" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88509,7 +88509,7 @@
     </row>
     <row r="2315">
       <c r="A2315" t="str">
-        <v>Kmu64rl7cx9u9</v>
+        <v>Kmu64t06bh68c</v>
       </c>
       <c r="B2315" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88547,7 +88547,7 @@
     </row>
     <row r="2316">
       <c r="A2316" t="str">
-        <v>Kmu64rl7c46ic</v>
+        <v>Kmu64t06brj31</v>
       </c>
       <c r="B2316" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88623,7 +88623,7 @@
     </row>
     <row r="2318">
       <c r="A2318" t="str">
-        <v>Kmu64rl7ctrcq</v>
+        <v>Kmu64t06bh2tu</v>
       </c>
       <c r="B2318" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88661,7 +88661,7 @@
     </row>
     <row r="2319">
       <c r="A2319" t="str">
-        <v>Kmu64rl7cs2eq</v>
+        <v>Kmu64t06btpqs</v>
       </c>
       <c r="B2319" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88699,7 +88699,7 @@
     </row>
     <row r="2320">
       <c r="A2320" t="str">
-        <v>Kmu64rl7ctbhe</v>
+        <v>Kmu64t06b1y1l</v>
       </c>
       <c r="B2320" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88775,7 +88775,7 @@
     </row>
     <row r="2322">
       <c r="A2322" t="str">
-        <v>Kmu64rl7c40e9</v>
+        <v>Kmu64t06bhcd6</v>
       </c>
       <c r="B2322" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88813,7 +88813,7 @@
     </row>
     <row r="2323">
       <c r="A2323" t="str">
-        <v>Kmu64rl7ch6dx</v>
+        <v>Kmu64t06bsn65</v>
       </c>
       <c r="B2323" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -88851,7 +88851,7 @@
     </row>
     <row r="2324">
       <c r="A2324" t="str">
-        <v>Kmu64rl7cknh4</v>
+        <v>Kmu64t06bhpge</v>
       </c>
       <c r="B2324" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -88927,7 +88927,7 @@
     </row>
     <row r="2326">
       <c r="A2326" t="str">
-        <v>Kmu64rl7cbtju</v>
+        <v>Kmu64t06bucxv</v>
       </c>
       <c r="B2326" t="str">
         <v>Penata Layanan Operasional</v>
@@ -88965,7 +88965,7 @@
     </row>
     <row r="2327">
       <c r="A2327" t="str">
-        <v>Kmu64rl7c7eyo</v>
+        <v>Kmu64t06bo3kr</v>
       </c>
       <c r="B2327" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89003,7 +89003,7 @@
     </row>
     <row r="2328">
       <c r="A2328" t="str">
-        <v>Kmu64rl7cpfb1</v>
+        <v>Kmu64t06bim87</v>
       </c>
       <c r="B2328" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89117,7 +89117,7 @@
     </row>
     <row r="2331">
       <c r="A2331" t="str">
-        <v>Kmu64rl7c2i7b</v>
+        <v>Kmu64t06bo0b6</v>
       </c>
       <c r="B2331" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89155,7 +89155,7 @@
     </row>
     <row r="2332">
       <c r="A2332" t="str">
-        <v>Kmu64rl7cmtud</v>
+        <v>Kmu64t06bgebe</v>
       </c>
       <c r="B2332" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89193,7 +89193,7 @@
     </row>
     <row r="2333">
       <c r="A2333" t="str">
-        <v>Kmu64rl7czr6k</v>
+        <v>Kmu64t06bwg1h</v>
       </c>
       <c r="B2333" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89269,7 +89269,7 @@
     </row>
     <row r="2335">
       <c r="A2335" t="str">
-        <v>Kmu64rl7c14s7</v>
+        <v>Kmu64t06b5ado</v>
       </c>
       <c r="B2335" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89307,7 +89307,7 @@
     </row>
     <row r="2336">
       <c r="A2336" t="str">
-        <v>Kmu64rl7cwt7z</v>
+        <v>Kmu64t06b9f50</v>
       </c>
       <c r="B2336" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89345,7 +89345,7 @@
     </row>
     <row r="2337">
       <c r="A2337" t="str">
-        <v>Kmu64rl7c7mf6</v>
+        <v>Kmu64t06bed49</v>
       </c>
       <c r="B2337" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89383,7 +89383,7 @@
     </row>
     <row r="2338">
       <c r="A2338" t="str">
-        <v>Kmu64rl7cgbtn</v>
+        <v>Kmu64t06bm8kh</v>
       </c>
       <c r="B2338" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Utama/Analis Keuangan Negara Ahli Utama</v>
@@ -89421,7 +89421,7 @@
     </row>
     <row r="2339">
       <c r="A2339" t="str">
-        <v>Kmu64rl7cg8j6</v>
+        <v>Kmu64t06bf8b4</v>
       </c>
       <c r="B2339" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Madya/Analis Keuangan Negara Ahli Madya</v>
@@ -89459,7 +89459,7 @@
     </row>
     <row r="2340">
       <c r="A2340" t="str">
-        <v>Kmu64rl7cfsxw</v>
+        <v>Kmu64t06bt65p</v>
       </c>
       <c r="B2340" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Muda/Analis Keuangan Negara Ahli Muda</v>
@@ -89497,7 +89497,7 @@
     </row>
     <row r="2341">
       <c r="A2341" t="str">
-        <v>Kmu64rl7c5hzv</v>
+        <v>Kmu64t06bu8z0</v>
       </c>
       <c r="B2341" t="str">
         <v>Analis Pembiayaan Risiko dan Keuangan Ahli Pertama/Analis Keuangan Negara Ahli Pertama</v>
@@ -89611,7 +89611,7 @@
     </row>
     <row r="2344">
       <c r="A2344" t="str">
-        <v>Kmu64rl7ckc2n</v>
+        <v>Kmu64t06bx48r</v>
       </c>
       <c r="B2344" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -89649,7 +89649,7 @@
     </row>
     <row r="2345">
       <c r="A2345" t="str">
-        <v>Kmu64rl7cwawa</v>
+        <v>Kmu64t06bfm5l</v>
       </c>
       <c r="B2345" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89687,7 +89687,7 @@
     </row>
     <row r="2346">
       <c r="A2346" t="str">
-        <v>Kmu64rl7cff7m</v>
+        <v>Kmu64t06b0v5j</v>
       </c>
       <c r="B2346" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89801,7 +89801,7 @@
     </row>
     <row r="2349">
       <c r="A2349" t="str">
-        <v>Kmu64rl7c40cy</v>
+        <v>Kmu64t06b9u58</v>
       </c>
       <c r="B2349" t="str">
         <v>Penata Layanan Operasional</v>
@@ -89839,7 +89839,7 @@
     </row>
     <row r="2350">
       <c r="A2350" t="str">
-        <v>Kmu64rl7c7ydl</v>
+        <v>Kmu64t06bth8q</v>
       </c>
       <c r="B2350" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -89877,7 +89877,7 @@
     </row>
     <row r="2351">
       <c r="A2351" t="str">
-        <v>Kmu64rl7cvbrt</v>
+        <v>Kmu64t06byaby</v>
       </c>
       <c r="B2351" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -89953,7 +89953,7 @@
     </row>
     <row r="2353">
       <c r="A2353" t="str">
-        <v>Kmu64rl7cw21t</v>
+        <v>Kmu64t06bs9nc</v>
       </c>
       <c r="B2353" t="str">
         <v>Penata Layanan Operasional</v>
@@ -89991,7 +89991,7 @@
     </row>
     <row r="2354">
       <c r="A2354" t="str">
-        <v>Kmu64rl7cguo8</v>
+        <v>Kmu64t06bdnd6</v>
       </c>
       <c r="B2354" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90029,7 +90029,7 @@
     </row>
     <row r="2355">
       <c r="A2355" t="str">
-        <v>Kmu64rl7cul1k</v>
+        <v>Kmu64t06bz8nd</v>
       </c>
       <c r="B2355" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90067,7 +90067,7 @@
     </row>
     <row r="2356">
       <c r="A2356" t="str">
-        <v>Kmu64rl7c7w03</v>
+        <v>Kmu64t06b10dt</v>
       </c>
       <c r="B2356" t="str">
         <v>Penata Keprotokolan*</v>
@@ -90143,7 +90143,7 @@
     </row>
     <row r="2358">
       <c r="A2358" t="str">
-        <v>Kmu64rl7cr4ra</v>
+        <v>Kmu64t06bvowx</v>
       </c>
       <c r="B2358" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90181,7 +90181,7 @@
     </row>
     <row r="2359">
       <c r="A2359" t="str">
-        <v>Kmu64rl7c6oxi</v>
+        <v>Kmu64t06bz5eb</v>
       </c>
       <c r="B2359" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90219,7 +90219,7 @@
     </row>
     <row r="2360">
       <c r="A2360" t="str">
-        <v>Kmu64rl7cvqtn</v>
+        <v>Kmu64t06bitpy</v>
       </c>
       <c r="B2360" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90333,7 +90333,7 @@
     </row>
     <row r="2363">
       <c r="A2363" t="str">
-        <v>Kmu64rl7chwmz</v>
+        <v>Kmu64t06bgm1u</v>
       </c>
       <c r="B2363" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -90371,7 +90371,7 @@
     </row>
     <row r="2364">
       <c r="A2364" t="str">
-        <v>Kmu64rl7cmbou</v>
+        <v>Kmu64t06bbgux</v>
       </c>
       <c r="B2364" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90409,7 +90409,7 @@
     </row>
     <row r="2365">
       <c r="A2365" t="str">
-        <v>Kmu64rl7cs7mr</v>
+        <v>Kmu64t06bnu08</v>
       </c>
       <c r="B2365" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90485,7 +90485,7 @@
     </row>
     <row r="2367">
       <c r="A2367" t="str">
-        <v>Kmu64rl7c0ojn</v>
+        <v>Kmu64t06bfahc</v>
       </c>
       <c r="B2367" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90523,7 +90523,7 @@
     </row>
     <row r="2368">
       <c r="A2368" t="str">
-        <v>Kmu64rl7cx1ah</v>
+        <v>Kmu64t06ba3m8</v>
       </c>
       <c r="B2368" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90561,7 +90561,7 @@
     </row>
     <row r="2369">
       <c r="A2369" t="str">
-        <v>Kmu64rl7cjp1y</v>
+        <v>Kmu64t06b8u70</v>
       </c>
       <c r="B2369" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90637,7 +90637,7 @@
     </row>
     <row r="2371">
       <c r="A2371" t="str">
-        <v>Kmu64rl7ck04f</v>
+        <v>Kmu64t06bfwz7</v>
       </c>
       <c r="B2371" t="str">
         <v>Penelaah Teknis Kebijakan</v>
@@ -90675,7 +90675,7 @@
     </row>
     <row r="2372">
       <c r="A2372" t="str">
-        <v>Kmu64rl7cxvom</v>
+        <v>Kmu64t06bbice</v>
       </c>
       <c r="B2372" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90713,7 +90713,7 @@
     </row>
     <row r="2373">
       <c r="A2373" t="str">
-        <v>Kmu64rl7cm0zv</v>
+        <v>Kmu64t06b6q5t</v>
       </c>
       <c r="B2373" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90789,7 +90789,7 @@
     </row>
     <row r="2375">
       <c r="A2375" t="str">
-        <v>Kmu64rl7czjo9</v>
+        <v>Kmu64t06b4y0r</v>
       </c>
       <c r="B2375" t="str">
         <v>Penata Layanan Operasional</v>
@@ -90827,7 +90827,7 @@
     </row>
     <row r="2376">
       <c r="A2376" t="str">
-        <v>Kmu64rl7cjaud</v>
+        <v>Kmu64t06bqpry</v>
       </c>
       <c r="B2376" t="str">
         <v>Pengolah Data dan Informasi</v>
@@ -90865,7 +90865,7 @@
     </row>
     <row r="2377">
       <c r="A2377" t="str">
-        <v>Kmu64rl7ckcyo</v>
+        <v>Kmu64t06bokfj</v>
       </c>
       <c r="B2377" t="str">
         <v>Pengadministrasi Perkantoran</v>
@@ -90903,7 +90903,7 @@
     </row>
     <row r="2378">
       <c r="A2378" t="str">
-        <v>Kmu64rl7ch3p7</v>
+        <v>Kmu64t06buz82</v>
       </c>
       <c r="B2378" t="str">
         <v xml:space="preserve">Analis Pembiayaan Risiko dan Keuangan/ Analis Keuangan Negara Ahli Utama									</v>

</xml_diff>